<commit_message>
feat(hadith): add narrator and isnad fields, refresh content from updated workbook
Adds Hadith.narrator (الراوي) and Hadith.isnad (عنعنة) alongside a new
shortExplanation field, sourced from the workbook's new columns. The
detail screen now shows the isnad phrase right before the hadith text,
a narrator badge, and a short-explanation card ahead of the full one.
Regenerates hadiths.json from the updated workbook (refined
explanations, narrator/isnad data for all 42 hadiths).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/data/الأربعون_النووية_رسائل_يومية.xlsx
+++ b/assets/data/الأربعون_النووية_رسائل_يومية.xlsx
@@ -453,15 +453,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,20 +479,30 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>الراوي</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>عنعنة</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Hadith_Text_Tashkeel</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Full_Explanation</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Short_Explanation</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Messages_Count</t>
         </is>
@@ -507,24 +519,35 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
+          <t>عمر بن الخطاب رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَمِيرِ الْمُؤْمِنِينَ أَبِي حَفْصٍ عُمَرَ بْنِ الْخَطَّابِ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ: سَمِعْتُ رَسُولَ اللهِ صَلَّى اللهُ تَعَالَى عَلَيْهِ وَآلِهِ وَسَلَّمَ يَقُولُ:</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
           <t>إِنَّمَا الْأَعْمَالُ بِالنِّيَّاتِ، وَإِنَّمَا لِكُلِّ امْرِئٍ مَا نَوَى، فَمَنْ كَانَتْ هِجْرَتُهُ إِلَى اللهِ وَرَسُولِهِ فَهِجْرَتُهُ إِلَى اللهِ وَرَسُولِهِ، وَمَنْ كَانَتْ هِجْرَتُهُ لِدُنْيَا يُصِيبُهَا أَوِ امْرَأَةٍ يَنْكِحُهَا فَهِجْرَتُهُ إِلَى مَا هَاجَرَ إِلَيْهِ</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>هذا الحديث من أصح الأحاديث وأعظمها موقعاً، وقد قال الإمام أحمد والشافعي رحمهما الله: يدخل في حديث النيات ثلث العلم، لأن كسب العبد يكون بقلبه ولسانه وجوارحه، والنية أحد هذه الأقسام الثلاثة. واستحب العلماء أن تُفتتح المصنفات بهذا الحديث تنبيهاً للطالب على تصحيح النية قبل كل عمل.
-وهو حديث مشهور من حيث المتن، لكنه غريب من جهة الإسناد؛ فلم يروه عن النبي صلى الله عليه وسلم إلا عمر بن الخطاب، ولم يروه عن عمر إلا علقمة بن وقاص، ولم يروه عن علقمة إلا محمد بن إبراهيم التيمي، ولم يروه عن محمد إلا يحيى بن سعيد الأنصاري، ثم اشتهر عنه بعد ذلك فرواه أكثر من مائتي راوٍ.
+وهذا الحديث مشهور بالنسبة إلى آخره، غريب بالنسبة إلى أوله؛ لأنه لم يروه عن النبي صلى الله عليه وسلم إلا عمر بن الخطاب رضي الله عنه، ولم يروه عن عمر إلا علقمة بن وقاص، ولم يروه عن علقمة إلا محمد بن إبراهيم التيمي، ولم يروه عن محمد إلا يحيى بن سعيد الأنصاري، ثم اشتهر بعد ذلك فرواه عنه أكثر من مائتي إنسان من أكابر الأئمة.
 ومعنى (إنما) هنا أداة حصر، وهي تارة تقتضي الحصر المطلق وتارة تقتضي حصراً خاصاً بحسب سياق الكلام والقرائن. والمراد هنا: أن الأعمال الشرعية المعتد بها هي المقترنة بالنية، فلا اعتداد شرعاً بعمل خلا من نية، كالوضوء والغسل والتيمم والصلاة والزكاة والصوم والحج وسائر العبادات؛ أما إزالة النجاسة والبر ونحوهما فلا تحتاج إلى نية لأنها ليست من باب التقرب المحض.
-وقوله (وإنما لكل امرئ ما نوى) فيه بيان أن العمل الواحد قد يقع صحيحاً أو باطلاً، كاملاً أو ناقصاً، بحسب النية المصاحبة له. وقد قال الشيخ محيي الدين النووي: فائدة تعيين المنوي أنه شرط، فلو كان على إنسان صلاة فائتة لم يكفه أن ينوي قضاء الفائتة مطلقاً، بل يشترط أن يعين كونها ظهراً أو عصراً أو غيرهما، ولولا اللفظ الثاني لاقتضى اللفظ الأول صحة النية بلا تعيين.
+وفي قوله صلى الله عليه وسلم (إنما الأعمال بالنيات) خبر محذوف، واختلف العلماء في تقديره: فالذين اشترطوا النية قدّروه: صحة الأعمال بالنيات، والذين لم يشترطوها قدّروه: كمال الأعمال بالنيات.
+وقوله (وإنما لكل امرئ ما نوى) قال الخطابي: يفيد معنى خاصاً غير الأول، وهو تعيين العمل بالنية. وفيه بيان أن العمل الواحد قد يقع صحيحاً أو باطلاً، كاملاً أو ناقصاً، بحسب النية المصاحبة له. وقد قال الشيخ محيي الدين النووي: فائدة تعيين المنوي أنه شرط، فلو كان على إنسان صلاة فائتة لم يكفه أن ينوي قضاء الفائتة مطلقاً، بل يشترط أن يعين كونها ظهراً أو عصراً أو غيرهما، ولولا اللفظ الثاني لاقتضى اللفظ الأول صحة النية بلا تعيين.
 وقوله (فمن كانت هجرته إلى الله ورسوله...) هذا من باب الشرط والجزاء، والمتقرر عند أهل العربية أن الشرط والجزاء والمبتدأ والخبر لابد أن يتغايرا، وهنا وقع الاتحاد لفظاً، فوجب تأويله بأن من كانت هجرته إلى الله ورسوله نية وقصداً، حكم له بذلك شرعاً وثواباً. وسبب ورود هذا الحديث -كما نقله بعضهم- أن رجلاً هاجر من مكة إلى المدينة ليتزوج امرأة يقال لها (أم قيس)، لا يريد بذلك فضيلة الهجرة، فكان يقال له (مهاجر أم قيس)، والله أعلم.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>كل عمل نقوم به - عبادة كان أو عملاً دنيوياً - قيمته الحقيقية عند الله ليست في صورته الظاهرة، بل في النية التي تسكن القلب وراءه. الفعل الواحد قد يكرره شخصان تماماً، لكن يفترقان كل الفراق في الأجر لأن نية أحدهما خالصة والآخر مشوبة بغرض آخر. ولهذا كانت الهجرة - وهي أعظم تضحية - تُقاس بمقصدها لا بمسافتها: من هاجر لله ورسوله فهجرته صادقة مقبولة، ومن هاجر لغرض دنيوي فهو حصل ما نواه فقط ولا أجر له عند الله. وهذا يدفعنا لمراجعة دوافعنا باستمرار في كل ما نقدم عليه: عملنا، دراستنا، حتى عباداتنا الظاهرة، فالمعيار الأول هو: لماذا أفعل هذا؟</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>8</v>
       </c>
     </row>
@@ -539,26 +562,37 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>عمر بن الخطاب رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ عُمَرَ رَضِيَ اللهُ تَعَالَى عَنْهُ أَيْضًا قَالَ:</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>بَيْنَمَا نَحْنُ جُلُوسٌ عِنْدَ رَسُولِ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ ذَاتَ يَوْمٍ إِذْ طَلَعَ عَلَيْنَا رَجُلٌ شَدِيدُ بَيَاضِ الثِّيَابِ شَدِيدُ سَوَادِ الشَّعْرِ لَا يُرَى عَلَيْهِ أَثَرُ السَّفَرِ وَلَا يَعْرِفُهُ مِنَّا أَحَدٌ، حَتَّى جَلَسَ إِلَى النَّبِيِّ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ فَأَسْنَدَ رُكْبَتَيْهِ إِلَى رُكْبَتَيْهِ وَوَضَعَ كَفَّيْهِ عَلَى فَخِذَيْهِ وَقَالَ: يَا مُحَمَّدُ أَخْبِرْنِي عَنِ الْإِسْلَامِ، فَقَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ: الْإِسْلَامُ أَنْ تَشْهَدَ أَنْ لَا إِلَهَ إِلَّا اللهُ وَأَنَّ مُحَمَّدًا رَسُولُ اللهِ، وَتُقِيمَ الصَّلَاةَ، وَتُؤْتِيَ الزَّكَاةَ، وَتَصُومَ رَمَضَانَ، وَتَحُجَّ الْبَيْتَ إِنِ اسْتَطَعْتَ إِلَيْهِ سَبِيلًا، قَالَ: صَدَقْتَ. فَعَجِبْنَا لَهُ يَسْأَلُهُ وَيُصَدِّقُهُ. قَالَ: فَأَخْبِرْنِي عَنِ الْإِيمَانِ، قَالَ: أَنْ تُؤْمِنَ بِاللهِ وَمَلَائِكَتِهِ وَكُتُبِهِ وَرُسُلِهِ وَالْيَوْمِ الْآخِرِ، وَتُؤْمِنَ بِالْقَدَرِ خَيْرِهِ وَشَرِّهِ، قَالَ: صَدَقْتَ. قَالَ: فَأَخْبِرْنِي عَنِ الْإِحْسَانِ، قَالَ: أَنْ تَعْبُدَ اللهَ كَأَنَّكَ تَرَاهُ، فَإِنْ لَمْ تَكُنْ تَرَاهُ فَإِنَّهُ يَرَاكَ. قَالَ: فَأَخْبِرْنِي عَنِ السَّاعَةِ، قَالَ: مَا الْمَسْؤُولُ عَنْهَا بِأَعْلَمَ مِنَ السَّائِلِ. قَالَ: فَأَخْبِرْنِي عَنْ أَمَارَاتِهَا، قَالَ: أَنْ تَلِدَ الْأَمَةُ رَبَّتَهَا، وَأَنْ تَرَى الْحُفَاةَ الْعُرَاةَ الْعَالَةَ رِعَاءَ الشَّاءِ يَتَطَاوَلُونَ فِي الْبُنْيَانِ. ثُمَّ انْطَلَقَ فَلَبِثْتُ مَلِيًّا، ثُمَّ قَالَ: يَا عُمَرُ أَتَدْرِي مَنِ السَّائِلُ؟ قُلْتُ: اللهُ وَرَسُولُهُ أَعْلَمُ، قَالَ: فَإِنَّهُ جِبْرِيلُ أَتَاكُمْ يُعَلِّمُكُمْ دِينَكُمْ</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>هذا حديث عظيم قد اشتمل على جميع وظائف الأعمال الظاهرة والباطنة، وعلوم الشريعة كلها راجعة إليه ومتشعبة منه، حتى قيل: هو للسنة كأم القرآن للقرآن، لجمعه معانيها. وفيه دليل على تحسين الثياب والهيئة عند الدخول على العلماء والفضلاء والملوك، لأن جبريل عليه السلام أتى بهذه الصورة معلماً الناس بحاله ومقاله.
-قوله (لا يُرى عليه أثر السفر) فيه أن جبريل جاء بصورة رجل غريب لم يُعرف، وهذا من كمال الإعجاز في تعليم الدين بأسلوب السؤال والجواب أمام الصحابة ليرسخ في أذهانهم.
-قوله (فأسند ركبتيه إلى ركبتيه ووضع كفيه على فخذيه) هيئة أدب وتواضع عند الجلوس للتعلم، وفيها استحباب هذه الهيئة لطالب العلم أمام شيخه.
-ومما يستفاد من هذا الحديث: أن الإسلام والإيمان حقيقتان متباينتان لغة وشرعاً إذا اجتمعا، ويفترقان إذا افترقا، فإذا ذُكر أحدهما منفرداً دخل فيه الآخر، وهذا هو الأصل في الأسماء المتقاربة في الشرع، وقد يُطلق أحدهما على الآخر على سبيل التجوّز. وقد ثبت في الصحيحين من حديث سعد بن أبي وقاص أنه قسّم الإيمان والإسلام بحسب الأحوال والأشخاص، وهذا لا ينافي كون الإيمان يشمل الإسلام عند الإطلاق.
+قوله (لا يُرى عليه أثر السفر) المشهور ضمّ الياء من (يُرى) مبنياً للمجهول، ورواه بعضهم بالنون المفتوحة (لا نرى)، وكلاهما صحيح.
+وقوله (فأسند ركبتيه إلى ركبتيه ووضع كفيه على فخذيه) هكذا هو المشهور الصحيح، وروى النسائي بمعناه (فوضع يديه على ركبتي النبي صلى الله عليه وسلم)، فارتفع بهذه الرواية الاحتمال الذي في لفظ مسلم، فإنه قال فيه (وضع كفيه على فخذيه) وهو لفظ محتمل.
+ومما يستفاد من هذا الحديث: أن الإسلام والإيمان حقيقتان متباينتان لغة وشرعاً إذا اجتمعا، ويفترقان إذا افترقا، فإذا ذُكر أحدهما منفرداً دخل فيه الآخر، وهذا هو الأصل في الأسماء المتقاربة في الشرع، وقد يُطلق أحدهما على الآخر على سبيل التجوّز.
 قوله في الإحسان (أن تعبد الله كأنك تراه، فإن لم تكن تراه فإنه يراك) حاصله: مراقبة الله تعالى في العبادات، بمعنى استحضار عظمة الله وجلاله حال العبادة حتى تصير أقرب إلى إتقانها وكمالها، فمن استحضر أنه بمرأى من الله ازداد خشوعاً وإخلاصاً.
 وقوله عن أمارات الساعة (أن تلد الأمة ربتها) فُسّر بأن يفشو سبي الإماء وبيعهن حتى تلد الأمة ولداً يصير سيدها من جهة أبيه، وقيل غير ذلك. وقوله (رعاء الشاء يتطاولون في البنيان) إشارة إلى انقلاب الأحوال، بأن يصير أهل الفقر والبداوة أهل ثروة وعمران دون أن يصلح ذلك حالهم في الدين.
+وقد حُكي في هذا الحديث خلاف طويل بين العلماء في زيادة الإيمان ونقصانه: فذهب جمهور أهل السنة إلى أن الإيمان قول وعمل يزيد وينقص، لقوله تعالى (ليزدادوا إيماناً مع إيمانهم)، وقال بعضهم: نفس التصديق الشرعي لا يزيد ولا ينقص، وإنما يزيد وينقص الإيمان بزيادة ثمراته ونقصانها وهي الأعمال. وحكى الشيخ أبو عمرو بن الصلاح أن قوله صلى الله عليه وسلم (الإسلام أن تشهد...) بيان لأصل الإيمان الباطن الذي هو التصديق والانقياد، وأن حكم الإسلام في الظاهر ثبت بالشهادتين، وإنما أضاف إليها الصلاة والزكاة والصوم والحج لكونها أظهر شعائر الإسلام؛ ولهذا لا يقع اسم المؤمن المطلق الكامل على من ارتكب كبيرة أو ترك فريضة، كما في حديث (لا يزني الزاني حين يزني وهو مؤمن). وقال الإمام فخر الدين الرازي: الإيمان والإسلام يجتمعان ويفترقان، فكل مؤمن مسلم وليس كل مسلم مؤمناً، وهذا موافق لمذهب جماهير العلماء وأهل الحديث، والله أعلم.
 ثم ختم الحديث ببيان أن هذا السائل هو جبريل عليه السلام، أتى ليعلّم الناس دينهم بطريقة السؤال والجواب، وهذا من أعظم طرق التعليم وأنفعها.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>في هذا الحديث يظهر جبريل عليه السلام في صورة إنسان ليسأل النبي صلى الله عليه وسلم أمام الصحابة عن أركان الدين الثلاثة: الإسلام (الأعمال الظاهرة كالشهادتين والصلاة والزكاة والصوم والحج)، والإيمان (التصديق القلبي بالله وملائكته وكتبه ورسله واليوم الآخر والقدر)، والإحسان (أعلى درجة، وهي أن تعبد الله وأنت تستحضر أنه يراك، حتى لو لم تستطع أن تتخيل رؤيته). هذا الحديث يعطينا خريطة كاملة للدين: تصرفات نلتزم بها، وقناعات نؤمن بها، وحالة قلبية نعيشها في كل لحظة عبادة. أعلى درجات الإيمان ليست في كثرة الأفعال فقط، بل في استحضار المراقبة الدائمة، وكأنك تتصرف وأنت واثق أن أحداً يراك دائماً.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -573,22 +607,32 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>عبد الله بن عمر بن الخطاب رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي عَبْدِ الرَّحْمَٰنِ عَبْدِ اللهِ بْنِ عُمَرَ بْنِ الْخَطَّابِ رَضِيَ اللهُ تَعَالَى عَنْهُمَا قَالَ: سَمِعْتُ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ يَقُولُ:</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>بُنِيَ الْإِسْلَامُ عَلَى خَمْسٍ: شَهَادَةِ أَنْ لَا إِلَهَ إِلَّا اللهُ وَأَنَّ مُحَمَّدًا رَسُولُ اللهِ، وَإِقَامِ الصَّلَاةِ، وَإِيتَاءِ الزَّكَاةِ، وَحَجِّ الْبَيْتِ، وَصَوْمِ رَمَضَانَ</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>قال أبو العباس القرطبي رحمه الله تعالى: يعني أن هذه الخمس أساس دين الإسلام وقواعده التي يقوم عليها ويثبت بها، وإنما خصّها بالذكر مع أن الجهاد يظهر معها عناد الكافرين ويقمع الدين، لأن هذه الخمس فروض أعيان دائمة على كل مسلم في كل الأوقات، وأما الجهاد ففرض كفاية يسقط في بعض الأوقات بخلافها.
 وقد وقع اختلاف في بعض الروايات في هذا الحديث بتقديم الحج على الصوم، وهو -والله أعلم- وهم من الرواة، لأن ابن عمر رضي الله عنهما لما سمع المستفتي يقدم الحج على الصوم أنكر عليه ذلك وزجره عن هذا الترتيب، وقال: سمعته من رسول الله صلى الله عليه وسلم بتقديم الصوم على الحج.
-وهذا الحديث أصل عظيم في معرفة الدين وعليه اعتماده، لأنه قد جمع أركانه: الشهادتان أساس التصديق والانقياد الظاهر والباطن، والصلاة عماد الدين وصلة العبد بربه المتكررة في اليوم والليلة، والزكاة تطهير للمال ومواساة للفقراء وتحقيق للتكافل الاجتماعي، والصوم تربية للنفس على ضبط الشهوات، والحج رحلة جامعة بين العبادة البدنية والمالية تُختم بها أركان الإسلام لمن استطاع إليها سبيلاً.</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+وهذا الحديث أصل عظيم في معرفة الدين وعليه اعتماده، فإنه قد جمع أركانه.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>الإسلام كالبناء له أساسه: شهادة أن لا إله إلا الله وأن محمداً رسول الله وهي الإقرار القلبي واللساني، ثم الصلاة وهي الصلة اليومية المتكررة مع الله، ثم الزكاة وهي تطهير المال والقلب من الشح، ثم الصوم وهي تدريب النفس على الانضباط، ثم الحج وهي رحلة تجمع كل هذه المعاني لمن استطاع. هذه الأركان الخمسة ليست طقوساً منفصلة، بل بنية متكاملة يشد بعضها بعضاً، فإذا ضعف ركن تأثر البناء كله، وإذا قامت جميعاً معاً كان الإيمان راسخاً وظاهراً في السلوك.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -603,24 +647,34 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>إِنَّ أَحَدَكُمْ يُجْمَعُ خَلْقُهُ فِي بَطْنِ أُمِّهِ أَرْبَعِينَ يَوْمًا نُطْفَةً، ثُمَّ يَكُونُ عَلَقَةً مِثْلَ ذَلِكَ، ثُمَّ يَكُونُ مُضْغَةً مِثْلَ ذَلِكَ، ثُمَّ يُرْسَلُ إِلَيْهِ الْمَلَكُ فَيَنْفُخُ فِيهِ الرُّوحَ، وَيُؤْمَرُ بِأَرْبَعِ كَلِمَاتٍ: بِكَتْبِ رِزْقِهِ، وَأَجَلِهِ، وَعَمَلِهِ، وَشَقِيٍّ أَوْ سَعِيدٍ، فَوَاللهِ الَّذِي لَا إِلَهَ غَيْرُهُ، إِنَّ أَحَدَكُمْ لَيَعْمَلُ بِعَمَلِ أَهْلِ الْجَنَّةِ حَتَّى مَا يَكُونُ بَيْنَهُ وَبَيْنَهَا إِلَّا ذِرَاعٌ فَيَسْبِقُ عَلَيْهِ الْكِتَابُ فَيَعْمَلُ بِعَمَلِ أَهْلِ النَّارِ فَيَدْخُلُهَا، وَإِنَّ أَحَدَكُمْ لَيَعْمَلُ بِعَمَلِ أَهْلِ النَّارِ حَتَّى مَا يَكُونُ بَيْنَهُ وَبَيْنَهَا إِلَّا ذِرَاعٌ فَيَسْبِقُ عَلَيْهِ الْكِتَابُ فَيَعْمَلُ بِعَمَلِ أَهْلِ الْجَنَّةِ فَيَدْخُلُهَا</t>
+          <t>أبو عبد الرحمن عبد الله بن مسعود رضي الله عنه</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>قوله (وهو الصادق المصدوق) أي الصادق في قوله، المصدَّق فيما يأتيه من الوحي الكريم. وقد فسّر بعض العلماء قوله (إن أحدكم يجمع خلقه في بطن أمه) بأن النطفة إذا وقعت في الرحم وأراد الله أن يخلق منها بشراً، طارت في بشرة المرأة تحت كل ظفر وشعر، ثم تمكث أربعين ليلة ثم تصير دماً فتنصب في الرحم فيجمعها، فتكون علقة.
+          <t>عَنْ أَبِي عَبْدِ الرَّحْمَٰنِ عَبْدِ اللهِ بْنِ مَسْعُودٍ رَضِيَ اللهُ عَنْهُ قَالَ: حَدَّثَنَا رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ وَهُوَ الصَّادِقُ الْمَصْدُوقُ:</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>إِنَّ أَحَدَكُمْ يُجْمَعُ خَلْقُهُ فِي بَطْنِ أُمِّهِ أَرْبَعِينَ يَوْمًا نُطْفَةً، ثُمَّ يَكُونُ عَلَقَةً مِثْلَ ذَلِكَ، ثُمَّ يَكُونُ مُضْغَةً مِثْلَ ذَلِكَ، ثُمَّ يُرْسَلُ إِلَيْهِ الْمَلَكُ فَيَنْفُخُ فِيهِ الرُّوحَ، وَيُؤْمَرُ بِأَرْبَعِ كَلِمَاتٍ: بِكَتْبِ رِزْقِهِ، وَأَجَلِهِ، وَعَمَلِهِ، وَشَقِيٌّ أَوْ سَعِيدٌ، فَوَاللهِ الَّذِي لَا إِلَهَ غَيْرُهُ، إِنَّ أَحَدَكُمْ لَيَعْمَلُ بِعَمَلِ أَهْلِ الْجَنَّةِ حَتَّى مَا يَكُونُ بَيْنَهُ وَبَيْنَهَا إِلَّا ذِرَاعٌ فَيَسْبِقُ عَلَيْهِ الْكِتَابُ فَيَعْمَلُ بِعَمَلِ أَهْلِ النَّارِ فَيَدْخُلُهَا، وَإِنَّ أَحَدَكُمْ لَيَعْمَلُ بِعَمَلِ أَهْلِ النَّارِ حَتَّى مَا يَكُونُ بَيْنَهُ وَبَيْنَهَا إِلَّا ذِرَاعٌ فَيَسْبِقُ عَلَيْهِ الْكِتَابُ فَيَعْمَلُ بِعَمَلِ أَهْلِ الْجَنَّةِ فَيَدْخُلُهَا</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>قوله (وهو الصادق المصدوق) أي الصادق في قوله، المصدَّق فيما يأتيه من الوحي الكريم. وقد جاء عن ابن مسعود رضي الله عنه راوي هذا الحديث في تفسير قوله (إن أحدكم يجمع خلقه في بطن أمه): أن النطفة إذا وقعت في الرحم وأراد الله أن يخلق منها بشراً، طارت في بشرة المرأة تحت كل ظفر وشعر، ثم تمكث أربعين ليلة ثم تصير دماً فتنصب في الرحم فيجمعها، فتكون علقة.
 وظاهر الحديث أن العامل بعمل أهل الجنة كان عمله صحيحاً وأنه قرُب من الجنة حتى بقي له ذراع من دخولها، لكن منعه من ذلك ما سبق به القدر الذي لا يظهر إلا عند الخاتمة؛ فإذا كانت السوابق مستورة عنا، ظهرت لنا حقيقتها في الأعمال بالخواتيم، يعني ما نُطلع عليه من الأعمال في نهاياتها بالنسبة لاطلاعنا في معنى الأحوال وبعض الأشخاص.
 وذكر مسلم في صحيحه في كتاب الإيمان أن رسول الله صلى الله عليه وسلم قال: (إن الرجل ليعمل بعمل أهل الجنة فيما يبدو للناس وهو من أهل النار، فإنه لم يكن عمله صحيحاً في نفسه، وإنما كان رياء وسمعة)، فيستفاد من ذلك ترك الالتفات إلى الأعمال والركون إليها، والتعويل على كرم الله تعالى ورحمته.
 وقوله (ويؤمر بأربع كلمات) بالباء الموحدة في أوله بدلاً على (أربع كلمات)، وقوله (شقي أو سعيد) مرفوع لأنه خبر مبتدأ محذوف، تقديره: وهو شقي أو سعيد.
-وهذا الحديث من أدلة إثبات القدر، وأن جميع الواقعات بقضاء الله تعالى وقدره، خيرها وشرها ونفعها وضرها. قال تعالى: (لا يُسأل عما يفعل وهم يُسألون) ولا اعتراض عليه فيما يفعل في ملكه ومايشاء. وهذا مع كون الله تعالى غير ظالم فيما يقدره، ولا يقدر شيئاً إلا لحكمة قد لا يدركها العباد. وقد ثبتت الأحاديث بالنهي عن ترك العمل اتكالاً على ما سبق من العلم بالقدر، بل تجب الأعمال والتكاليف التي وردت بها الشرائع، وكل ميسر لما خُلق له لا يقدر على خلاف مقدوره؛ فمن كان من أهل السعادة يُيسّره الله لعمل أهل السعادة، ومن كان من أهل الشقاوة يُيسّره الله لعمل أهل الشقاوة، كما قال تعالى: (فسنيسره لليسرى) و(فسنيسره للعسرى).</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+وهذا الحديث من أدلة إثبات القدر، وأن جميع الواقعات بقضاء الله تعالى وقدره، خيرها وشرها ونفعها وضرها. قال تعالى: (لا يُسأل عما يفعل وهم يُسألون) ولا اعتراض عليه فيما يفعل في ملكه ومايشاء. قال الإمام السمعاني رحمه الله: معرفة سبيل هذا الباب من الكتاب والسنة، ومجرد العقول دون محض القياس، فمن عدل عن التوفيق منه ضلّ في مجال الحيرة، ولم يبلغ شفاء النفس ولا يصل إلى ما يطمئن به القلب؛ لأن أسرار القدر سرّ الله تعالى ضرب دونه الأستار، واختص به سبحانه وحجبه عن عقول الخلق ومعارفهم لما علمه من الحكمة، وواجب علينا أن نقف حيث حُدّ لنا فلا نتجاوزه، وقد حجب الله تعالى علم القدر عن العالَم، فلا يعلمه ملك مقرّب ولا نبي مرسل، وقيل: إن سرّ القدر ينكشف لهم إذا دخلوا الجنة ولا ينكشف قبل ذلك. وقد ثبتت الأحاديث بالنهي عن ترك العمل اتكالاً على ما سبق من العلم بالقدر، بل تجب الأعمال والتكاليف التي وردت بها الشرائع، وكل ميسر لما خُلق له لا يقدر على خلاف مقدوره؛ فمن كان من أهل السعادة يُيسّره الله لعمل أهل السعادة، ومن كان من أهل الشقاوة يُيسّره الله لعمل أهل الشقاوة، كما قال تعالى: (فسنيسره لليسرى) و(فسنيسره للعسرى).</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>هذا الحديث يفتح نافذة على مراحل تكوين الإنسان في رحم أمه: نطفة، فعلقة، فمضغة، كل مرحلة أربعين يوماً، ثم تنفخ فيه الروح ويُكتب رزقه وأجله وعمله وشقاوته أو سعادته. لكن الحديث لا يتوقف عند الخلق، بل يذكّرنا بأن الأعمال تُقاس بخواتيمها، فقد يعمل الإنسان طويلاً بعمل أهل الجنة ثم ينحرف في آخر لحظة، والعكس صحيح. هذا لا يعني أن نعيش قلقين من مصيرنا، بل أن نفهم أن الإيمان بالقدر لا يعني ترك العمل، بل يعني أن نعمل بجدّ وأن نطلب من الله الثبات حتى النهاية، فكل ميسر لما خُلق له، والعبرة بحسن الخاتمة لا بلحظة عابرة من التقصير أو الصلاح.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -635,22 +689,32 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
+          <t>أم المؤمنين أم عبد الله عائشة بنت أبي بكر رضي الله عنها</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أُمِّ الْمُؤْمِنِينَ أُمِّ عَبْدِ اللهِ عَائِشَةَ رَضِيَ اللهُ عَنْهَا قَالَتْ: قَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ:</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
           <t>مَنْ أَحْدَثَ فِي أَمْرِنَا هَذَا مَا لَيْسَ مِنْهُ فَهُوَ رَدٌّ</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>قال أهل اللغة: الرد هنا بمعنى المردود، أي فهو باطل غير معتدّ به، وقوله (ليس عليه أمرنا) يعني ليس عليه حكمنا.
 هذا الحديث قاعدة عظيمة من قواعد الدين، وهو من جوامع الكلم التي أوتيها المصطفى صلى الله عليه وسلم، فإنه صريح في رد كل بدعة مخترعة، ويستدل به على إبطال جميع العقود الممنوعة وعدم وجود ثمرتها. واستدل به بعض الأصوليين على أن النهي يقتضي الفساد. والرواية الأخرى (من عمل عملاً ليس عليه أمرنا فهو رد) صريحة في رد كل عمل ليس عليه دليل شرعي، سواء أحدثها فاعلها أو تقدمه أسبقها إليها، فإنه يقدح فيه بعض المعاندين إذا فعل بدعة فيقول: ما أحدثت شيئاً، فيحتج عليه بهذه الرواية.
 وهذا الحديث مما ينبغي حفظه وإشاعته واستعماله في إبطال المنكرات كلها، فأما تفريغ الأصول التي لا تتناولها السنة فلا يتناولها هذا الرد، ككتابة العزيز في المصاحف، والمذاهب التي عن حسن نظر الفقهاء المجتهدين يردّون الفروع إلى الأصول التي هي قول رسول الله صلى الله عليه وسلم، وكالكتب الموضوعة في النحو والحساب والفرائض وغير ذلك من العلوم مرجعه ومبناه على أقوال رسول الله صلى الله عليه وسلم وأوامره، فإن ذلك لا يدخل في هذا الحديث.</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>هذا الحديث القصير قاعدة كبيرة: أي أمر جديد يُدخل في الدين وليس له أصل من كتاب الله أو سنة نبيه فهو مرفوض، مهما بدا حسناً في الظاهر أو حماسياً في نيته. الدين ليس مجالاً للاجتهاد الشخصي في العبادات، فحدوده واضحة وضبطها من الله ورسوله لا من أهوائنا. لكن هذا لا يعني رفض كل جديد في الحياة، فالوسائل والعلوم والتقنيات التي تخدم الدين ولا تخالفه لا تدخل في هذا الرد، إنما المقصود ما يُبتدع في صلب العبادة والتشريع نفسه دون أصل شرعي.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -665,25 +729,36 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>النعمان بن بشير رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي عَبْدِ اللهِ النُّعْمَانِ بْنِ بَشِيرٍ رَضِيَ اللهُ عَنْهُمَا قَالَ: سَمِعْتُ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ يَقُولُ:</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>إِنَّ الْحَلَالَ بَيِّنٌ، وَإِنَّ الْحَرَامَ بَيِّنٌ، وَبَيْنَهُمَا أُمُورٌ مُشْتَبِهَاتٌ لَا يَعْلَمُهُنَّ كَثِيرٌ مِنَ النَّاسِ، فَمَنِ اتَّقَى الشُّبُهَاتِ فَقَدِ اسْتَبْرَأَ لِدِينِهِ وَعِرْضِهِ، وَمَنْ وَقَعَ فِي الشُّبُهَاتِ وَقَعَ فِي الْحَرَامِ، كَالرَّاعِي يَرْعَى حَوْلَ الْحِمَى يُوشِكُ أَنْ يَرْتَعَ فِيهِ، أَلَا وَإِنَّ لِكُلِّ مَلِكٍ حِمًى، أَلَا وَإِنَّ حِمَى اللهِ مَحَارِمُهُ، أَلَا وَإِنَّ فِي الْجَسَدِ مُضْغَةً إِذَا صَلَحَتْ صَلَحَ الْجَسَدُ كُلُّهُ، وَإِذَا فَسَدَتْ فَسَدَ الْجَسَدُ كُلُّهُ، أَلَا وَهِيَ الْقَلْبُ</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>هذا حديث أصل عظيم من أصول الدين، وقال أبو داود: الإسلام يدور على أربعة أحاديث، ذكر هذا الحديث منها، وأجمع العلماء على عظم موقعه وكثرة فوائده.
 قوله (إن الحلال بيّن وإن الحرام بيّن وبينهما أمور مشتبهات) يعني أن الأشياء ثلاثة أقسام: ما نصّ الشرع على تحليله كقوله تعالى (أحل لكم الطيبات وطعام الذين أوتوا الكتاب حل لكم)، وما نصّ على تحريمه مثل قوله تعالى (حرمت عليكم أمهاتكم وبناتكم) وتحريم صيد البر مادام محرماً، وما لم يُنص عليه فهو من الشبهات التي تنازعتها الأدلة من الكتاب والسنة وتجاذبتها المعاني، فالإمساك عنه ورع.
-وقد اختلف العلماء في المشتبهات التي أشار إليها النبي صلى الله عليه وسلم في هذا الحديث، فقالت طائفة: هي حرام لقوله (استبرأ لدينه وعرضه)، من لم يستبرئ فقد وقع عرضه ودينه في الحرام. وقالت طائفة أخرى: هي حلال بدليل قوله في الحديث (كالراعي يرعى حول الحمى) فدلّ ذلك على خلال، وأن تركه ورع. وقالت طائفة ثالثة: المشتبهات المذكورة في هذا الحديث لا نقول إنها حلال ولا حرام، فإنه صلى الله عليه وسلم جعلها بين الحلال البين والحرام البين، فينبغي أن نتوقف عنها.
-قوله (فمن اتقى الشبهات فقد استبرأ لدينه وعرضه) أي من ترك الشبهات فقد حفظ دينه من الوقوع فيما يشينه، وحفظ عرضه من أن يتحدث الناس عنه بالسوء لمخالطته موضع الريبة، ولو لم يكن حراماً في نفس الأمر فقد سلم من مقالة الناس فيه.
-قوله (كالراعي يرعى حول الحمى يوشك أن يرتع فيه) وأصله أن العرب كانت تحمي مراعي لمواشيها وتتوعد بالعقوبة من يقرب حماها، فمن قارب حماها بماشيته يوشك أن تقع فيه لأنه قد يقرب منه فيغفل عن ضبطها فتقع فيه، والحذر أن يجعل بينه وبين ذلك الحمى مسافة يأمن معها الوقوع فيه، وهكذا محارم الله عز وجل من القتل والربا والسرقة والقذف والغيبة والنميمة ونحو ذلك، فينبغي أن يحوم حولها مخافة الوقوع فيها.
+وقد اختلف العلماء في المشتبهات التي أشار إليها النبي صلى الله عليه وسلم في هذا الحديث، فقالت طائفة: هي حرام لقوله (استبرأ لدينه وعرضه)، قالوا: من لم يستبرئ لدينه وعرضه فقد وقع في الحرام. وقال آخرون: هي حلال بدليل قوله في الحديث (كالراعي يرعى حول الحمى) فدلّ ذلك على حلال، وأن تركه ورع. وقالت طائفة أخرى: المشتبهات المذكورة في هذا الحديث لا نقول إنها حلال ولا حرام، فإنه صلى الله عليه وسلم جعلها بين الحلال البين والحرام البين، فينبغي أن نتوقف عنها، وهذا من باب الورع أيضاً.
+وقد ثبت في الصحيحين من حديث عائشة رضي الله عنها قصة اختصام سعد بن أبي وقاص وعبد بن زمعة في نسب غلام، وفيها أن النبي صلى الله عليه وسلم مع رؤيته شبهاً بيّناً بعتبة بن أبي وقاص قضى بالولد لعبد بن زمعة عملاً بقاعدة (الولد للفراش وللعاهر الحجر)، ثم احتاط فأمر سودة رضي الله عنها بالاحتجاب منه لأجل ذلك الشبه. وكذلك حديث عدي بن حاتم حين سأل عن كلبه إذا وجد معه عند الصيد كلباً آخر ولم يدرِ أيهما قتل الصيد، فأفتاه النبي صلى الله عليه وسلم بترك الأكل احتياطاً وقال: (لا تأكل، إنما سمّيت على كلبك ولم تسمِّ على غيره). وقال بعض العلماء: المشتبهات على هذا ثلاثة أقسام: ما يُعلم تحريمه أصلاً ثم يُشك في زواله فالأصل بقاء التحريم، وعكسه ما يُعلم حِلّه ثم يُشك في تحريمه فالأصل بقاء الحل، وما لا يُعرف أصله البتة فالأحسن فيه التنزه، كما فعل النبي صلى الله عليه وسلم في التمرة الساقطة إذ قال: (لولا أني أخشى أن تكون من الصدقة لأكلتها)، وأما مجرد الوهم الذي لا دليل عليه فليس من الورع في شيء بل هو من وسوسة الشيطان.
+قوله (فمن اتقى الشبهات فقد استبرأ لدينه وعرضه)، وأما قوله (ومن وقع في الشبهات وقع في الحرام) فذلك من وجهين: أحدهما أن من لم يتق الله وتجرأ على الشبهات أفضت به إلى المحرمات، إذ يحمله التساهل فيها على الجرأة على الحرام، كما قيل: الصغيرة تجرّ الكبيرة، والكبيرة تجرّ الكفر، وروي أن (المعاصي بريد الكفر). والوجه الثاني: أن كثرة مواقعة الشبهات تُظلم القلب فينطفئ فيه نور العلم ونور الورع، فيقع صاحبه في الحرام وهو لا يشعر به.
+قوله (كالراعي يرعى حول الحمى يوشك أن يرتع فيه) وأصله أن العرب كانت تحمي مراعي لمواشيها وتتوعد بالعقوبة من يقرب حماها، فمن قارب حماها بماشيته يوشك أن تقع فيه لأنه قد يقرب منه فيغفل عن ضبطها فتقع فيه، والحذر أن يجعل بينه وبين ذلك الحمى مسافة يأمن معها الوقوع فيه، وهكذا محارم الله عز وجل من القتل والربا والسرقة والقذف والغيبة والنميمة ونحو ذلك: فلا ينبغي أن يحوم حولها مخافة الوقوع فيها.
 قوله (ألا وإن في الجسد مضغة إذا صلحت صلح الجسد كله، وإذا فسدت فسد الجسد كله، ألا وهي القلب) هذا العضو هو أشرف الأعضاء لسرعة الخواطر فيه وتردده عليه، وقد خصّ الله تعالى بهذا العضو جنس الحيوان وأودع فيه تنظم المصالح المقصودة، ثم خصّ نوع الإنسان من سائر الحيوان بالعقل وأضافه إلى القلب. فإذا فهمت هذا ظهر لك قوله صلى الله عليه وسلم (ألا وإن في الجسد مضغة إذا صلحت صلح الجسد كله وإذا فسدت فسد الجسد كله)، فنسأل الله العظيم أن يصلح فساد قلوبنا، يا مقلب القلوب ثبت قلوبنا على دينك، يا مصرف القلوب صرف قلوبنا إلى طاعتك.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>الأشياء في حياتنا تنقسم إلى ثلاثة: حلال واضح، وحرام واضح، ومنطقة رمادية بينهما لا يعرف حكمها كثير من الناس. الحديث يعلمنا أن الابتعاد عن هذه المنطقة الرمادية هو حماية لديننا وسمعتنا معاً، لأن من اقترب من حدود الحرام - حتى لو لم يقع فيه فعلاً - عرّض نفسه لخطر الانزلاق فيه شيئاً فشيئاً، تماماً كراعٍ يرعى غنمه قرب أرض محمية ممنوعة، فمن السهل أن تتجاوز الحدود دون أن يشعر. ثم يختم الحديث بأعظم فائدة: أن كل هذا مرتبط بصلاح القلب، فهو الأمير الذي يتحكم في الجسد كله، إن صلح صلحت التصرفات، وإن فسد فسدت مهما بدت حسنة في الظاهر.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -698,25 +773,35 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
+          <t>أبو رقية تميم بن أوس الداري رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي رُقَيَّةَ تَمِيمِ بْنِ أَوْسٍ الدَّارِيِّ رَضِيَ اللهُ تَعَالَى عَنْهُ أَنَّ النَّبِيَّ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ:</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
           <t>الدِّينُ النَّصِيحَةُ. قُلْنَا: لِمَنْ؟ قَالَ: للهِ، وَلِكِتَابِهِ، وَلِرَسُولِهِ، وَلِأَئِمَّةِ الْمُسْلِمِينَ وَعَامَّتِهِمْ</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>ليس لتميم الداري رضي الله عنه في صحيح مسلم غير هذا الحديث. وقوله (النصيحة) كلمة جامعة معناها إرادة الخير للمنصوح له، وهي من أوجز الألفاظ وأجمعها للمعنى، وليس في كلام العرب كلمة مفردة تستوفي بها هذه العبارة عن المعنى المقصود منها. ومعنى قوله (الدين النصيحة) أي عماد الدين وقوامه النصيحة، كقوله (الحج عرفة) أي عماده ومعظمه.
 وأما تفسير النصيحة وأنواعها فقال الخطابي وغيره من العلماء: النصيحة لله تعالى معناها منصرف إلى الإيمان به ونفي الشرك عنه، وترك الإلحاد في صفاته، ووصفه بصفات الكمال والجلال، وتنزيهه عن جميع النقائص، والقيام بطاعته واجتناب معصيته، والحب فيه والبغض فيه، وجهاد من كفر به، والاعتراف بنعمته والشكر عليها، والإخلاص في جميع الأمور، والدعاء إلى جميع الأوصاف المذكورة والحث عليها والتلطف بالناس في ذلك.
 وأما النصيحة لكتابه سبحانه وتعالى فبالإيمان بأن كلام الله تعالى لا يشبهه شيء من كلام الخلق ولا يقدر على مثاله أحد من الخلق، ثم تعظيمه وتلاوته حق تلاوته، وتحسينها والخشوع عندها، وإقامة حروفه في التلاوة، والذب عنه من تأويل المحرِّفين، وتفهم علومه وأمثاله، والاعتبار بمواعظه، والتفكر في عجائبه، والعمل بمحكمه، والتسليم لمتشابهه، والبحث عن عمومه وخصوصه، والدعاء إليه.
 وأما النصيحة لرسوله صلى الله عليه وسلم فتصديقه في الرسالة، والإيمان بجميع ماجاء به، وطاعته في أمره ونهيه، ونصرته حياً وميتاً، ومعاداة من عاداه وموالاة من والاه، وإعظام حقه وتوقيره، وإحياء طريقته وسنته، ونشر سنته ونفي التهمة عنها، واستثمار علومها والتفقه فيها، والتلطف في تعليمها، وإجلالها وإجلال أهلها لانتسابهم إليها، والتخلق بأخلاقه، والتأدب بآدابه، ومحبة أهل بيته وأصحابه، ومجانبة من ابتدع في سنته أو تعرض لأحد من أصحابه.
 وأما نصيحة أئمة المسلمين فمعاونتهم على الحق وطاعتهم فيه، وأمرهم به وتنبيههم وتذكيرهم برفق ولطف، وإعلامهم بما أغفلوا عنه، وترك الخروج عليهم بالسيف، وتأليف قلوب الناس لطاعتهم فيما يوافق الحق. وأما نصيحة عامة المسلمين فإرشادهم لمصالحهم في آخرتهم ودنياهم، وإعانتهم عليها، وستر عوراتهم وسدّ خللهم، ودفع المضار عنهم وجلب المنافع لهم، وأمرهم بالمعروف ونهيهم عن المنكر بإخلاص وشفقة، وتوقير كبيرهم ورحمة صغيرهم، وتخوّلهم بالموعظة الحسنة، وترك غشهم وحسدهم، وأن يحب لهم ما يحب لنفسه من الخير ويكره لهم ما يكره لنفسه من المكروه.
-والنصيحة فرض كفاية، إذا قام بها من يكفي سقط عن غيره، وهي لازمة على قدر الطاقة.</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
+والنصيحة فرض كفاية، إذا قام بها من يكفي سقط عن غيره، وهي لازمة على قدر الطاقة. والنصيحة في اللغة: الإخلاص، يقال: نصحت العسل إذا صفّيته.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>كلمة واحدة تلخص الدين كله: النصيحة، أي إرادة الخير الصادقة. نصيحة لله بالإيمان الخالص وطاعته، ونصيحة لكتابه بتلاوته وتدبره والعمل به، ونصيحة لرسوله بمحبته واتباع سنته، ونصيحة لقادة المسلمين بمساندتهم في الحق وتنبيههم برفق لا بالتشهير، ونصيحة لعامة الناس بأن نريد لهم الخير كما نريده لأنفسنا، بستر عيوبهم ومساعدتهم والصدق معهم. الدين إذن ليس طقوساً منعزلة عن الناس، بل شبكة علاقات أساسها إرادة الخير الصادقة لكل طرف حولنا.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -731,23 +816,33 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
+          <t>عبد الله بن عمر رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>عَنِ ابْنِ عُمَرَ رَضِيَ اللهُ تَعَالَى عَنْهُمَا أَنَّ رَسُولَ اللهِ صَلَّى اللهُ تَعَالَى عَلَيْهِ وَعَلَى آلِهِ وَسَلَّمَ قَالَ:</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
           <t>أُمِرْتُ أَنْ أُقَاتِلَ النَّاسَ حَتَّى يَشْهَدُوا أَنْ لَا إِلَهَ إِلَّا اللهُ وَأَنَّ مُحَمَّدًا رَسُولُ اللهِ، وَيُقِيمُوا الصَّلَاةَ، وَيُؤْتُوا الزَّكَاةَ، فَإِذَا فَعَلُوا ذَلِكَ عَصَمُوا مِنِّي دِمَاءَهُمْ وَأَمْوَالَهُمْ إِلَّا بِحَقِّ الْإِسْلَامِ، وَحِسَابُهُمْ عَلَى اللهِ تَعَالَى</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>هذا حديث عظيم وقاعدة من قواعد الدين، وقد روي عن أنس رضي الله عنه بلفظ قريب منه. فإذا فعلوا ذلك عصموا منا دماءهم وأموالهم إلا بحقها، وحسابهم على الله تعالى. وجاء في صحيح مسلم من رواية أبي هريرة (حتى يشهدوا أن لا إله إلا الله ويؤمنوا بي وبما جئت به) وذلك موافق لرواية عمر رضي الله عنه في المعنى.
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>هذا حديث عظيم وقاعدة من قواعد الدين، وقد روي هذا الحديث عن أنس رضي الله عنه بلفظ: (حتى يشهدوا أن لا إله إلا الله وأن محمداً عبده ورسوله، وأن يستقبلوا قبلتنا، ويأكلوا ذبيحتنا، ويصلوا صلاتنا، فإذا فعلوا ذلك حرمت علينا دماؤهم وأموالهم إلا بحقها، ولهم ما للمسلمين وعليهم ما على المسلمين). وجاء في صحيح مسلم من رواية أبي هريرة (حتى يشهدوا أن لا إله إلا الله ويؤمنوا بي وبما جئت به) وذلك موافق لرواية عمر رضي الله عنه في المعنى.
 وأما معاني هذا الحديث فقال العلماء بالسر فيه: لما توفي رسول الله صلى الله عليه وسلم واستُخلف أبو بكر الصديق رضي الله عنه بعده، كفر من كفر من العرب، وعزم أبو بكر على قتالهم، ومنهم من منع الزكاة ولم يكفر وتأوّل في ذلك، فقال له عمر رضي الله عنه: كيف تقاتل الناس وقد قالوا لا إله إلا الله؟ وقد قال رسول الله صلى الله عليه وسلم (أمرت أن أقاتل الناس حتى يقولوا لا إله إلا الله)، فقال أبو بكر: إن الزكاة حق المال، والله لو منعوني عناقاً كانوا يؤدونه إلى رسول الله صلى الله عليه وسلم لقاتلتهم على منعه. فتابعه عمر رضي الله عنه على قتال القوم.
 قوله (أمرت أن أقاتل الناس حتى يقولوا لا إله إلا الله) فمن قال لا إله إلا الله فقد عصم مني نفسه وماله إلا بحقه وحسابه على الله. قال الخطابي وغيره: المراد بهذا أهل الأوثان ومشركي العرب ومن لا يؤمن دون أهل الكتاب ومن يقر بالتوحيد، إذ كان اكتفاؤه بقولهم لا إله إلا الله وهي من اعتقادهم في كفره، وكذلك جاء في الحديث الآخر (وأني رسول الله ويقيموا الصلاة ويؤتوا الزكاة)، ولابد مع هذا من الإيمان بجميع ماجاء به، كما جاء في الرواية الأخرى لأبي هريرة (حتى يشهدوا أن لا إله إلا الله ويؤمنوا بي وبما جئت به) ومعنى (وحسابهم على الله) أي فيما يسترونه ويخفونه دون ما يخالطون به في الظاهر من الأحكام الواجبة.
 وفيه أن من أظهر الإسلام وأسرّ الكفر يُقبل إسلامه في الظاهر، وذهب مالك إلى أن توبة الزنديق لا تُقبل، وهي رواية عن الإمام أحمد. وفيه أن أقاتل الناس حتى يشهدوا أن لا إله إلا الله ويؤمنوا بي وبما جئت به دلالة ظاهرة لمذهب المحققين من السلف والجماهير أن الإنسان إذا اعتقد دين الإسلام اعتقاداً جازماً لا يجب عليه تعلم أدلة المتكلمين ومعرفة الله بها، خلافاً لمن أوجب ذلك وجعله شرطاً في نحو أهل القبلة، فإن هذا خطأ ظاهر، فإن المراد التصديق الجازم لأن النبي صلى الله عليه وسلم اكتفى بما حصل، ولم يشترط المعرفة بهذا الدليل، وقد تظاهرت الأحاديث الصحيحة في مجموعها بحصول التواتر وأصلها العلم القطعي.</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>الإسلام دين واضح المعالم: شهادة التوحيد، وصلاة، وزكاة. من التزم بهذه الأمور الظاهرة يُعامل معاملة المسلمين في الحقوق والحرمة، وما في قلبه من صدق أو نفاق فأمره إلى الله وحده لا إلى الناس. هذا الحديث يعلمنا أن نحكم على تصرفات الناس الظاهرة لا على نواياهم الخفية، وأن نثق أن الحساب الحقيقي والدقيق ليس بأيدينا. كما يذكرنا بموقف أبي بكر الصديق الذي وقف بثبات في قرار صعب دفاعاً عن حق واضح، رغم معارضة من حوله في البداية، فكان الحق معه.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -762,25 +857,36 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة عبد الرحمن بن صخر رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ عَبْدِ الرَّحْمَنِ بْنِ صَخْرٍ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ: سَمِعْتُ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ يَقُولُ:</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
           <t>مَا نَهَيْتُكُمْ عَنْهُ فَاجْتَنِبُوهُ، وَمَا أَمَرْتُكُمْ بِهِ فَأْتُوا مِنْهُ مَا اسْتَطَعْتُمْ، فَإِنَّمَا أَهْلَكَ الَّذِينَ مِنْ قَبْلِكُمْ كَثْرَةُ مَسَائِلِهِمْ وَاخْتِلَافُهُمْ عَلَى أَنْبِيَائِهِمْ</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>هذا اللفظ رواه مسلم في كتابه عن أبي هريرة، وفي رواية أخرى: خطبنا رسول الله صلى الله عليه وسلم فقال: (يا أيها الناس، قد فرض الله عليكم الحج فحجوا)، فقال رجل: أكل عام يا رسول الله؟ فسكت، حتى قالها ثلاثاً، فقال النبي صلى الله عليه وسلم: (لو قلت نعم لوجبت، ولما استطعتم)، ثم قال: (ذروني ما تركتكم، فإنما أهلك من كان قبلكم كثرة سؤالهم واختلافهم على أنبيائهم، فإذا أمرتكم بشيء فأتوا منه ما استطعتم، وإذا نهيتكم عن شيء فدعوه).
-اختلف الأصوليون في الأمر المطلق هل يقتضي التكرار؟ فاختار أكثر الفقهاء والمتكلمين أنه لا يقتضي التكرار، وقال آخرون: يقتضيه، وهذا الحديث يُستدل به من قال بعدم اقتضائه التكرار، لأنه لو كان الأمر المطلق يقتضي التكرار لم يقل النبي صلى الله عليه وسلم لما سأل (أكل عام) (لو قلت نعم لوجبت)، بل كان محمولاً على ذلك أصلاً، وأجمعت الأمة على أن الحج لا يجب في العمر إلا مرة واحدة بأصل الشرع.
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>هذا اللفظ رواه مسلم في كتابه عن أبي هريرة، وفي رواية أخرى: خطبنا رسول الله صلى الله عليه وسلم فقال: (يا أيها الناس، قد فرض الله عليكم الحج فحجوا)، فقال رجل -وهو الأقرع بن حابس كما جاء مبيناً في غير هذه الرواية-: أكل عام يا رسول الله؟ فسكت، حتى قالها ثلاثاً، فقال النبي صلى الله عليه وسلم: (لو قلت نعم لوجبت، ولما استطعتم)، ثم قال: (ذروني ما تركتكم، فإنما أهلك من كان قبلكم كثرة سؤالهم واختلافهم على أنبيائهم، فإذا أمرتكم بشيء فأتوا منه ما استطعتم، وإذا نهيتكم عن شيء فدعوه).
+واختلف الأصوليون في الأمر المطلق هل يقتضي التكرار؟ فاختار أكثر الفقهاء والمتكلمين أنه لا يقتضي التكرار، وقال آخرون: لا يُحكم بإيجابه ولا بمنعه، بل يُتوقف فيما زاد على مرة حتى يرد البيان. وهذا الحديث يُستدل به على ذلك، لأنه لما سأل السائل (أكل عام؟) لو كان الأمر المطلق يقتضي التكرار أو عدمه على وجه معلوم لم يكن للسؤال معنى، ولم يقل له النبي صلى الله عليه وسلم (لو قلت نعم لوجبت)، بل كان محمولاً على ذلك أصلاً. وأجمعت الأمة على أن الحج لا يجب في العمر إلا مرة واحدة بأصل الشرع، وأما قوله (ذروني ما تركتكم) فهو ظاهر في أن الأمر لا يقتضي التكرار.
 ويدل هذا اللفظ أيضاً على أن الأصل عدم الوجوب لا الحكم قبل ورود الشرع، وهو الصحيح عند كثير من الأصوليين، ودليل على المذهب الصحيح في أنه صلى الله عليه وسلم كان له أن يجتهد له في الأحكام وأنه لا يشترط أن يكون حكمه بوحي.
-وقوله (وما أمرتكم به فأتوا منه ما استطعتم) من قواعد الإسلام المهمة، ومما أوتيه صلى الله عليه وسلم من جوامع الكلم، ويدخل فيه ما لا يُحصى من الأحكام: كالصلاة، إذا عجز عن بعض أركانها أتى بالباقي وما عجز عن بعض شروطها أتى بالممكن، وكذلك إذا عجز عن غسل بعض أعضاء الوضوء غسل الممكن، وكذلك إذا وجبت فطرة من جماعة يلزمهم نفقته أن يزيلوا المنكرات بحسب الإمكان لمن لا يمكنه إزالتها جميعاً، وأشباه ذلك مما لا ينحصر، وهذا مشهور في كتب الفقه كقوله تعالى (فاتقوا الله ما استطعتم).
+قوله (وما أمرتكم به فأتوا منه ما استطعتم) من قواعد الإسلام المهمة، ومما أوتيه صلى الله عليه وسلم من جوامع الكلم، ويدخل فيه ما لا يُحصى من الأحكام: كالصلاة، إذا عجز عن بعض أركانها أتى بالباقي وما عجز عن بعض شروطها أتى بالممكن، وكذلك إذا عجز عن غسل بعض أعضاء الوضوء غسل الممكن، وكذلك إذا وجبت فطرة من جماعة يلزمهم نفقته أن يزيلوا المنكرات بحسب الإمكان لمن لا يمكنه إزالتها جميعاً، وأشباه ذلك مما لا ينحصر، وهذا مشهور في كتب الفقه كقوله تعالى (فاتقوا الله ما استطعتم).
+وأما قوله تعالى: (يا أيها الذين آمنوا اتقوا الله حق تقاته) فقيل: هي منسوخة بقوله تعالى (فاتقوا الله ما استطعتم). وقال بعضهم: ليست منسوخة بها، بل هي مفسِّرة لها ومبيّنة للمراد منها، قالوا: و(حق تقاته) هو امتثال أمره واجتناب نواهيه، فإن الله سبحانه لا يأمر إلا بالمستطاع، قال تعالى (لا يكلف الله نفساً إلا وسعها)، وقال تعالى (وما جعل عليكم في الدين من حرج).
 وأما النهي فالأصل فيه أن لا يكون ممتثلاً للنهي حتى يترك كل ما نُهي عنه ولا يخرج عن ذلك فعل واحد بخلاف الأمر، إلا عند الضرورة ونحوها فهذا لا يكون منهياً عنه في هذا الحال.
 وقوله (فإنما أهلك من قبلكم كثرة مسائلهم واختلافهم على أنبيائهم) أراد بذلك كثرة السؤال وربما يكثر الجواب عليه لكثرته، فيضاهي ذلك قصة بني إسرائيل لما أُمروا بأن يذبحوا بقرة، فلو اقتصروا على ما يصدق عليه اللفظ أي بقرة وبادروا بذبحها لأجزأت عنهم، لكن لما أكثروا السؤال وشددوا عليهم وذمّوا على ذلك، فخاف النبي صلى الله عليه وسلم مثل ذلك على أمته.</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>قاعدة عملية بسيطة توزّع علينا الجهد بعدل: كل ما نهانا الله عنه علينا تركه كاملاً بلا استثناء، وأما ما أمرنا به فنؤديه بقدر طاقتنا، لا يُطلب منا الكمال المطلق فيه دفعة واحدة. سبب هذا التوجيه أن أمماً سابقة هلكت بسبب كثرة الأسئلة والتعقيد والاختلاف على أنبيائها، فبدل أن يأخذوا الأمر ببساطة، حمّلوا أنفسهم تفاصيل وتشديدات لم تكن مطلوبة منهم أصلاً. الحديث يعلمنا أن نبدأ بالمتاح ونتدرج، بدل أن نتوقف عن الفعل بحجة أننا لا نستطيع الكمال، وأن نتجنب المبالغة في التساؤل عما لم يُطلب منا أصلاً.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -795,22 +901,32 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ: قَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ:</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
           <t>إِنَّ اللهَ تَعَالَى طَيِّبٌ لَا يَقْبَلُ إِلَّا طَيِّبًا، وَإِنَّ اللهَ أَمَرَ الْمُؤْمِنِينَ بِمَا أَمَرَ بِهِ الْمُرْسَلِينَ فَقَالَ تَعَالَى: يَا أَيُّهَا الرُّسُلُ كُلُوا مِنَ الطَّيِّبَاتِ وَاعْمَلُوا صَالِحًا، وَقَالَ تَعَالَى: يَا أَيُّهَا الَّذِينَ آمَنُوا كُلُوا مِنْ طَيِّبَاتِ مَا رَزَقْنَاكُمْ، ثُمَّ ذَكَرَ الرَّجُلَ يُطِيلُ السَّفَرَ أَشْعَثَ أَغْبَرَ يَمُدُّ يَدَيْهِ إِلَى السَّمَاءِ: يَا رَبِّ يَا رَبِّ، وَمَطْعَمُهُ حَرَامٌ، وَمَشْرَبُهُ حَرَامٌ، وَمَلْبَسُهُ حَرَامٌ، وَغُذِيَ بِالْحَرَامِ، فَأَنَّى يُسْتَجَابُ لَهُ</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>قيل: (الطيب) في صفات الله بمعنى المنزّه عن النقائص. وهذا الحديث أحد الأحاديث التي عليها قواعد الإسلام ومباني الأحكام، وفيه الحث على الإنفاق من الحلال، والنهي عن الإنفاق من غيره، وأن المأكول والمشروب والملبوس ونحوها ينبغي أن يكون حلالاً لا شبهة فيه، وفيه أن من أراد الدعاء كان أولى بالاعتناء بذلك أن ينفق مما فيه نفقة طيبة تزكو وتنمو، وأن الطعام اللذيذ غير المباح يكون وبالاً على آكله ولا يقبل الله عمله ولا يقبل معه دعاء.
 ثم ذكر الرجل يطيل السفر أشعث أغبر يمد يديه إلى السماء، معناه -والله أعلم- يطيل السفر في وجوه الطاعات من حج وجهاد وغير ذلك من وجوه البر، ومع ذلك لا يُستجاب له لكون مطعمه ومشربه وملبسه حراماً، فكيف بمن هو منهمك في الدنيا في مظالم العباد أو من الغافلين عن أنواع العبادات والخيرات؟
 قوله (يمد يديه) أي يرفعهما بالدعاء مع مخالفته لله ومعصيته. وقوله (وغُذِي بالحرام) هو بضم الغين المعجمة وتخفيف الذال المكسورة. وقوله (فأنّى يستجاب له) أي من أين يستجاب لمن هذه صفته؟ فإنه ليس أهلاً للإجابة، لكن يجوز أن يستجيب الله له تفضلاً ولطفاً وكرماً.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>الله سبحانه طيب لا يقبل من الأعمال والصدقات والأموال إلا ما كان طيباً حلالاً، ويأمر المؤمنين بما أمر به الأنبياء أنفسهم: الأكل من الطيبات. ثم يضرب مثلاً مؤثراً: رجل أنهكه السفر، أشعث الشعر مغبر الثياب، يرفع يديه للسماء بإلحاح يا رب يا رب، لكن طعامه وشرابه وملبسه كلها حرام، فكيف يُستجاب له؟ هذا الحديث يذكرنا أن الحرص على الدعاء وحده لا يكفي، بل لابد أن يكون أساسنا نظيفاً: مصدر رزقنا، وطريقة كسبنا، وما ندخله لبيوتنا وبطوننا. فالتعب والإلحاح في الدعاء لا يعوّض عن تلوث المصدر.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -825,21 +941,31 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
+          <t>أبو محمد الحسن بن علي بن أبي طالب سبط رسول الله صلى الله عليه وسلم وريحانته رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي مُحَمَّدٍ الْحَسَنِ بْنِ عَلِيِّ بْنِ أَبِي طَالِبٍ سِبْطِ رَسُولِ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ وَرَيْحَانَتِهِ رَضِيَ اللهُ عَنْهُمَا قَالَ: حَفِظْتُ مِنْ رَسُولِ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ:</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
           <t>دَعْ مَا يَرِيبُكَ إِلَى مَا لَا يَرِيبُكَ</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>قوله (يريبك) يروى بفتح الياء وضمها، والفتح أفصح وأشهر، ويجوز الضم أيضاً، يقال: رابني الشيء وأرابني، ومعناه: اترك الشيء الذي تشك فيه إلى ما لا تشك فيه، واعدل إلى ما لا يشكّك فيه.
 وهذا راجع إلى معنى الحديث السادس (إن الحلال بيّن وإن الحرام بيّن وبينهما أمور مشتبهات) وقد جاء في حديث آخر أن النبي صلى الله عليه وسلم قال: (لا يبلغ العبد أن يكون من المتقين حتى يترك ما لا بأس به مخافة ما به بأس)، وهذه درجة أعلى من مجرد اتقاء الشبهات، فهي تدفع الإنسان إلى ترك حتى ما لا شبهة فيه احتياطاً وورعاً، وذلك من كمال التقوى.</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>قاعدة موجزة لكنها عميقة: كلما شعرت بالتردد أو القلق تجاه أمر، اتركه إلى ما يريحك ويقينك فيه أوضح. هذا الحديث درجة أرقى من مجرد اجتناب الحرام الواضح، فهو يدعو إلى الاحتياط حتى في الأمور التي لا شبهة واضحة فيها، إذا كان القلب لا يطمئن إليها. فاليقين طريق الراحة، والشك طريق القلق، ومن اعتاد أن يختار اليقين في كل قراراته الصغيرة والكبيرة عاش حياة أكثر استقراراً وسكينة.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -854,22 +980,32 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ: قَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ:</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
           <t>مِنْ حُسْنِ إِسْلَامِ الْمَرْءِ تَرْكُهُ مَا لَا يَعْنِيهِ</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>قال بعض من صحح طرق هذا الحديث: هذا من الكلام الجامع للمعاني الجليلة الكثيرة في الألفاظ القليلة، ونحو ذلك قول أبي ذر رضي الله عنه في بعض حديثه: هذا من جوامع كلامه. ومن حسب كلامه من عمله قلّ كلامه فيما لا يعنيه.
 وذكر مالك أنه بلغه أن لقمان الحكيم قيل له: ما بلغ بك ما نرى -يريدون الفضل- قال: صدق الحديث، وأداء الأمانة، وترك ما لا يعنيني. وروي عن الحسن قال: من علامة إعراض الله تعالى عن العبد أن يجعل شغله فيما لا يعنيه.
 قال أبو داود: أصول السنن تدور على أربعة أحاديث، وذكر منها هذا الحديث، وذلك لعظم موقعه وكثرة فوائده في ضبط الإنسان لوقته وجهده ولسانه وفكره فيما ينفعه في دينه ودنياه.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>علامة رقي إيمان الإنسان أنه يترك الانشغال بما لا يخصه: أخبار الناس التي لا تعنيه، تفاصيل حياتهم التي لا شأن له بها، جدالات لا طائل منها. هذا لا يعني البرود أو عدم الاهتمام بالآخرين، بل يعني توجيه الطاقة والوقت لما ينفع فعلاً: نفسه، أهله، عمله، آخرته. فحسن الإسلام هنا مقياس عملي بسيط: كل ما لا فائدة منه ولا تعنيك نتيجته، الأفضل أن تتركه وتفرغ نفسك لما هو أجدى.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="H13" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -884,10 +1020,20 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
+          <t>أبو حمزة أنس بن مالك رضي الله عنه، خادم رسول الله صلى الله عليه وسلم</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي حَمْزَةَ أَنَسِ بْنِ مَالِكٍ رَضِيَ اللهُ تَعَالَى عَنْهُ خَادِمِ رَسُولِ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ عَنِ النَّبِيِّ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ:</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
           <t>لَا يُؤْمِنُ أَحَدُكُمْ حَتَّى يُحِبَّ لِأَخِيهِ مَا يُحِبُّ لِنَفْسِهِ</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>هكذا جاء في صحيح البخاري (لأخيه) من غير شك، وجاء في صحيح مسلم (لأخيه -أو لجاره- على الشك). قال العلماء: يعني لا يؤمن أحدكم الإيمان الكامل التام إلا بهذه الصفة، وإلا فأصل الإيمان يحصل لمن لم يكن بهذه الصفة. والمراد: يحب لأخيه من الطاعات والأشياء المباحة، ويدل عليه ما جاء في رواية النسائي (حتى يحب لأخيه من الخير ما يحب لنفسه).
 قال الشيخ أبو عمرو بن الصلاح: وهذا قد يُعدّ من الصعب الممتنع، وليس كذلك، إذ لا يلزم من حصول ذلك القيام بأن يحصل له من جهة أخيه مثل ما يحب أن يحصل له من النعمة بحيث لا ينتقص عليه شيء منها، وإنما يكون ذلك سهلاً قريباً على القلب السليم، ويعسر ذلك على القلب الدَّغِل، عافانا الله تعالى وإخواننا أجمعين.
@@ -896,12 +1042,12 @@
 وقال بعض العلماء: في هذا الحديث من الفقه أن المؤمن مع المؤمن كالنفس الواحدة، فينبغي أن يحب له ما يحب لنفسه، من حيث إنهما نفس واحدة، كما جاء في الحديث الآخر (المؤمنون كالجسد الواحد إذا اشتكى منه عضو تداعى له سائر الجسد بالحمى والسهر).</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>المقياس الحقيقي لكمال الإيمان في هذا الحديث ليس العبادة وحدها، بل أن تتمنى لأخيك الإنسان الخير الذي تتمناه لنفسك، وأن تفرح لنجاحه كما تفرح لنجاحك. هذا صعب على النفس التي تحب التميز وحدها، لكنه سهل وطبيعي على القلب النقي الخالي من الحسد. والحديث لا يطلب المستحيل - أن تحصل لأخيك كل نعمة تحصل لك بالضبط - بل يطلب أن تكون رغبتك الصادقة أن يناله الخير مثلك، وهذا هو أساس المجتمع المتماسك الذي يشعر أفراده ببعضهم كأنهم جسد واحد.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -916,24 +1062,36 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
+          <t>عبد الله بن مسعود رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>عَنِ ابْنِ مَسْعُودٍ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ: قَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ:</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
           <t>لَا يَحِلُّ دَمُ امْرِئٍ مُسْلِمٍ إِلَّا بِإِحْدَى ثَلَاثٍ: الثَّيِّبُ الزَّانِي، وَالنَّفْسُ بِالنَّفْسِ، وَالتَّارِكُ لِدِينِهِ الْمُفَارِقُ لِلْجَمَاعَةِ</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>وفي بعض الروايات المتفق عليها (لا يحل دم امرئ مسلم يشهد أن لا إله إلا الله وأني رسول الله إلا بإحدى ثلاث)، فقوله (يشهد أن لا إله إلا الله وأني رسول الله) كالتفسير لقوله (مسلم)، وكذا قوله (التارك لدينه المفارق للجماعة) كالتفسير للحالة الثالثة، وهؤلاء الثلاثة مباحو الدم بالنص، والمراد المسلمون.
 وقوله (التارك لدينه المفارق للجماعة) عام في كل مرتد بأي ردة كانت، فيجب قتله إن لم يرجع إلى الإسلام. قال العلماء: ويتناول أيضاً كل خارج عن الجماعة ببدعة أو بغي أو غيرهما، والله أعلم.
-وقد استدلّ بعضهم على أن تارك الصلاة يُقتل لأنه يُسمى من تركها من هذه الثلاثة، وفي هذه المسألة خلاف بين العلماء: منهم من يكفّر تارك الصلاة، ومنهم من لا يكفّره.
+والظاهر أن هذا الحديث عامٌّ يُخصّ منه الصائل ونحوه، فيُباح قتله دفعاً لأذاه، وقد يُجاب عن هذا بأنه داخل في معنى (المفارق للجماعة)، ويكون المراد: لا يحل تعمّد قتله إلا في هؤلاء الثلاثة، والله أعلم.
+وقد استدلّ بعضهم على أن تارك الصلاة يُقتل، لأن ترك الصلاة تُلحقه بـ(التارك لدينه) من هذه الثلاث، وفي هذه المسألة خلاف بين العلماء: منهم من يكفّر تارك الصلاة، ومنهم من لا يكفّره. واستدلّ بعض من يكفّره بالحديث الآخر، وهو قوله صلى الله عليه وسلم (أُمرت أن أقاتل الناس حتى يشهدوا أن لا إله إلا الله، ويقيموا الصلاة، ويؤتوا الزكاة)، ووجه الاستدلال أنه صلى الله عليه وسلم وقف عصمة الدم والمال على مجموع الشهادتين وإقام الصلاة وإيتاء الزكاة معاً، فإذا انتفى واحد منها انتفت العصمة.
+وقد أُجيب عن هذا الاستدلال بأن في الحديث فرقاً بين المقاتلة والقتل: فقوله (أُمرت أن أقاتل الناس) إنما يقتضي وجوب قتالهم حتى يأتوا بهذه الأمور، والمقاتلة مفاعلة تقتضي الحصول من الجانبين معاً، فلا يلزم من وجوب مقاتلة تارك الصلاة إذا امتنع وقاتَل، وجوبُ قتله مجرداً إذا تركها من غير أن يقاتلنا أو يخرج علينا. والله أعلم.
 وقوله (الثيّب الزاني) هو المحصن، ويدخل فيه الذكر والأنثى، وهو حجة على ما اتفق عليه المسلمون من أن حكم الزاني المحصن الرجم بشروطه المذكورة في أبواب الفقه.
 وقوله (النفس بالنفس) موافق لقوله تعالى (وكتبنا عليهم فيها أن النفس بالنفس)، ويُعنى به النفوس المتكافئة في الإسلام والحرية، بدليل قوله صلى الله عليه وسلم (لا يُقتل مسلم بكافر)، وكذلك الحرية شرط عند مالك والشافعي وأحمد، وذهب أصحاب الرأي إلى أن المسلم يُقتل بالذمي، وأن الحر يُقتل بالعبد، وقد يستدلون بهذا الحديث خلاف ذلك.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>الحياة الإنسانية في الإسلام محفوظة الحرمة تماماً، ولا يجوز إزهاق نفس مسلمة إلا في ثلاث حالات محددة بدقة: القتل قصاصاً عن قتل، والزنا بعد الإحصان بشروطه الشرعية الصارمة، والردة عن الدين مع الخروج على الجماعة ومحاربتها. هذا الحديث يرسم حدوداً واضحة لتقدير الحياة الإنسانية، فلا مجال للانتقام الفردي أو الحكم العشوائي، فالأمر محكوم بضوابط شرعية وقضائية دقيقة، وليس متروكاً للأهواء أو الغضب اللحظي.</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -948,23 +1106,35 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ رَضِيَ اللهُ تَعَالَى عَنْهُ أَنَّ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ:</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
           <t>مَنْ كَانَ يُؤْمِنُ بِاللهِ وَالْيَوْمِ الْآخِرِ فَلْيَقُلْ خَيْرًا أَوْ لِيَصْمُتْ، وَمَنْ كَانَ يُؤْمِنُ بِاللهِ وَالْيَوْمِ الْآخِرِ فَلْيُكْرِمْ جَارَهُ، وَمَنْ كَانَ يُؤْمِنُ بِاللهِ وَالْيَوْمِ الْآخِرِ فَلْيُكْرِمْ ضَيْفَهُ</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>قوله (من كان يؤمن بالله واليوم الآخر) يعني من كان يؤمن الإيمان الكامل المنجي من عذاب الله الموصل إلى رضوان الله، فليقل خيراً أو ليصمت، لأن من آمن بالله حق إيمانه خاف وعيده ورجا ثوابه، واجتهد في فعل ما أُمر به وترك ما نُهي عنه. وأهم ما عليه من ذلك: ضبط جوارحه التي هي رعاياه وهو مسؤول عنها، كما قال تعالى (إن السمع والبصر والفؤاد كل أولئك كان عنه مسؤولاً) وقال تعالى (ما يلفظ من قول إلا لديه رقيب عتيد)، وآفات اللسان كثيرة.
 وقد قال النبي صلى الله عليه وسلم (هل يكبّ الناس في النار على مناخرهم إلا حصائد ألسنتهم؟). وقال: كل كلام ابن آدم عليه لا له، إلا أمراً بمعروف أو نهياً عن منكر أو ذكر الله تعالى.
 وإذا أراد الإنسان أن يتكلم، فإن كان ما يتكلم به خيراً محققاً يُثاب عليه فليتكلم، وإلا فليمسك عن الكلام سواء ظهر أنه حرام أو مكروه أو مباح، فعل هذا الكلام المباح مأموراً بتركه إلى الإمساك مخافة أن يجرّ إلى المحرم أو المكروه، وقد يقع ذلك كثيراً.
-وقوله صلى الله عليه وسلم (فليكرم جاره... فليكرم ضيفه) فيه تعريف لحق الجار والضيف وحث وبرّ لحفظ الجوارح. وقد أوصى الله تعالى في كتابه بالجار، وقال صلى الله عليه وسلم (ما زال جبريل عليه السلام يوصيني بالجار حتى ظننت أنه سيورّثه). والضيافة من الإسلام وخلق النبيين والصالحين، وقد أوجبها بعض العلماء وأكثرهم على أنها من مكارم الأخلاق، وذلك بأن يبادر بالبشاشة في وجه الضيف ويطيب الحديث له، وعماد أمر الضيافة إطعام الطعام بما فتح الله من غير كلفة.</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
+واختلف العلماء: هل يُكتب على الإنسان جميع ما يتلفّظ به وإن كان مباحاً، أو لا يُكتب عليه إلا ما يترتب عليه ثواب أو عقاب؟ فذهب ابن عباس رضي الله عنهما وغيره إلى القول الثاني، وعلى هذا يكون قوله تعالى (ما يلفظ من قول إلا لديه رقيب عتيد) مخصوصاً، أي: ما يلفظ من قول له جزاء إلا لديه رقيب عتيد.
+وقوله صلى الله عليه وسلم (فليكرم جاره... فليكرم ضيفه) فيه تعريف لحق الجار والضيف وحث وبرّ لحفظ الجوارح. وقد أوصى الله تعالى في كتابه بالجار، وقال صلى الله عليه وسلم (ما زال جبريل عليه السلام يوصيني بالجار حتى ظننت أنه سيورّثه). والضيافة من الإسلام وخلق النبيين والصالحين، وقد أوجبها بعض العلماء وأكثرهم على أنها من مكارم الأخلاق، وذلك بأن يبادر بالبشاشة في وجه الضيف ويطيب الحديث له، وعماد أمر الضيافة إطعام الطعام بما فتح الله من غير كلفة.
+وأما قوله صلى الله عليه وسلم (فليقل خيراً أو ليصمت) ففيه دليل على أن قول الخير أفضل من الصمت، وأن الصمت خير من قول الشر؛ وذلك أنه صلى الله عليه وسلم أمر بلام الأمر بقول الخير وبدأ به قبل ذكر الصمت. ومن قول الخير: الإبلاغ عن الله تعالى وعن رسوله صلى الله عليه وسلم، وتعليم المسلمين، والأمر بالمعروف عن علم، والنهي عن المنكر عن علم، والإصلاح بين الناس، وأن يقول للناس حسناً. ومن أفضل الكلمات كلمة حق تُقال عند من يُخاف حسابه ويُرجى ثوابه.</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>علامات الإيمان الحقيقي الثلاث في هذا الحديث كلها تتعلق بحقوق الآخرين علينا: أن تتحكم في لسانك فلا تقول إلا خيراً وإلا صمتّ، وأن تحسن إلى جارك، وأن تكرم من يزورك ضيفاً. اللسان أداة قوية جداً، وأكثر خطايا الناس تأتي من كلمة قيلت في غير محلها، لذلك يضع الحديث معياراً بسيطاً وحاسماً: إما كلام نافع، وإما صمت. أما إكرام الجار والضيف فهما امتحان حقيقي للأخلاق في أقرب دوائرنا الاجتماعية، حيث لا يوجد مجال للتظاهر، فالجار يرانا كما نحن فعلاً.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="H16" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -979,22 +1149,32 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ رَضِيَ اللهُ تَعَالَى عَنْهُ</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
           <t>أَنَّ رَجُلًا قَالَ لِلنَّبِيِّ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ: أَوْصِنِي، قَالَ: لَا تَغْضَبْ، فَرَدَّدَ مِرَارًا، قَالَ: لَا تَغْضَبْ</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>قال صاحب الإفصاح: من الجائز أن النبي صلى الله عليه وسلم علم من هذا الرجل كثرة الغضب فخصّه بهذه الوصية. وقد مدح النبي صلى الله عليه وسلم من يملك نفسه عند الغضب فقال: (ليس الشديد بالصُّرَعة، إنما الشديد الذي يملك نفسه عند الغضب)، ومدح الله تعالى الكاظمين الغيظ والعافين عن الناس. وقد روي عن النبي صلى الله عليه وسلم أنه قال: (من كظم غيظه وهو يستطيع أن ينفذه دعاه الله عز وجل على رؤوس الخلائق يوم القيامة حتى يخيّره من الحور ما شاء).
 وقد جاء في الحديث (إن الغضب من الشيطان)، ولهذا يخرج به الإنسان من اعتدال حاله، فيتكلم بالباطل، ويرتكب المذموم، وينوي الحقد والبغضاء وغير ذلك من القبائح المحرمة، كل ذلك من الغضب أعاذنا الله منه.
-وقد جاء في حديث سليمان بن صرد (إن الاستعاذة بالله من الشيطان الرجيم تذهب الغضب) وذلك أن الشيطان هو الذي يزيّن الغضب، وكل من حرص على ما تحمد عاقبته فإن الشيطان يبعده من رضى الله عز وجل، فالاستعاذة بالله من ذلك من أقوى السلاح لدفع كيده.</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
+وقد جاء في حديث سليمان بن صرد (إن الاستعاذة بالله من الشيطان الرجيم تذهب الغضب) وذلك أن الشيطان هو الذي يزيّن الغضب، وكل من حرص على ما تحمد عاقبته فإن الشيطان يبعده من رضى الله عز وجل، فالاستعاذة بالله من ذلك من أقوى السلاح على دفع كيده.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>طلب رجل من النبي صلى الله عليه وسلم وصية جامعة، فكررها عليه مرات: لا تغضب. لأن الغضب باب يُفتح منه كل شر: كلام لا يُقال في الهدوء، قرارات نادمون عليها، علاقات تنكسر في لحظة. الوصية بسيطة لكنها عميقة: كظم الغيظ فضيلة عظيمة مدح الله أهلها، والاستعاذة بالله من الشيطان عند اشتعال الغضب سلاح فعّال لإخماده قبل أن يتحكم في تصرفاتنا وكلامنا.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1009,22 +1189,32 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
+          <t>أبو يعلى شداد بن أوس رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي يَعْلَى شَدَّادِ بْنِ أَوْسٍ رَضِيَ اللهُ تَعَالَى عَنْهُ عَنْ رَسُولِ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ:</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
           <t>إِنَّ اللهَ كَتَبَ الْإِحْسَانَ عَلَى كُلِّ شَيْءٍ، فَإِذَا قَتَلْتُمْ فَأَحْسِنُوا الْقِتْلَةَ، وَإِذَا ذَبَحْتُمْ فَأَحْسِنُوا الذَّبْحَةَ، وَلْيُحِدَّ أَحَدُكُمْ شَفْرَتَهُ، وَلْيُرِحْ ذَبِيحَتَهُ</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>هذا الحديث من الأحاديث الجامعة لقواعد كثيرة، فقد كتب الله الإحسان على كل شيء حتى في أصعب المواقف التي قد يظن الإنسان أنه لا مجال للرفق فيها.
-ومعنى إحسان القتل (في القتل المشروع كالقصاص): أن يجتهد الفاعل في ذلك ولا يقصد التعذيب أو الإطالة في الإيلام. وإحسان الذبح: أن يرفق بالبهيمة، ولا يجرها من موضع إلى موضع، ويوجهها إلى القبلة، ويسمي ويحمد، ويحدّ شفرته قبل الذبح حتى لا يطيل عليها الألم، ويقطع الحلقوم والودجين، ويتركها إلى أن تبرد ولا يسلخها قبل أن تموت تماماً.
-وفي هذا الحديث الاعتراف لله تعالى بالمنّة والشكر على نعمه، فإنه سبحانه سخّر لنا البهائم وما شاء لنا وأباح لنا منها ما شاء وحرّم علينا ما شاء، فينبغي أن نقابل هذا التسخير بالرفق لا بالقسوة.</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
+ومعنى إحسان القتل (في القتل المشروع كالقصاص): أن يجتهد الفاعل في ذلك ولا يقصد التعذيب أو الإطالة في الإيلام. وإحسان الذبح: أن يرفق بالبهيمة، ولا يجرها من موضع إلى موضع، ولا يصرعها بغتة، ويوجهها إلى القبلة، ويسمي ويحمد، ويحدّ شفرته قبل الذبح حتى لا يطيل عليها الألم، ويقطع الحلقوم والودجين، ويتركها إلى أن تبرد.
+وفي هذا الحديث الاعتراف لله تعالى بالمنّة والشكر على نعمه، فإنه سبحانه سخّر لنا ما لا سلطة لنا عليه، وأباح لنا ما لو شاء لحرّمه علينا، فينبغي أن نقابل هذا التسخير بالرفق لا بالقسوة.</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>قاعدة عامة تشمل كل تصرفاتنا: الإحسان مكتوب على كل شيء، حتى في أشد المواقف قسوة كالقتل المشروع (القصاص) والذبح. فإذا كان الشرع يطلب الرفق حتى مع الحيوان في لحظة إزهاق روحه - بشحذ الأداة وعدم إطالة الألم - فكيف بتعاملنا اليومي مع البشر من حولنا؟ هذا الحديث يرسخ مبدأ أن الرحمة ليست خياراً في اللحظات السهلة فقط، بل التزام حتى في أصعب الظروف وأكثرها توتراً.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="H18" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1039,22 +1229,32 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
+          <t>أبو ذر جندب بن جنادة، وأبو عبد الرحمن معاذ بن جبل رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي ذَرٍّ جُنْدُبِ بْنِ جُنَادَةَ، وَأَبِي عَبْدِ الرَّحْمَنِ مُعَاذِ بْنِ جَبَلٍ رَضِيَ اللهُ تَعَالَى عَنْهُمَا عَنْ رَسُولِ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ:</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
           <t>اتَّقِ اللهَ حَيْثُمَا كُنْتَ، وَأَتْبِعِ السَّيِّئَةَ الْحَسَنَةَ تَمْحُهَا، وَخَالِقِ النَّاسَ بِخُلُقٍ حَسَنٍ</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>مناقب أبي ذر رضي الله عنه كثيرة، أسلم ورسول الله صلى الله عليه وسلم بمكة، وأمره أن يلحق بقومه، فلما رأى حرصه على المقام معه بمكة وعلم أنه لا يقدر له على ذلك، قال له رسول الله صلى الله عليه وسلم: (اتق الله حيثما كنت وأتبع السيئة الحسنة تمحها).
-وهذا موافق لقوله تعالى (إن الحسنات يذهبن السيئات). وقوله (وخالق الناس بخلق حسن) معناه: عامل الناس بما تحب أن يعاملوك به، واعلم أن أنبل موضوع في الميزان الخلق الحسن.
-وقال رسول الله صلى الله عليه وسلم: (إن أحبكم إليّ وأقربكم مني مجلساً يوم القيامة أحسنكم أخلاقاً)، وحسن الخلق من صفات النبيين والمرسلين وخيار المؤمنين، لا يجزعون بالسيئة، بل يعفون ويصفحون ويحسنون مع الإساءة إليهم.</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
+وهذا موافق لقوله تعالى (إن الحسنات يذهبن السيئات). وقوله (وخالق الناس بخلق حسن) معناه: عامل الناس بما تحب أن يعاملوك به، واعلم أن أثقل ما يوضع في الميزان الخلق الحسن.
+وقال رسول الله صلى الله عليه وسلم: (إن أحبكم إليّ وأقربكم مني مجلساً يوم القيامة أحاسنكم أخلاقاً)، وحسن الخلق من صفات النبيين والمرسلين وخيار المؤمنين، لا يجزعون بالسيئة، بل يعفون ويصفحون ويحسنون مع الإساءة إليهم.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>ثلاث وصايا عملية مكثفة تصلح لأي زمان ومكان: تقوى الله في كل مكان -سواء كنت وسط الناس أو وحدك تماماً- لا تتغير بتغير المكان أو الظروف؛ ومتابعة كل خطأ بحسنة تمحوه فلا نبقى أسرى الشعور بالذنب دون فعل يعوضه؛ وحسن الخلق مع الناس جميعاً، وهو أثقل شيء في ميزان الأعمال يوم القيامة. هذه الوصية الجامعة تجعل التدين واقعياً وعملياً: لا يُقاس بمكان العبادة فقط، بل بكيفية تعاملنا مع أخطائنا ومع الناس من حولنا في كل موقف.</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="H19" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1069,25 +1269,35 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
+          <t>أبو العباس عبد الله بن عباس رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي الْعَبَّاسِ عَبْدِ اللهِ بْنِ عَبَّاسٍ رَضِيَ اللهُ تَعَالَى عَنْهُمَا قَالَ:</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
           <t>كُنْتُ خَلْفَ النَّبِيِّ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ يَوْمًا فَقَالَ: يَا غُلَامُ، إِنِّي أُعَلِّمُكَ كَلِمَاتٍ: احْفَظِ اللهَ يَحْفَظْكَ، احْفَظِ اللهَ تَجِدْهُ تُجَاهَكَ، إِذَا سَأَلْتَ فَاسْأَلِ اللهَ، وَإِذَا اسْتَعَنْتَ فَاسْتَعِنْ بِاللهِ، وَاعْلَمْ أَنَّ الْأُمَّةَ لَوِ اجْتَمَعَتْ عَلَى أَنْ يَنْفَعُوكَ بِشَيْءٍ لَمْ يَنْفَعُوكَ إِلَّا بِشَيْءٍ قَدْ كَتَبَهُ اللهُ لَكَ، وَإِنِ اجْتَمَعُوا عَلَى أَنْ يَضُرُّوكَ بِشَيْءٍ لَمْ يَضُرُّوكَ إِلَّا بِشَيْءٍ قَدْ كَتَبَهُ اللهُ عَلَيْكَ، رُفِعَتِ الْأَقْلَامُ وَجَفَّتِ الصُّحُفُ. وَفِي رِوَايَةٍ غَيْرِ التِّرْمِذِيِّ: احْفَظِ اللهَ تَجِدْهُ أَمَامَكَ، تَعَرَّفْ إِلَى اللهِ فِي الرَّخَاءِ يَعْرِفْكَ فِي الشِّدَّةِ، وَاعْلَمْ أَنَّ مَا أَخْطَأَكَ لَمْ يَكُنْ لِيُصِيبَكَ، وَمَا أَصَابَكَ لَمْ يَكُنْ لِيُخْطِئَكَ، وَاعْلَمْ أَنَّ النَّصْرَ مَعَ الصَّبْرِ، وَأَنَّ الْفَرَجَ مَعَ الْكَرْبِ، وَأَنَّ مَعَ الْعُسْرِ يُسْرًا</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>مناقب عبد الله بن عباس رضي الله عنهما أكثر من أن تُحصر، وقد دعا له النبي صلى الله عليه وسلم فقال (اللهم فقّهه في الدين وعلّمه التأويل)، ودعا له بأن يؤتى الحكمة مرتين، وثبت عنه أنه رأى جبريل عليه السلام مرتين، وهو بحر هذه الأمة وحبرها.
 وقد رآه رسول الله صلى الله عليه وسلم أهلاً للوصية مع صغر سنه، فقال له (احفظ الله يحفظك) ومعناه: كن مطيعاً لربك، مؤتمراً بأوامره، منتهياً عن نواهيه، تجده حافظاً لك في مصالحك جميعها، كما جرى للثلاثة الذين آووا إلى غار فانطبقت صخرة عليهم، فقالوا: انظروا أعمالكم الصالحة فاسألوا الله تعالى بها ينجيكم، فذكر كل منهم سابقة له مع ربه، فانحدرت عنهم الصخرة فخرجوا يمشون، وقصتهم مشهورة في الصحيح.
 وقوله (إذا سألت فاسأل الله وإذا استعنت فاستعن بالله) أرشده إلى التوكل على مولاه، وأن لا يتخذ إلهاً سواه، ولا يتعلق بغيره في جميع أموره ما أمكن، فقال الله تعالى (ومن يتوكل على الله فهو حسبه)، بقدر ما يكرس الشخص إلى غير الله تعالى بطلبه أو قلبه أو أمله فقد أعرض عن ربه ولا ينفعه ولا يضره من غير الله، وكذلك الخوف من غير الله.
-وقد أكد النبي صلى الله عليه وسلم ذلك فقال (واعلم أن الأمة لو اجتمعت على أن ينفعوك بشيء لم ينفعوك إلا بشيء قد كتبه الله لك) وكذلك في الضر، وهذا هو الإيمان بالقدر والواجب الإيمان به خيره وشره.
+وقد أكد النبي صلى الله عليه وسلم ذلك فقال (واعلم أن الأمة لو اجتمعت على أن ينفعوك بشيء لم ينفعوك إلا بشيء قد كتبه الله لك) وكذلك في الضر، وهذا هو الإيمان بالقدر والواجب الإيمان به خيره وشره. وإذا تيقّن المؤمن بذلك فما فائدة سؤال غير الله والاستعانة به؟ ومن أروع الأمثلة على ذلك إجابة الخليل إبراهيم عليه الصلاة والسلام لجبريل عليه السلام حين سأله وهو في الهواء: ألك حاجة؟ فقال: أما إليك فلا. وقوله (رفعت الأقلام وجفت الصحف) تأكيد لما تقدّم، أي: لا يكون خلاف ما تقدّم لك بنسخ ولا تبديل.
 ثم قال: (واعلم أن النصر مع الصبر، وأن الفرج مع الكرب، وأن مع العسر يسرا) فنبّه على أن الإنسان في الدنيا -ولا سيما الصالحون- معرّضون للمصاب، لقوله عز وجل (ولنبلونّكم بشيء من الخوف والجوع ونقص من الأموال والأنفس والثمرات وبشّر الصابرين).</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>وصية نبوية لطفل صغير (ابن عباس) لكنها من أعمق وصايا الحياة: احفظ حدود الله وأوامره يحفظك الله في كل شؤونك. لا تتعلق بغير الله في طلبك أو استعانتك، فما كتبه الله لك سيصلك مهما حاول الناس منعه، وما لم يكتبه لك لن يصل إليك مهما اجتمع الناس على إعطائه لك. ثم يختم بثلاث حقائق مطمئنة: النصر يأتي مع الصبر لا بعده، والفرج يأتي مع الكرب لا بعد انتهائه، ومع العسر يسر يرافقه لا يتبعه فقط. هذا يعني أن الله معنا في قلب الأزمة، لا بعد أن تمر فقط.</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
-        <v>6</v>
+      <c r="H20" s="2" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="21" ht="90" customHeight="1">
@@ -1101,22 +1311,32 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
+          <t>أبو مسعود عقبة بن عمرو الأنصاري البدري رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي مَسْعُودٍ عُقْبَةَ بْنِ عَمْرٍو الْأَنْصَارِيِّ الْبَدْرِيِّ رَضِيَ اللهُ عَنْهُ قَالَ: قَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ:</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
           <t>إِنَّ مِمَّا أَدْرَكَ النَّاسُ مِنْ كَلَامِ النُّبُوَّةِ الْأُولَى: إِذَا لَمْ تَسْتَحِ فَاصْنَعْ مَا شِئْتَ</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>معنى قوله (من كلام النبوة الأولى) أن الحياء لم يزل ممدوحاً مستحسناً مأموراً به في شرائع الأنبياء الأولين لم يُنسخ.
-وقوله (فاصنع ما شئت) فيه وجهان: أحدهما أن يكون خرج بلفظ الأمر ولم يُرد به الأمر، بل معناه الوعيد والتهديد، كقوله تعالى (اعملوا ما شئتم) فإنه قد بيّن لهم ما يأتونه ويتركون فله جزاؤه من وعد أو وعيد. الوجه الثاني: أن معناه ما لم تستحِ منه إذا ظهر منه فاعله فافعله، فالمعصية الظاهرة التي يستحيا منها أمام الناس مذمومة أشد الذم.
+وقوله (فاصنع ما شئت) فيه وجهان: أحدهما أن يكون خرج بلفظ الأمر ولم يُرد به الأمر، بل معناه الوعيد والتهديد، كقوله تعالى (اعملوا ما شئتم) فإنه قد بيّن لهم ما يأتونه ويتركون فله جزاؤه من وعد أو وعيد، وكقوله صلى الله عليه وسلم (من باع الخمر فليشقص الخنازير) وليس في هذا إباحة لتشقيص الخنازير، بل هو على معنى التهديد. الوجه الثاني: أن معناه ما لم تستحِ منه إذا ظهر منه فاعله فافعله، فالمعصية الظاهرة التي يستحيا منها أمام الناس مذمومة أشد الذم.
 ونحو هذا قوله صلى الله عليه وسلم (الحياء من الإيمان) معناه: أنه لما كان يمنع صاحبه من الفواحش ويحمله على البر والخير، كما يمنع الإيمان صاحبه من ذلك ويحمله على الطاعات، صار الحياء بمنزلة الإيمان له، والله أعلم.</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>الحياء صفة أخلاقية باقية في كل الشرائع منذ الأنبياء الأولين، لم تُنسخ ولم تتغير. هذا الحديث يضع الحياء كرادع أخلاقي داخلي: من فقده أقدم على أي فعل مهما كان قبيحاً دون رادع يمنعه، لأن الحياء هو الذي يمنع الإنسان من الفواحش ويدفعه إلى البر والخير تماماً كما يفعل الإيمان. فالحياء ليس ضعفاً أو خجلاً سلبياً، بل هو حس داخلي يحفظ كرامة الإنسان وأخلاقه حتى حين لا يراقبه أحد.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1131,22 +1351,32 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
+          <t>أبو عمرو -وقيل أبو عمرة- سفيان بن عبد الله رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي عَمْرٍو - وَقِيلَ أَبِي عَمْرَةَ - سُفْيَانَ ابْنِ عَبْدِ اللهِ رَضِيَ اللهُ عَنْهُ قَالَ</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
           <t>قُلْتُ: يَا رَسُولَ اللهِ، قُلْ لِي فِي الْإِسْلَامِ قَوْلًا لَا أَسْأَلُ عَنْهُ أَحَدًا غَيْرَكَ، قَالَ: قُلْ آمَنْتُ بِاللهِ ثُمَّ اسْتَقِمْ</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>معنى قوله (قل لي في الإسلام قولاً لا أسأل عنه أحداً غيرك) أي علّمني قولاً جامعاً لمعاني الإسلام واضحاً في نفسه بحيث لا أحتاج إلى تفسير غيرك، أعمل به وأتقي به، فأجابه صلى الله عليه وسلم بقوله (قل آمنت بالله ثم استقم). هذا من جوامع الكلم التي أوتيها صلى الله عليه وسلم، فإنه جمع لهذا السائل جميع معاني الإسلام والإيمان في هاتين الكلمتين، فإنه أمره أن يجدد إيمانه بلسانه متذكراً بقلبه، وأن يستقيم على أعمال الطاعات والانتهاء عن جميع المخالفات، إذ لا تأتي الاستقامة مع شيء من الاعوجاج فإنها ضدّه.
 وهذا كقوله تعالى (إن الذين قالوا ربنا الله ثم استقاموا) الآية: أي آمنوا بالله وحده واستقاموا على ذلك وعلى الطاعة إلى أن توفاهم الله عليها. قال عمر بن الخطاب رضي الله عنه: استقاموا والله على طاعته ولم يروغوا روغان الثعلب. ومعناه: اعتدلوا على أكثر طاعة الله عقداً وقولاً وفعلاً، وكذلك قوله سبحانه (فاستقم كما أمرت).
-قال ابن عباس: ما نزلت على رسول الله صلى الله عليه وسلم آية في جميع القرآن كانت أشق عليه من هذه الآية، ولذلك قال صلى الله عليه وسلم (شيّبتني هود وأخواتها). قال الأستاذ أبو القاسم القشيري رحمه الله تعالى: الاستقامة درجة بها كمال الأمور وتمامها، وبوجودها حصول الخيرات ونظامها، ومن لم يكن مستقيماً في حاله ضاع سعيه وخاب جداً. وقيل: الاستقامة لا يطيقها إلا الأكابر، لأنها الخروج عن المعهودات، ومفارقة الرسوم والعادات، والقيام بين يدي الله تعالى على حقيقة الصدق، ولذلك قال النبي صلى الله عليه وسلم (استقيموا ولن تُحصوا). وقال الواسطي: الخصلة التي بها كملت المحاسن وبفقدها قبحت المحاسن هي الاستقامة، والله أعلم.</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
+قال ابن عباس: ما نزلت على رسول الله صلى الله عليه وسلم آية في جميع القرآن كانت أشق عليه من هذه الآية، ولذلك قال صلى الله عليه وسلم (شيّبتني هود وأخواتها). قال الأستاذ أبو القاسم القشيري رحمه الله تعالى: الاستقامة درجة بها كمال الأمور وتمامها، وبوجودها حصول الخيرات ونظامها، ومن لم يكن مستقيماً في حاله ضاع سعيه وخاب جدّه. وقيل: الاستقامة لا يطيقها إلا الأكابر، لأنها الخروج عن المعهودات، ومفارقة الرسوم والعادات، والقيام بين يدي الله تعالى على حقيقة الصدق، ولذلك قال النبي صلى الله عليه وسلم (استقيموا ولن تُحصوا). وقال الواسطي: الخصلة التي بها كملت المحاسن وبفقدها قبحت المحاسن هي الاستقامة، والله أعلم.</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>طلب رجل من النبي صلى الله عليه وسلم كلمة جامعة يكتفي بها ولا يحتاج معها سؤال أحد آخر، فأجابه بجملتين بسيطتين وعميقتين: آمنت بالله ثم استقم. الإيمان قول وقناعة، لكن الاستقامة هي الاختبار الحقيقي: أن تثبت على الطريق يومياً دون انحراف، في السر كما في العلن، في الرخاء كما في الشدة. وقد وصف ابن عباس أن آيات الاستقامة كانت من أثقل ما نزل على النبي صلى الله عليه وسلم، مما يدل أنها ليست أمراً هيناً، بل درجة عالية تحتاج مجاهدة مستمرة، وهي أساس نجاح الإنسان في كل جوانب حياته لا في الدين وحده.</t>
         </is>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="H22" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1161,23 +1391,33 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
+          <t>أبو عبد الله جابر بن عبد الله الأنصاري رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي عَبْدِ اللهِ جَابِرِ بْنِ عَبْدِ اللهِ الْأَنْصَارِيِّ رَضِيَ اللهُ عَنْهُمَا أَنَّ رَجُلًا سَأَلَ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ فَقَالَ</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
           <t>أَرَأَيْتَ إِذَا صَلَّيْتُ الْمَكْتُوبَاتِ، وَصُمْتُ رَمَضَانَ، وَأَحْلَلْتُ الْحَلَالَ، وَحَرَّمْتُ الْحَرَامَ، وَلَمْ أَزِدْ عَلَى ذَلِكَ شَيْئًا، أَأَدْخُلُ الْجَنَّةَ؟ قَالَ: نَعَمْ</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>قال الشيخ أبو عمرو بن الصلاح رحمه الله تعالى: الظاهر أنه أراد بقوله (وحرّمت الحرام وأحللت الحلال) أحد أمرين، أحدهما: أن يعتقد الحلال حلالاً والحرام حراماً، والثاني: أن لا يفعل الحرام فإنه يكفي فيه مجرد اعتقاده حراماً.
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>ومعنى (حرّمت الحرام): اجتنبته، ومعنى (أحللت الحلال): فعلته معتقداً حِلَّه. قال الشيخ أبو عمرو بن الصلاح رحمه الله تعالى: الظاهر أنه أراد بقوله (وحرّمت الحرام) أحد أمرين: أحدهما أن يعتقد كونه حراماً، والثاني أن لا يفعله؛ بخلاف (أحللت الحلال) فإنه يكفي فيه مجرد اعتقاده حلالاً.
 قال صاحب المهم: لم يذكر النبي صلى الله عليه وسلم في هذا الحديث شيئاً من التطوعات على الجملة، وهذا يدل على جواز ترك التطوعات على الجملة، لكن من تركها ولم يفعل شيئاً منها فقد فوّت على نفسه ربما ثواباً عظيماً وأجراً جسيماً، فإن كان ذلك رغبة عنها وتهاوناً بها كان ذلك نقصاً في دينه وقدحاً في عدالته، وربما كان فسقاً يستحق به ذماً.
 قال علماؤنا: لو أن أهل بلدة تواطؤوا على ترك سنة لقوتلوا عليها حتى يرجعوا، ولقد كان صدر الصحابة رضي الله عنهم ومن بعدهم يثابرون على فعل السنن والفضائل مثابرتهم على الفرائض، ولم يكونوا يفرقون بينهما في اغتنام ثوابها. وإنما احتاج إلى ذكر الفرق أئمة الفقهاء لما يترتب عليه من وجوب الإعادة وخوف العقاب على تركها ونفي ذلك إن حصل تركه بوجه ما.
 وإنما ترك النبي صلى الله عليه وسلم تنبيه هذا السائل على السنن والفضائل تسهيلاً وتيسيراً لقرب عهده بالإسلام، لئلا يكون الإكثار عليه مؤدياً لتنفيره عن ذلك، وعلم أنه إذا تمكّن إسلامه وشرح الله صدره رغب فيما فيه غيره من السنن والتطوعات. وقد جاء في الحديث الآخر أن رجلاً سأل النبي صلى الله عليه وسلم عن الصلاة فأخبره أنها خمس، فقال: هل عليّ غيرها؟ قال: لا، إلا أن تطّوّع، ثم سأله عن الصوم والزكاة والحج فأجابه، ثم قال في آخر ذلك: والله لا أزيد على هذا ولا أنقص منه، فقال صلى الله عليه وسلم: أفلح إن صدق -وفي رواية: إن تمسك بما أُمر به دخل الجنة- وهذا يبيّن أن من حافظ على فرائضه وأقامها في أوقاتها من غير إخلال بها كان فلاحه ونجاحه محققاً، ومن أتى بالفرائض وأتبعها بالنوافل كان أكثر فلاحاً ونجاحاً.</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>سأل صحابي النبي صلى الله عليه وسلم: هل يكفيني أن أصلي الفرائض، وأصوم رمضان، وألتزم بالحلال، وأجتنب الحرام، دون أن أزيد شيئاً، لأدخل الجنة؟ فأجابه النبي صلى الله عليه وسلم بنعم. هذا الحديث يريح كل من يشعر بالتقصير في النوافل والمستحبات، فالأساسيات وحدها كافية لدخول الجنة إن أُديت بصدق والتزام، والزيادة عليها بالنوافل والسنن تزيد الفلاح والقرب من الله لكنها ليست شرطاً لأصل النجاة. الدين إذن ليس منافسة في الكمال، بل التزام صادق بالحد الأدنى الواجب، مع الترحيب بكل زيادة خير دون ضغط أو شعور بالذنب لمن اكتفى بالفرائض.</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="H23" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1192,25 +1432,35 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
+          <t>أبو مالك الحارث بن عاصم الأشعري رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي مَالِكٍ الْحَارِثِ بْنِ عَاصِمٍ الْأَشْعَرِيِّ رَضِيَ اللهُ عَنْهُ قَالَ: قَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
           <t>الطُّهُورُ شَطْرُ الْإِيمَانِ، وَالْحَمْدُ لِلَّهِ تَمْلَأُ الْمِيزَانَ، وَسُبْحَانَ اللهِ وَالْحَمْدُ لِلَّهِ تَمْلَآنِ -أَوْ تَمْلَأُ- مَا بَيْنَ السَّمَاءِ وَالْأَرْضِ، وَالصَّلَاةُ نُورٌ، وَالصَّدَقَةُ بُرْهَانٌ، وَالصَّبْرُ ضِيَاءٌ، وَالْقُرْآنُ حُجَّةٌ لَكَ أَوْ عَلَيْكَ، كُلُّ النَّاسِ يَغْدُو: فَبَائِعٌ نَفْسَهُ فَمُعْتِقُهَا أَوْ مُوبِقُهَا</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>هذا حديث أصل من أصول الإسلام، وقد اشتمل على مهمات من قواعد الإسلام والدين. أما (الطهور) فالمراد به هنا الفعل، واختلف في معناه: فقيل إن الأجر فيه ينتهي إلى نصف أجر الإيمان، وقيل: المراد بالإيمان هنا الصلاة، والطهارة شرط في صحتها، فصارت كالشطر منها.
 وأما قوله (والحمد لله تملأ الميزان) فمعناه أنها أعظم أجراً لعظم ميزان الحامد لله تعالى، وقد تظاهرت نصوص القرآن والسنة على ثقل الموازين بوزن الأعمال، وكذلك قوله (سبحان الله والحمد لله تملآن ما بين السماء والأرض) وسبب علو منزلتهما ما اشتملتا عليه من التنزيه لله تعالى والافتقار إليه.
-وأما قوله صلى الله عليه وسلم (والصلاة نور) فمعناه أنها تمنع من المعاصي وتنهى عن الفحشاء والمنكر، وتهدي إلى الصواب كما يُستضاء بالنور، وقيل: إنها تكون نوراً ظاهراً على وجه صاحبها في الدنيا والآخرة بخلاف من لم يصلِّ.
-وأما قوله صلى الله عليه وسلم (والصدقة برهان) فمعناه أنها حجة على صدق إيمان صاحبها، لأن المنافق يمتنع منها لكونه لا يعتقدها، فمن تصدق استدل بصدقته على قوة إيمانه.
-وأما قوله صلى الله عليه وسلم (والصبر ضياء) فمعناه: الصبر المحبوب في الشرع، وهو الصبر على طاعة الله والصبر عن معصيته، والصبر أيضاً على النوائب وأنواع المكاره في الدنيا، والمراد أن الصبر محمود لا يزال صاحبه مستضيئاً به مهتدياً مستمراً على الصواب.
-وأما قوله صلى الله عليه وسلم (والقرآن حجة لك أو عليك) فمعناه ظاهر: أي إن انتفعت به إذ تلوته وعملت به فهو حجة لك، وإلا فهو حجة عليك. وقوله (كل الناس يغدو فبائع نفسه فمعتقها أو موبقها) معناه: أن كل إنسان يسعى لنفسه، فمنهم من يبيعها بطاعته فيعتقها من العذاب، ومنهم من يبيعها للشيطان والهوى فيوبقها أي يهلكها.</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
+وأما قوله صلى الله عليه وسلم (والصلاة نور) فمعناه أنها تمنع من المعاصي وتنهى عن الفحشاء والمنكر، وتهدي إلى الصواب كما يُستضاء بالنور، وقيل: معناه أن يكون آخرها نوراً لصاحبها يوم القيامة، وقيل: إنها تكون نوراً ظاهراً على وجه صاحبها في الدنيا والآخرة بخلاف من لم يصلِّ.
+وأما قوله صلى الله عليه وسلم (والصدقة برهان) فقال صاحب التجريد: معناه أنه يفزع إليها للبرهان، كما يفزع العبد إذا سُئل يوم القيامة عن مصرف ماله فكانت له صدقاته برهاناً في جواب هذا السؤال فيقول: تصدقت به. وقال غيره: معناه أنها حجة على صدق إيمان صاحبها، لأن المنافق يمتنع منها لكونه لا يعتقدها، فمن تصدق استدل بصدقته على قوة إيمانه.
+وأما قوله صلى الله عليه وسلم (والصبر ضياء) فمعناه: الصبر المحبوب في الشرع، وهو الصبر على طاعة الله والصبر عن معصيته، والصبر أيضاً على النوائب وأنواع المكاره في الدنيا، والمراد أن الصبر محمود لا يزال صاحبه مستضيئاً به مهتدياً مستمراً على الصواب. وقد اختلف العلماء في حقيقة الصبر: فقال إبراهيم الخوّاص: الصبر هو الثبات على الكتاب والسنة، وقيل: هو الوقوف مع البلاء بحسن الأدب، وقال أبو الدقّاق رحمه الله: الصبر أن لا يعترض العبد على المقدور، فأما إظهار البلاء ووجه الشكوى فلا ينافي الصبر، كما قال الله تعالى في حق أيوب عليه السلام (إنا وجدناه صابراً نعم العبد إنه أواب) مع أنه قال (أني مسّني الضرّ وأنت أرحم الراحمين).
+وأما قوله صلى الله عليه وسلم (والقرآن حجة لك أو عليك) فمعناه ظاهر: أي إن انتفعت به إذ تلوته وعملت به فهو حجة لك، وإلا فهو حجة عليك. وقوله (كل الناس يغدو فبائع نفسه فمعتقها أو موبقها) معناه: أن كل إنسان يسعى لنفسه، فمنهم من يبيعها بطاعته فيعتقها من العذاب كما قال الله تعالى (إن الله اشترى من المؤمنين أنفسهم وأموالهم بأن لهم الجنة)، ومنهم من يبيعها للشيطان والهوى فيوبقها أي يهلكها.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>هذا الحديث يرسم خريطة مكثفة لعبادات يومية بسيطة وقيمتها الحقيقية: الطهارة نصف الإيمان، والحمد لله يملأ ميزان الأعمال، والتسبيح والتحميد يملآن ما بين السماء والأرض، والصلاة نور يهدي في الظلام، والصدقة دليل صدق إيمانك، والصبر ضياء يرشدك للصواب في أصعب اللحظات، والقرآن إما شاهد لك أو شاهد عليك بحسب تعاملك معه. ثم يختم بصورة معبرة: كل إنسان يخرج كل يوم يبيع نفسه، إما لطاعة الله فيحررها من العذاب، وإما لهواه فيهلكها. فحياتنا اليومية سلسلة قرارات صغيرة تحدد مصير هذه الصفقة.</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="H24" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1225,10 +1475,20 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
+          <t>أبو ذر الغفاري رضي الله عنه، عن النبي صلى الله عليه وسلم فيما يرويه عن ربه عز وجل (حديث قدسي)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي ذَرٍّ الْغِفَارِيِّ رَضِيَ اللهُ تَعَالَى عَنْهُ عَنِ النَّبِيِّ صَلَّى اللهُ تَعَالَى عَلَيْهِ وَآلِهِ وَسَلَّمَ فِيمَا يَرْوِيهِ عَنْ رَبِّهِ عَزَّ وَجَلَّ قَالَ</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
           <t>يَا عِبَادِي، إِنِّي حَرَّمْتُ الظُّلْمَ عَلَى نَفْسِي وَجَعَلْتُهُ بَيْنَكُمْ مُحَرَّمًا فَلَا تَظَالَمُوا، يَا عِبَادِي، كُلُّكُمْ ضَالٌّ إِلَّا مَنْ هَدَيْتُهُ فَاسْتَهْدُونِي أَهْدِكُمْ، يَا عِبَادِي، كُلُّكُمْ جَائِعٌ إِلَّا مَنْ أَطْعَمْتُهُ فَاسْتَطْعِمُونِي أُطْعِمْكُمْ، يَا عِبَادِي، كُلُّكُمْ عَارٍ إِلَّا مَنْ كَسَوْتُهُ فَاسْتَكْسُونِي أَكْسُكُمْ، يَا عِبَادِي، إِنَّكُمْ تُخْطِئُونَ بِاللَّيْلِ وَالنَّهَارِ وَأَنَا أَغْفِرُ الذُّنُوبَ جَمِيعًا فَاسْتَغْفِرُونِي أَغْفِرْ لَكُمْ، يَا عِبَادِي، إِنَّكُمْ لَنْ تَبْلُغُوا ضُرِّي فَتَضُرُّونِي، وَلَنْ تَبْلُغُوا نَفْعِي فَتَنْفَعُونِي، يَا عِبَادِي، لَوْ أَنَّ أَوَّلَكُمْ وَآخِرَكُمْ وَإِنْسَكُمْ وَجِنَّكُمْ كَانُوا عَلَى أَتْقَى قَلْبِ رَجُلٍ وَاحِدٍ مِنْكُمْ مَا زَادَ ذَلِكَ فِي مُلْكِي شَيْئًا، يَا عِبَادِي، لَوْ أَنَّ أَوَّلَكُمْ وَآخِرَكُمْ وَإِنْسَكُمْ وَجِنَّكُمْ كَانُوا عَلَى أَفْجَرِ قَلْبِ رَجُلٍ وَاحِدٍ مِنْكُمْ مَا نَقَصَ ذَلِكَ مِنْ مُلْكِي شَيْئًا، يَا عِبَادِي، لَوْ أَنَّ أَوَّلَكُمْ وَآخِرَكُمْ وَإِنْسَكُمْ وَجِنَّكُمْ قَامُوا فِي صَعِيدٍ وَاحِدٍ فَسَأَلُونِي فَأَعْطَيْتُ كُلَّ وَاحِدٍ مَسْأَلَتَهُ، مَا نَقَصَ ذَلِكَ مِمَّا عِنْدِي إِلَّا كَمَا يَنْقُصُ الْمِخْيَطُ إِذَا أُدْخِلَ الْبَحْرَ، يَا عِبَادِي، إِنَّمَا هِيَ أَعْمَالُكُمْ أُحْصِيهَا لَكُمْ ثُمَّ أُوَفِّيكُمْ إِيَّاهَا، فَمَنْ وَجَدَ خَيْرًا فَلْيَحْمَدِ اللهَ، وَمَنْ وَجَدَ غَيْرَ ذَلِكَ فَلَا يَلُومَنَّ إِلَّا نَفْسَهُ</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>قوله (إني حرّمت الظلم على نفسي وجعلته بينكم محرماً) معناه: وما ينبغي لي ولا يجوز عليّ، فالظلم محال في حق الله تعالى سبحانه، إذ لا يُتصور أن يظلم أحداً وهو مالك كل شيء ولا يسأل عما يفعل. وقوله (فلا تظالموا) أصله: فلا تتظالموا، حُذفت إحدى التاءين تخفيفاً.
 وقوله (كلكم ضالّ إلا من هديته) تنبيه على أن العبد عاجز عن جلب المنافع لنفسه ودفع المضار عنها إلا أن يعينه الله سبحانه على ذلك، وهو يرجع إلى معنى (لا حول ولا قوة إلا بالله)، وليعلم العبد أنه إذا رأى آثار هذه النعمة عليه أن ذلك من عند الله، فيزداد بذلك حمداً وشكراً لله تعالى. وقوله (فاستهدوني أهدكم) أي اطلبوا هدايتي أهدكم. وكذلك (كلكم جائع إلا من أطعمته) يعني أنه خالق الخلق كلهم ذوي فقر إلى الطعام، فكل طاعم حتى يُطعمه يسوق الله الرزق إليه، فلا يظنن ذو الثروة أن الرزق الذي بين يديه من غير الله تعالى.
@@ -1238,12 +1498,12 @@
 وقوله (إنما هي أعمالكم أحصيها لكم ثم أوفيكم إياها، فمن وجد خيراً فليحمد الله ومن وجد غير ذلك فلا يلومن إلا نفسه) يعني أن الإنسان لا يسند نجاته إلى عمله وعبادته وحدها، بل إلى التوفيق والفضل من الله عز وجل، وإن وجد غير الخير فلا يلومن إلا نفسه لأنه هو المقصر.</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>حديث قدسي عظيم يكشف صورة الله الرحيم الغني عن خلقه تماماً: حرّم الظلم على نفسه أولاً قبل أن يحرّمه بيننا، ويدعونا أن نطلب منه كل ما نحتاجه: الهداية، والطعام، والكسوة، والمغفرة، لأنه وحده القادر على العطاء دون أن ينقص ذلك من ملكه شيئاً، حتى لو سأله كل الخلق في لحظة واحدة وأعطاهم جميعاً. ويؤكد أن طاعتنا لا تنفعه وأن معصيتنا لا تضره، فكل ما يطلبه منا هو لمصلحتنا نحن. ويختم بحقيقة عادلة: أعمالنا محفوظة بدقة، فمن وجد خيراً فليحمد الله، ومن وجد غير ذلك فلا يلوم إلا نفسه.</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="H25" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1258,21 +1518,32 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
+          <t>أبو ذر الغفاري رضي الله عنه (عن نفر من أصحاب رسول الله صلى الله عليه وسلم)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي ذَرٍّ رَضِيَ اللهُ عَنْهُ أَيْضًا أَنَّ نَاسًا مِنْ أَصْحَابِ رَسُولِ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالُوا لِلنَّبِيِّ صَلَّى اللهُ تَعَالَى عَلَيْهِ وَآلِهِ وَسَلَّمَ</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
           <t>يَا رَسُولَ اللهِ، ذَهَبَ أَهْلُ الدُّثُورِ بِالْأُجُورِ: يُصَلُّونَ كَمَا نُصَلِّي، وَيَصُومُونَ كَمَا نَصُومُ، وَيَتَصَدَّقُونَ بِفُضُولِ أَمْوَالِهِمْ، قَالَ: أَوَ لَيْسَ قَدْ جَعَلَ اللهُ لَكُمْ مَا تَصَدَّقُونَ؟ إِنَّ بِكُلِّ تَسْبِيحَةٍ صَدَقَةً، وَكُلِّ تَكْبِيرَةٍ صَدَقَةً، وَكُلِّ تَحْمِيدَةٍ صَدَقَةً، وَكُلِّ تَهْلِيلَةٍ صَدَقَةً، وَأَمْرٌ بِمَعْرُوفٍ صَدَقَةٌ، وَنَهْيٌ عَنْ مُنْكَرٍ صَدَقَةٌ، وَفِي بُضْعِ أَحَدِكُمْ صَدَقَةٌ. قَالُوا: يَا رَسُولَ اللهِ، أَيَأْتِي أَحَدُنَا شَهْوَتَهُ وَيَكُونُ لَهُ فِيهَا أَجْرٌ؟ قَالَ: أَرَأَيْتُمْ لَوْ وَضَعَهَا فِي حَرَامٍ أَكَانَ عَلَيْهِ وِزْرٌ؟ فَكَذَلِكَ إِذَا وَضَعَهَا فِي الْحَلَالِ كَانَ لَهُ أَجْرٌ</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>شكا بعض الصحابة الفقراء للنبي صلى الله عليه وسلم أن أهل الأموال (الدثور) يسبقونهم بالأجر لأنهم يصلون ويصومون مثلهم، ثم يتصدقون بفضول أموالهم زيادة، فبيّن لهم النبي صلى الله عليه وسلم أن الله فتح لهم أبواباً أخرى للأجر لا تحتاج مالاً: فكل تسبيحة وتكبيرة وتحميدة وتهليلة صدقة، والأمر بالمعروف والنهي عن المنكر صدقة، بل وفي العلاقة الزوجية الحلال صدقة يُثاب عليها الإنسان.
+ونبّه العلماء إلى أن ذكر (الأمر بالمعروف والنهي عن المنكر) هنا آكد وأعظم مما قبله من التسبيح والتكبير والتحميد والتهليل، لأن الأمر بالمعروف والنهي عن المنكر فرض كفاية وقد يتعيّن أحياناً، بخلاف هذه الأذكار فإنها نوافل، وأجر الفرائض أعظم من أجر النوافل، كما جاء في الحديث القدسي (وما تقرّب إليّ عبدي بشيء أحبّ إليّ مما افترضته عليه)، بل قال بعض العلماء: يزيد ثواب الفرض على ثواب النفل سبعين درجة. وفي هذا تذكير بأن مراتب الأعمال عند الله متفاوتة، وأن الفرائض مقدَّمة في الفضل على النوافل وإن كانت النوافل كلها مأجورة.
 فلما استغربوا أن يكون في قضاء الشهوة أجر، أوضح لهم النبي صلى الله عليه وسلم القياس بأبسط صورة: أرأيتم لو وضعها في حرام أكان عليه وزر؟ قالوا: نعم. قال: فكذلك إذا وضعها في الحلال كان له أجر. ومعنى ذلك أن الفعل الواحد يتحدد حكمه بموضعه ووجهته، فما كان مذموماً في الحرام يكون مأجوراً في الحلال، وهذا يبيّن أن الشريعة لا تحصر الأجر في العبادات المحضة فقط، بل توسّع دائرة العبادة لتشمل كل تصرف مباح يُقصد به وجه الله أو يُؤدى في حدوده المشروعة.</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>اشتكى بعض الصحابة الفقراء أن الأغنياء يسبقونهم بالأجر بسبب صدقاتهم الزائدة، فطمأنهم النبي صلى الله عليه وسلم بأن أبواب الأجر مفتوحة للجميع بلا حاجة إلى مال: كل تسبيحة وتكبيرة وتحميدة وتهليلة صدقة، والأمر بالمعروف والنهي عن المنكر صدقة، وحتى العلاقة الزوجية الحلال فيها أجر. هذا الحديث يوسّع مفهوم العبادة والصدقة ليشمل كل تفاصيل حياتنا اليومية، ويطمئن كل من يشعر أنه محروم من فرص الخير بسبب ضيق ذات يده، فالأجر الحقيقي في النية والفعل الطيب لا في حجم المال.</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="H26" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1287,22 +1558,31 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ: قَالَ رَسُولُ اللَّهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
           <t>كُلُّ سُلَامَى مِنَ النَّاسِ عَلَيْهِ صَدَقَةٌ، كُلَّ يَوْمٍ تَطْلُعُ فِيهِ الشَّمْسُ: تَعْدِلُ بَيْنَ اثْنَيْنِ صَدَقَةٌ، وَتُعِينُ الرَّجُلَ فِي دَابَّتِهِ فَتَحْمِلُهُ عَلَيْهَا أَوْ تَرْفَعُ لَهُ عَلَيْهَا مَتَاعَهُ صَدَقَةٌ، وَالْكَلِمَةُ الطَّيِّبَةُ صَدَقَةٌ، وَبِكُلِّ خُطْوَةٍ تَمْشِيهَا إِلَى الصَّلَاةِ صَدَقَةٌ، وَتُمِيطُ الْأَذَى عَنِ الطَّرِيقِ صَدَقَةٌ</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>قوله (سُلامى) بضم السين المهملة وتخفيف اللام: وهي المفاصل والأعضاء، وقد ثبت في صحيح مسلم أنها ثلاثمائة وستون مفصلاً. قال القاضي عياض: أصله عظام الكف والأصابع والرجل، ثم استُعمل في سائر عظام الجسد ومفاصله. قال بعض العلماء: المراد صدقة ترهيب وترغيب لا إيجاب وإلزام.
-وقوله (تعدل بين اثنين صدقة) أي تصلح بينهما بالعدل. وفي رواية أخرى لمسلم (يصبح على كل سلامى من أحدكم صدقة، فكل تسبيحة صدقة، وكل تحميدة صدقة، وكل تهليلة صدقة، وكل تكبيرة صدقة، وأمر بالمعروف صدقة، ونهي عن المنكر صدقة، ويجزئ من ذلك ركعتان يركعهما من الضحى) أي يكفي من هذه الصدقات عن جميع الأعضاء ركعتان، فإن الصلاة عمل لجميع أعضاء الجسد، فإذا صلى فقد صلى كل عضو بوظيفته.
-وفي هذا الحديث فضيلة التسبيح وسائر الأذكار، والأمر بالمعروف والنهي عن المنكر، وإحضار النية في المباحات، وإنما تصير الطاعات والصدقات صادقة بالنيات الصادقة، وفيه دليل على جواز سؤال المستفتي عمن يخفى عليه بعض ما لا يعلمه من الدليل، إذا علم من حال المسؤول أنه لا يكرهه ولم يكن فيه سوء أدب.</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
+وقوله (تعدل بين اثنين صدقة) أي تصلح بينهما بالعدل. وفي رواية أخرى لمسلم (يصبح على كل سلامى من أحدكم صدقة، فكل تسبيحة صدقة، وكل تحميدة صدقة، وكل تهليلة صدقة، وكل تكبيرة صدقة، وأمر بالمعروف صدقة، ونهي عن المنكر صدقة، ويجزئ من ذلك ركعتان يركعهما من الضحى) أي يكفي من هذه الصدقات عن جميع الأعضاء ركعتان، فإن الصلاة عمل لجميع أعضاء الجسد، فإذا صلى فقد صلى كل عضو بوظيفته، والله أعلم.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>كل مفصل من مفاصل جسمك (وهي ثلاثمائة وستون مفصلاً) عليه صدقة واجبة كل يوم تطلع فيه الشمس، لكنها صدقات ميسّرة في متناول الجميع: أن تعدل بين اثنين متخاصمين، أن تساعد شخصاً على حمل متاعه أو ركوب دابته، أن تقول كلمة طيبة، أن تمشي خطوة نحو الصلاة، أن تزيل أذى عن الطريق. هذا الحديث يفتح أعيننا على أن حياتنا اليومية مليئة بفرص الخير الصغيرة التي لا تحتاج مالاً ولا مجهوداً كبيراً، وأن الإحسان يمكن أن يكون نمط حياة لا مناسبة عابرة.</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="H27" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1317,23 +1597,33 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>الْبِرُّ حُسْنُ الْخُلُقِ، وَالْإِثْمُ مَا حَاكَ فِي نَفْسِكَ وَكَرِهْتَ أَنْ يَطَّلِعَ عَلَيْهِ النَّاسُ. وَعَنْ وَابِصَةَ بْنِ مَعْبَدٍ رَضِيَ اللهُ عَنْهُ قَالَ: أَتَيْتُ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ فَقَالَ: جِئْتَ تَسْأَلُ عَنِ الْبِرِّ؟ قُلْتُ: نَعَمْ، قَالَ: اسْتَفْتِ قَلْبَكَ، الْبِرُّ مَا اطْمَأَنَّتْ إِلَيْهِ النَّفْسُ وَاطْمَأَنَّ إِلَيْهِ الْقَلْبُ، وَالْإِثْمُ مَا حَاكَ فِي النَّفْسِ وَتَرَدَّدَ فِي الصَّدْرِ، وَإِنْ أَفْتَاكَ النَّاسُ وَأَفْتَوْكَ</t>
+          <t>النواس بن سمعان رضي الله عنه، ووابصة بن معبد رضي الله عنه</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>قوله (البر حسن الخلق) يعني: أن حسن الخلق أعظم خصال البر، كما قال (الحج عرفة). والمراد بحسن الخلق: الإنصاف في المعاملة، والرفق في المحاولة، والعدل في الأحكام، والبذل في الإحسان، وغير ذلك من صفات المؤمنين الذين وصفهم الله تعالى في سورة الأنفال وسورة الفرقان. فمن أشكل عليه حاله فليعرض نفسه على هذه الآيات، فوجود جميعها علامة حسن الخلق كله، ووجود بعضها دون بعض يدل بعضها على البعض. ولا يظنن أن حسن الخلق عبارة عن لين الجانب فقط وترك الفواحش والمعاصي، بل هو أشمل من ذلك، ومن حسن الخلق احتمال الأذى.
-وقد ورد في الصحيحين: أن أعرابياً جذب برد النبي صلى الله عليه وسلم حتى أثرت حاشيته في عاتقه الشريف، وقال بجفاء: مُر لي من مال الله الذي عندك، فالتفت إليه رسول الله صلى الله عليه وسلم وضحك ثم أمر له بعطاء، وهذا مثال حي لحسن الخلق عند الاستفزاز.
-وقوله (والإثم ما حاك في نفسك وكرهت أن يطّلع عليه الناس) يعني: هو الشيء الذي يورث نفرة في القلب، وهذا أصل يُتمسك به في معرفة الإثم من البر.
+          <t>عَنِ النَّوَّاسِ بْنِ سَمْعَانَ رَضِيَ اللهُ تَعَالَى عَنْهُ عَنِ النَّبِيِّ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>الْبِرُّ حُسْنُ الْخُلُقِ، وَالْإِثْمُ مَا حَاكَ فِي نَفْسِكَ وَكَرِهْتَ أَنْ يَطَّلِعَ عَلَيْهِ النَّاسُ. وَعَنْ وَابِصَةَ بْنِ مَعْبَدٍ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ: أَتَيْتُ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ فَقَالَ: جِئْتَ تَسْأَلُ عَنِ الْبِرِّ؟ قُلْتُ: نَعَمْ، قَالَ: اسْتَفْتِ قَلْبَكَ، الْبِرُّ مَا اطْمَأَنَّتْ إِلَيْهِ النَّفْسُ وَاطْمَأَنَّ إِلَيْهِ الْقَلْبُ، وَالْإِثْمُ مَا حَاكَ فِي النَّفْسِ وَتَرَدَّدَ فِي الصَّدْرِ، وَإِنْ أَفْتَاكَ النَّاسُ وَأَفْتَوْكَ</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>قوله (البر حسن الخلق) يعني: أن حسن الخلق أعظم خصال البر، كما قال (الحج عرفة). والمراد بحسن الخلق: الإنصاف في المعاملة، والرفق في المحاولة، والعدل في الأحكام، والبذل في الإحسان، وغير ذلك من صفات المؤمنين الذين وصفهم الله تعالى فقال في سورة الأنفال: (إنما المؤمنون الذين إذا ذُكر الله وجلت قلوبهم وإذا تُليت عليهم آياته زادتهم إيماناً وعلى ربهم يتوكلون، الذين يقيمون الصلاة ومما رزقناهم ينفقون، أولئك هم المؤمنون حقاً)، وقال تعالى: (التائبون العابدون الحامدون) إلى قوله (وبشر المؤمنين)، وقال: (قد أفلح المؤمنون) إلى قوله (أولئك هم الوارثون)، وقال: (وعباد الرحمن الذين يمشون على الأرض هوناً) إلى آخر السورة. فمن أشكل عليه حاله فليعرض نفسه على هذه الآيات، فوجود جميعها علامة حسن الخلق كله، وفقدها جميعاً علامة سوء الخلق، ووجود بعضها دون بعض يدل بعضها على البعض، فليشغل بحفظ ما وجده وتحصيل ما فقده. ولا يظنن ظانّ أن حسن الخلق عبارة عن لين الجانب فقط وترك الفواحش والمعاصي، بل هو أعم من ذلك وأشمل، ومن فعل ذلك فقد هذّب خلقه، بل حسن الخلق ما ذكرناه من صفات المؤمنين والتخلق بأخلاقهم، ومن حسن الخلق احتمال الأذى.
+وقد ورد في الصحيحين: أن أعرابياً جذب برد النبي صلى الله عليه وسلم حتى أثرت حاشيته في عاتقه الشريف، وقال: يا محمد، مُر لي من مال الله الذي عندك، فالتفت إليه رسول الله صلى الله عليه وسلم وضحك ثم أمر له بعطاء، وهذا مثال حي لحسن الخلق عند الاستفزاز.
+وقوله (والإثم ما حاك في نفسك وكرهت أن يطّلع عليه الناس) يعني: هو الشيء الذي يورث نفرة في القلب، وهذا أصل يُتمسك به لمعرفة الإثم من البر: إن الإثم ما يحوك في الصدر ويكره صاحبه أن يطّلع عليه الناس، والمراد بالناس -والله أعلم- أماثلهم ووجوههم لا أغوغاؤهم، فهذا هو الإثم فيتركه، والله أعلم.
 وأما حديث وابصة بن معبد، فقد جاءه يسأل عن البر، فأرشده النبي صلى الله عليه وسلم أن يستفتي قلبه: البر ما اطمأنت إليه النفس واطمأن إليه القلب، والإثم ما حاك في النفس وتردد في الصدر، وإن أفتاه الناس بجوازه.</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>البر كله يتلخص في كلمة واحدة جامعة: حسن الخلق -أي الإنصاف والرفق والعدل والبذل في التعامل مع الناس. أما الإثم فهو ما يترك في نفسك إحساساً بعدم الراحة، وتكره أن يطّلع عليه الناس حتى لو أفتاك كثيرون بجوازه. هذا الحديث يعطينا معياراً داخلياً بسيطاً: استفتِ قلبك، فالنفس المطمئنة والقلب الساكن علامة على الصواب، والتردد والقلق الداخلي علامة على أن هناك ما ينبغي إعادة النظر فيه، بصرف النظر عمن يوافقك أو يخالفك من الناس.</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1348,24 +1638,34 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
+          <t>أبو نجيح العرباض بن سارية رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي نَجِيحٍ الْعِرْبَاضِ بْنِ سَارِيَةَ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
           <t>وَعَظَنَا رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ مَوْعِظَةً وَجِلَتْ مِنْهَا الْقُلُوبُ وَذَرَفَتْ مِنْهَا الْعُيُونُ، فَقُلْنَا: يَا رَسُولَ اللهِ كَأَنَّهَا مَوْعِظَةُ مُوَدِّعٍ فَأَوْصِنَا، قَالَ: أُوصِيكُمْ بِتَقْوَى اللهِ عَزَّ وَجَلَّ وَالسَّمْعِ وَالطَّاعَةِ وَإِنْ تَأَمَّرَ عَلَيْكُمْ عَبْدٌ، فَإِنَّهُ مَنْ يَعِشْ مِنْكُمْ فَسَيَرَى اخْتِلَافًا كَثِيرًا، فَعَلَيْكُمْ بِسُنَّتِي وَسُنَّةِ الْخُلَفَاءِ الرَّاشِدِينَ الْمَهْدِيِّينَ عَضُّوا عَلَيْهَا بِالنَّوَاجِذِ، وَإِيَّاكُمْ وَمُحْدَثَاتِ الْأُمُورِ فَإِنَّ كُلَّ بِدْعَةٍ ضَلَالَةٌ</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>في بعض طرق هذا الحديث: إن هذه موعظة مودّع، فماذا تعهد إلينا؟ قال: (لقد تركتكم على البيضاء ليلها كنهارها لا يزيغ عنها إلا هالك). قوله: موعظة بليغة، يعني بلغت إلينا وأثرت في قلوبنا، ووجلت منها القلوب: أي خافت، وذرفت منها العيون: كأنه قام مقام تخويف ووعيد.
 وقوله (أوصيكم بتقوى الله والسمع والطاعة) يعني لولاة الأمور. وفي بعض الروايات (وإن تأمر عليكم عبد) قال بعض العلماء: العبد لا يكون والياً، ولكن ضُرب به المثل على التقدير وإن لم يكن، ويحتمل أن النبي صلى الله عليه وسلم أخبر بفساد الأمر ووضعه في غير أهله، فإذا كانت الولاية كذلك فاسمعوا وأطيعوا تغليباً لأهون الضررين، وهو الصبر على عدم الخروج على الولاية لئلا يفضي ذلك إلى فتنة عظيمة.
-وقوله (فإنه من يعش منكم فسيرى اختلافاً كثيراً) من هذا معجزاته صلى الله عليه وسلم: أخبر أصحابه بما يكون بعده من الاختلاف وغلبة المنكر، وقد كان عالماً به لكل أحد، إنما حذّر منه بعض الآحاد كحذيفة وأبي هريرة، وهو دليل على عظم منزلتهما.
+وقوله (فإنه من يعش منكم فسيرى اختلافاً كثيراً) من هذا بعض معجزاته صلى الله عليه وسلم: أخبر أصحابه بما يكون بعده من الاختلاف وغلبة المنكر على التفصيل، ولم يكن بيّنه لكل أحد، إنما حذّر منه بعض الآحاد كحذيفة وأبي هريرة، وهو دليل على عظم محلهما ومنزلتهما.
 وقوله (فعليكم بسنتي وسنة الخلفاء الراشدين المهديين) يعني الذين شملهم الهدى بالإجماع، وهم الأربعة: أبو بكر وعمر وعثمان وعلي رضي الله عنهم أجمعين. وأمر صلى الله عليه وسلم بالثبات على سنة الخلفاء الراشدين لأمرين: أحدهما التقليد لمن عجز عن النظر، والثاني الترجيح لما ذهبوا إليه عند اختلاف الصحابة.
 وقوله (وإياكم ومحدثات الأمور) اعلم أن المحدث ينقسم قسمين: محدث ليس له أصل في الشريعة، فهذا باطل مذموم، ومحدث له أصل يُحمل عليه، فلفظ (المحدث) و(البدعة) لا يذمّان لمجرد الاسم، بل لمعنى المخالفة للسنة والداعي إلى الضلالة، وقال عمر رضي الله عنه في التراويح: نعمت البدعة هذه، والله أعلم.</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>موعظة أخيرة مؤثرة من النبي صلى الله عليه وسلم بكت لها القلوب والعيون، كأنها وداع، فطلب الصحابة وصية جامعة. أوصاهم بأربعة أمور: تقوى الله في كل حال، طاعة ولاة الأمر بالمعروف حفاظاً على استقرار المجتمع، التمسك الشديد بسنته وسنة الخلفاء الراشدين خاصة عند كثرة الاختلاف الذي أخبر أنه سيحدث بعده، والحذر من كل بدعة محدثة في الدين لا أصل لها. هذا الحديث بوصلة ثابتة وقت الفتن والاختلافات: ارجع دائماً إلى الأصل الثابت (الكتاب والسنة وفهم السلف الصالح) بدل الانجراف مع كل رأي جديد.</t>
         </is>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="H29" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1380,24 +1680,34 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
+          <t>معاذ بن جبل رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ مُعَاذِ بْنِ جَبَلٍ رَضِيَ اللهُ عَنْهُ قَالَ</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
           <t>قُلْتُ: يَا رَسُولَ اللهِ أَخْبِرْنِي بِعَمَلٍ يُدْخِلُنِي الْجَنَّةَ وَيُبَاعِدُنِي عَنِ النَّارِ، قَالَ: لَقَدْ سَأَلْتَ عَنْ عَظِيمٍ وَإِنَّهُ لَيَسِيرٌ عَلَى مَنْ يَسَّرَهُ اللهُ تَعَالَى عَلَيْهِ: تَعْبُدُ اللهَ لَا تُشْرِكُ بِهِ شَيْئًا، وَتُقِيمُ الصَّلَاةَ، وَتُؤْتِي الزَّكَاةَ، وَتَصُومُ رَمَضَانَ، وَتَحُجُّ الْبَيْتَ. ثُمَّ قَالَ: أَلَا أَدُلُّكَ عَلَى أَبْوَابِ الْخَيْرِ؟ الصَّوْمُ جُنَّةٌ، وَالصَّدَقَةُ تُطْفِئُ الْخَطِيئَةَ كَمَا يُطْفِئُ الْمَاءُ النَّارَ، وَصَلَاةُ الرَّجُلِ فِي جَوْفِ اللَّيْلِ، ثُمَّ تَلَا: تَتَجَافَى جُنُوبُهُمْ عَنِ الْمَضَاجِعِ حَتَّى بَلَغَ يَعْمَلُونَ. ثُمَّ قَالَ: أَلَا أُخْبِرُكَ بِرَأْسِ الْأَمْرِ وَعَمُودِهِ وَذِرْوَةِ سَنَامِهِ؟ قُلْتُ: بَلَى يَا رَسُولَ اللهِ، قَالَ: رَأْسُ الْأَمْرِ الْإِسْلَامُ، وَعَمُودُهُ الصَّلَاةُ، وَذِرْوَةُ سَنَامِهِ الْجِهَادُ. ثُمَّ قَالَ: أَلَا أُخْبِرُكَ بِمِلَاكِ ذَلِكَ كُلِّهِ؟ قُلْتُ: بَلَى يَا رَسُولَ اللهِ، فَأَخَذَ بِلِسَانِهِ وَقَالَ: كُفَّ عَلَيْكَ هَذَا. قُلْتُ: يَا نَبِيَّ اللهِ وَإِنَّا لَمُؤَاخَذُونَ بِمَا نَتَكَلَّمُ بِهِ؟ فَقَالَ: ثَكِلَتْكَ أُمُّكَ، وَهَلْ يَكُبُّ النَّاسَ فِي النَّارِ عَلَى وُجُوهِهِمْ -أَوْ عَلَى مَنَاخِرِهِمْ- إِلَّا حَصَائِدُ أَلْسِنَتِهِمْ؟</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>قوله صلى الله عليه وسلم (لقد سألت عن عظيم، وإنه ليسير على من يسّره الله تعالى عليه) يعني على من وفّقه الله لعبادة مخلصة له الدين. ثم ذكر أركان الإسلام: عبادة الله وحده بلا شرك، وإقام الصلاة، وإيتاء الزكاة، وصوم رمضان، وحج البيت.
-ثم قال: ألا أدلك على أبواب الخير؟ الصوم هنا المراد به صوم التطوع (غير رمضان) لأنه قد تقدّم ذكره، ومراده الإكثار منه. والجُنّة أي المِجَنّ، أي الصوم سُترة لك ووقاية من النار. والصدقة هنا أراد بها غير صدقة الزكاة، تُطفئ الخطيئة. ثم قال: وصلاة الرجل في جوف الليل، ثم تلا آيات قيام الليل التي معناها: أن من قام في جوف الليل وترك لذة نومه وآثر رضا ربه على راحته، جزاه الله جزاء بما كان يعمل مما لا يعلمه أحد.
-ثم قال: ألا أخبرك برأس الأمر وعموده وذروة سنامه؟ فجعل الإسلام رأس الأمر كرأس الفحل من الإبل الذي لا يعيش الحيوان بدونه، وجعل عموده الصلاة، وهو الذي يقيمه في العادة (فلا يقوم البناء بغير عمود)، وذروة سنامه الجهاد، وذروة كل شيء أعلاه، والجهاد لا يقاومه شيء من الأعمال في الفضل.
-ثم قال: ألا أخبرك بملاك ذلك كله؟ فأخذ بلسانه وقال: كف عليك هذا. فسأله معاذ: وإنا لمؤاخذون بما نتكلم به؟ فقال له صلى الله عليه وسلم: ثكلتك أمك يا معاذ، وهل يكبّ الناس في النار على وجوههم -أو على مناخرهم- إلا حصائد ألسنتهم؟ وهذا يبيّن أن ضبط اللسان هو ملاك الأمر كله ومفتاح النجاة من كثير من المهالك.</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>سأل معاذ بن جبل النبي صلى الله عليه وسلم عن عمل يدخله الجنة ويبعده عن النار، فأجابه بأركان الإسلام أولاً: التوحيد، الصلاة، الزكاة، الصوم، الحج. ثم فتح له أبواب خير إضافية: الصوم التطوعي، الصدقة، وقيام الليل. ثم لخص كل الدين في ثلاث كلمات: رأس الأمر الإسلام (لا حياة بدونه)، وعموده الصلاة (لا يقوم البناء بدونها)، وذروة سنامه الجهاد (أعلى درجاته). وفي الختام كشف له سر كل هذا: ضبط اللسان، فهو ملاك الأمر كله، إذ إن أكثر ما يُدخل الناس النار هو حصائد ألسنتهم لا أفعالهم.</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>6</v>
+ثم قال: ألا أدلك على أبواب الخير؟ الصوم هنا المراد به صوم التطوع (غير رمضان) لأنه قد تقدّم ذكره، ومراده الإكثار منه. والجُنّة أي المِجَنّ، أي الصوم سُترة لك ووقاية من النار. والصدقة هنا أراد بها غير صدقة الزكاة، تُطفئ الخطيئة. ثم قال: وصلاة الرجل في جوف الليل، ثم تلا آيات قيام الليل التي معناها: أن من قام في جوف الليل وترك لذة نومه وآثر على ذلك ما يرجوه من ربه، جزاه الله جزاء ما في الآية من قوله (فلا تعلم نفس ما أُخفي لهم من قرة أعين جزاء بما كانوا يعملون). وقد جاء في بعض الأخبار: أن الله تعالى يباهي بقوّام الليل في الظلام يقول: (انظروا إلى عبادي وقد قاموا في ظلم الليل حيث لا يراهم أحد غيري، أشهدكم أني قد أبحتهم دار كرامتي).
+ثم قال: ألا أخبرك برأس الأمر وعموده وذروة سنامه؟ فجعل الإسلام رأس الأمر كرأس الفحل من الإبل الذي لا يعيش الحيوان بدونه، وجعل عموده الصلاة، وهو الذي يقيمه في العادة (فلا يقوم البناء بغير عمود)، وذروة سنامه الجهاد، وذروة كل شيء أعلاه وهو طرف سنام البعير، والجهاد لا يقاومه شيء من الأعمال في الفضل، كما روى أبو هريرة قال: جاء رجل إلى رسول الله صلى الله عليه وسلم فقال: دلني على عمل يعدل الجهاد؟ قال: (لا أجده) ثم قال: (هل تستطيع إذا خرج المجاهد أن تدخل مسجدك فتقوم ولا تفتر وتصوم ولا تفطر؟) فقال: ومن يستطيع ذلك؟
+ثم قال: ألا أخبرك بملاك ذلك كله؟ فأخذ بلسانه وقال: كف عليك هذا. فسأله معاذ: وإنا لمؤاخذون بما نتكلم به؟ فقال له صلى الله عليه وسلم: ثكلتك أمك يا معاذ، وهل يكبّ الناس في النار على وجوههم -أو على مناخرهم- إلا حصائد ألسنتهم؟ وهذا يبيّن أن ضبط اللسان هو ملاك الأمر كله ومفتاح النجاة من كثير من المهالك، وقد تقدّم في الحديث المتفق عليه (من كان يؤمن بالله واليوم الآخر فليقل خيراً أو ليصمت)، وفي حديث آخر (من يضمن لي ما بين لحييه وما بين رجليه أضمن له الجنة).</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>سأل معاذ بن جبل النبي صلى الله عليه وسلم عن عمل يدخله الجنة ويبعده عن النار، فأجابه بأركان الإسلام أولاً: التوحيد، الصلاة، الزكاة، الصوم، الحج. ثم فتح له أبواب خير إضافية: الصوم التطوعي، الصدقة، وقيام الليل. ثم لخص كل الدين في ثلاث كلمات: رأس الأمر الإسلام (لا حياة بدونه)، وعموده الصلاة (لا يقوم البناء بدونها)، وذروة سنامه الجهاد (أعلى درجاته، ولا يعدله عمل آخر). وفي الختام كشف له سر كل هذا: ضبط اللسان، فهو ملاك الأمر كله، إذ إن أكثر ما يُدخل الناس النار هو حصائد ألسنتهم لا أفعالهم.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="31" ht="90" customHeight="1">
@@ -1411,22 +1721,34 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
+          <t>أبو ثعلبة الخشني جرثوم بن ناشر رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي ثَعْلَبَةَ الْخُشَنِيِّ جُرْثُومِ بْنِ نَاشِرٍ رَضِيَ اللهُ تَعَالَى عَنْهُ عَنْ رَسُولِ اللَّهِ صَلَّى اللهُ عَلَيْهِ وَسَلَّمَ قَالَ</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
           <t>إِنَّ اللهَ تَعَالَى فَرَضَ فَرَائِضَ فَلَا تُضَيِّعُوهَا، وَحَدَّ حُدُودًا فَلَا تَعْتَدُوهَا، وَحَرَّمَ أَشْيَاءَ فَلَا تَنْتَهِكُوهَا، وَسَكَتَ عَنْ أَشْيَاءَ رَحْمَةً لَكُمْ غَيْرَ نِسْيَانٍ فَلَا تَبْحَثُوا عَنْهَا</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>قوله (فرض) أي أوجب وألزم. وقوله (فلا تضيعوها) أي فلا تتهاونوا في أدائها. هذا الحديث أصل عظيم يقسم أحكام الشريعة إلى أربعة أقسام واضحة: فرائض أوجبها الله يجب أداؤها والمحافظة عليها دون تفريط، وحدود وضعها الله للأحكام يجب الوقوف عندها دون تجاوز أو تعدٍّ، ومحرمات نهى الله عنها يجب الانتهاء عنها والابتعاد عنها بالكلية، وأشياء سكت عنها الشرع رحمة بالعباد لا نسياناً منه سبحانه (فهو منزّه عن النسيان)، فهذه لا ينبغي البحث عنها أو التنقيب عن حكمها بالتكلف، بل تُترك على أصل الإباحة تيسيراً على الناس.
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>قوله (فرض) أي أوجب وألزم. وقوله (فلا تنتهكوها) أي فلا تدخلوا فيها. هذا الحديث أصل عظيم يقسم أحكام الشريعة إلى أربعة أقسام واضحة: فرائض أوجبها الله يجب أداؤها والمحافظة عليها دون تفريط، وحدود وضعها الله للأحكام يجب الوقوف عندها دون تجاوز أو تعدٍّ، ومحرمات نهى الله عنها يجب الانتهاء عنها والابتعاد عنها بالكلية، وأشياء سكت عنها الشرع رحمة بالعباد لا نسياناً منه سبحانه (فهو منزّه عن النسيان)، فهذه لا ينبغي البحث عنها أو التنقيب عن حكمها بالتكلف، بل تُترك على أصل الإباحة تيسيراً على الناس.
+وأما النهي عن البحث عما سكت الله عنه فهو موافق لقوله صلى الله عليه وسلم: (ذروني ما تركتكم، فإنما أهلك الذين من قبلكم كثرة مسائلهم واختلافهم على أنبيائهم). قال بعض العلماء: كانت بنو إسرائيل يسألون فيُجابون ويُعطَون ما طلبوا حتى كان ذلك فتنة لهم، وأدّى ذلك إلى هلاكهم، وكان الصحابة رضي الله عنهم قد فهموا ذلك فكفّوا عن السؤال إلا فيما لا بد منه، وكان يعجبهم أن يجيء الأعراب يسألون رسول الله صلى الله عليه وسلم فيسمعون ويعون. وقد بالغ قوم حتى قالوا: لا يجوز السؤال في النوازل للعلماء حتى تقع، وقد كان السلف يقولون في مثلها: دعوها حتى تنزل، إلا أن العلماء لما خافوا ذهاب العلم أصّلوا وفرّعوا ومهّدوا وسطّروا.
+واختلف العلماء في الأشياء قبل ورود الشرع بحكمها: أهي على الحظر، أو الإباحة، أو الوقف؟ على ثلاثة مذاهب، وذلك مذكور في كتب الأصول.
 هذا التقسيم يعطي المسلم منهجاً واضحاً للتعامل مع الأحكام الشرعية: الجد في أداء الواجبات، الانضباط بالحدود، الاجتناب التام للمحرمات، والتوسع فيما سكت عنه الشرع دون تكلف السؤال عما لا حاجة إليه ولا فائدة من معرفته.</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>قاعدة تنظيمية جامعة لكل الأحكام الشرعية: فرائض يجب أداؤها كاملة دون تقصير، وحدود لا يجوز تجاوزها، ومحرمات يجب الابتعاد عنها تماماً، وأشياء سكت عنها الشرع رحمة بنا لا نسياناً، فلا داعي للتنقيب عنها أو تعقيد ما تركه الله بسيطاً. هذا الحديث يعلمنا أن الدين نظام متوازن: له واجبات واضحة، وحدود محفوظة، ومحرمات محددة، ومساحة واسعة من الإباحة والحرية لم يُقيدها الشرع عمداً رحمة بنا، فلا ينبغي أن نضيق على أنفسنا فيما وسّعه الله.</t>
         </is>
       </c>
-      <c r="F31" s="2" t="n">
-        <v>5</v>
+      <c r="H31" s="2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="32" ht="90" customHeight="1">
@@ -1440,22 +1762,32 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
+          <t>أبو العباس سهل بن سعد الساعدي رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي الْعَبَّاسِ سَهْلِ بْنِ سَعْدٍ السَّاعِدِيِّ رَضِيَ اللهُ تَعَالَى عَنْهُ قَالَ: جَاءَ رَجُلٌ إِلَى النَّبِيِّ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ فَقَالَ:</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
           <t>يَا رَسُولَ اللهِ، دُلَّنِي عَلَى عَمَلٍ إِذَا عَمِلْتُهُ أَحَبَّنِي اللهُ وَأَحَبَّنِي النَّاسُ، فَقَالَ: ازْهَدْ فِي الدُّنْيَا يُحِبَّكَ اللهُ، وَازْهَدْ فِيمَا عِنْدَ النَّاسِ يُحِبَّكَ النَّاسُ</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>اعلم أن رسول الله صلى الله عليه وآله وسلم قد حث على التقلل من الدنيا والزهد فيها، وقال: (كن في الدنيا كأنك غريب أو عابر سبيل)، وقال: (حب الدنيا رأس كل خطيئة)، وفي حديث آخر: (إن الزاهد في الدنيا يريح قلبه في الدنيا والآخرة، والراغب في الدنيا يتعب قلبه في الدنيا والآخرة).
 واعلم أن من في الدنيا ضيف، وما في يده عارية، والضيف مرتحل، والعارية مردودة، والدنيا عرض حاضر يأكل منها البر والفاجر، وهي مبغضة لأولياء الله، فمن شاركهم في محبوبهم أبغضوه. وقد أرشد رسول الله صلى الله عليه وسلم السائل إلى تركها بالزهد فيها ووعده على ذلك حب الله تعالى، وهو رضاه عنه، فإن الحب من الله تعالى لعباده رضاه عنهم. وأرشده إلى الزهد فيما في أيدي الناس إن أراد محبة الناس له، فإنه ليس في أيدي الناس شيء يتباغضون عليه ويتنافسون فيه إلا الدنيا.
 وقال صلى الله عليه وسلم: (من كانت الآخرة همه جمع الله شمله وجعل غناه في قلبه وأتته الدنيا وهي راغمة، ومن كانت الدنيا همه شتّت الله عليه شمله وجعل فقره بين عينيه ولم يأته من الدنيا إلا ما قُدّر له). السعيد من اختار الباقية التي يدوم نعيمها، على البالية التي يلحقها انقضاء وذهاب.</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>سأل صحابي النبي صلى الله عليه وسلم عن عمل يجلب له محبة الله ومحبة الناس معاً، فأجابه بوصفة بسيطة مزدوجة: ازهد في الدنيا يحبك الله، وازهد فيما عند الناس يحبك الناس. الزهد هنا لا يعني ترك العمل أو الطموح، بل عدم التعلق القلبي بالدنيا لدرجة أن تتحكم في قراراتنا وسعادتنا. فمن جعل الآخرة همه الأول، جمع الله له أمره ووضع الغنى في قلبه رغم قلة ما بيده، ومن جعل الدنيا كل همه تشتت وشعر بالفقر مهما امتلك. كما أن الزهد فيما بيد الناس - أي عدم التطلع لممتلكاتهم بحسد أو طمع - يجلب محبتهم الصادقة بدل التنافس المرير.</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="H32" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1470,22 +1802,33 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
+          <t>أبو سعيد سعد بن مالك بن سنان الخدري رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي سَعِيدٍ سَعْدِ بْنِ مَالِكِ بْنِ سِنَانٍ الْخُدْرِيِّ رَضِيَ اللهُ تَعَالَى عَنْهُ أَنَّ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ:</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
           <t>لَا ضَرَرَ وَلَا ضِرَارَ</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>اعلم أن من أضرّ بأخيه فقد ظلمه، والظلم حرام كما تقدم في حديث أبي ذر (يا عبادي إني حرمت الظلم على نفسي وجعلته بينكم محرماً فلا تظالموا)، وقال النبي صلى الله عليه وسلم: (إن دماءكم وأموالكم وأعراضكم عليكم حرام).
-وأما قوله (لا ضرر ولا ضرار) فقال ابن حبيب: الضرر عند أهل العربية الاسم، والضرار الفعل، فمعنى (لا ضرر) أي لا يُدخل أحد على أحد ضرراً لم يدخله هو على نفسه، ومعنى (لا ضرار) لا يُضارّ أحد بأحد. وقال المحاسبي: الضرر هو الذي لا منفعة فيه لضاره وفيه على جاره مضرة، وهذا وجه حسن. وقال بعضهم: الضرر والضرار مثل القتل والقتال، فالضرر أن يضرّك من غير جهة الاعتداء، والضرار أن تضرّ به من غير جهة الاعتداء بالمثل والانتصار بالحق.
-وقد اختلف الفقهاء في الذي يجحد حقاً عليه ثم يظفر بمال المجحود له بعد ذلك: فقال بعضهم: ليس له أن يأخذ من ذلك حقه من غير خيانة من خانه، لظاهر قوله (أدّ الأمانة إلى من ائتمنك ولا تخن من خانك)، وقال آخرون: له أن ينتصر منه ويأخذ حقه من تحت يده، واحتجوا بحديث عائشة في قصة هند مع أبي سفيان.</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
+وأما قوله (لا ضرر ولا ضرار) فقال ابن حبيب: الضرر عند أهل العربية الاسم، والضرار الفعل، فمعنى (لا ضرر) أي لا يُدخل أحد على أحد ضرراً لم يدخله هو على نفسه، ومعنى (لا ضرار) لا يُضارّ أحد بأحد. وقال المحاسبي: الضرر هو الذي له فيه منفعة وعلى جارك فيه مضرة، وهذا وجه حسن. وقال بعضهم: الضرر والضرار مثل القتل والقتال، فالضرر أن يضرّك من غير جهة الاعتداء، والضرار أن تضرّ به من غير جهة الاعتداء بالمثل والانتصار بالحق.
+وقد اختلف الفقهاء في الذي يجحد حقاً عليه ثم يظفر بمال المجحود له بعد ذلك: فقال بعضهم: ليس له أن يأخذ من ذلك حقه من غير خيانة من خانه، لظاهر قوله (أدّ الأمانة إلى من ائتمنك ولا تخن من خانك)، وقال آخرون: له أن ينتصر منه ويأخذ حقه من تحت يده، واحتجوا بحديث عائشة في قصة هند مع أبي سفيان. والذي يصح في النظر: أنه ليس لأحد أن يضرّ بأخيه سواء ضرّه أم لا، إلا أن له أن ينتصر ويعاقب إن قدر بما أُبيح له بالحق، وليس ذلك ظلماً ولا ضراراً إذا كان على الوجه الذي أباحته السنة.
+وقال الشيخ أبو عمرو بن الصلاح رحمه الله: أسند الدارقطني هذا الحديث من جميع وجوهه يقوّي بعضها بعضاً ويُحسّنه، وقد نقله جماهير أهل العلم واحتجّوا به. وعن أبي داود أنه قال: الفقه يدور على خمسة أحاديث، وعدّ هذا الحديث منها. قال الشيخ: وعَدُّ أبي داود له من الخمسة يُشعر بكونه عنده غير ضعيف. وقد نبّه على أن هذا الحديث يجري على ألسنة كثير من الفقهاء والمحدّثين بلفظ (لا ضرر ولا إضرار) بهمزة مكسورة قبل الضاد، والأصح هو ما تقدّم: (لا ضرر ولا ضرار).</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>قاعدة موجزة لكنها من أعظم قواعد الفقه الإسلامي: لا يجوز أن تبدأ بإلحاق الضرر بأحد، ولا أن تقابل الضرر بضرر مماثل أو أكبر انتقاماً. هذه القاعدة تحكم كثيراً من جوانب الحياة: العلاقات الأسرية، المعاملات المالية، الجوار، العمل. فكل تصرف يُلحق أذى بالآخرين دون مبرر شرعي محرم، وحتى في حالات الدفاع عن الحق يبقى هناك حدود لا يجوز تجاوزها. هذا المبدأ يرسخ فكرة أن الحرية الشخصية تقف عند حدود عدم الإضرار بالآخرين.</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="H33" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1500,22 +1843,33 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
+          <t>عبد الله بن عباس رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>عَنِ ابْنِ عَبَّاسٍ رَضِيَ اللهُ عَنْهُمَا أَنَّ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ:</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
           <t>لَوْ يُعْطَى النَّاسُ بِدَعْوَاهُمْ لَادَّعَى رِجَالٌ أَمْوَالَ قَوْمٍ وَدِمَاءَهُمْ، لَكِنَّ الْبَيِّنَةَ عَلَى الْمُدَّعِي وَالْيَمِينَ عَلَى مَنْ أَنْكَرَ</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>معنى هذا الحديث: أنه لو يُعطى الناس بمجرد دعواهم من غير بينة لادّعى رجال أموال قوم ودماءهم، لكن البيّنة على المدّعي واليمين على من أنكر. وهذا الحديث أصل من أصول الأحكام وأعظم مرجع عند التنازع والخصام، ويقتضي أن لا يحكم أحد بمجرد دعواه.
-وقوله (لادّعى رجال دماء رجال وأموالهم) استدل بهذا بعض الناس على إبطال قول القائل عند سماع قول القتيل (فلان قتلني) أو (دمي عند فلان)، لأنه إذا لم يُسمع قول فلان (له عند فلان دينار) لا يُسمع (دمي عند فلان)، وقد أجاب مالك بأن هذا لا حجة لهم فيه، لأنه لم يُسند رفع الدية أو القصاص إلى قول المدعى، بل يجعل قول القتيل (دمي عند فلان) لوثاً يُنتزى به إلى قسامة تبرأ بها الأيمان، كسائر أنواع اللوث.
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>الذي في الصحيحين من هذا الحديث: قال ابن أبي مليكة: كتب ابن عباس رضي الله عنهما أن النبي صلى الله عليه وسلم قضى باليمين على المدّعى عليه. وفي رواية: أن النبي صلى الله عليه وسلم قال (لو يُعطى الناس بدعواهم لادّعى رجال دماء رجال وأموالهم ولكن اليمين على المدّعى عليه). وقد روى هذا الحديث بتمامه البخاري ومسلم في صحيحيهما مرفوعاً من رواية ابن عباس، وهكذا رواه أصحاب السنن وغيرهم، وقال الأصيلي: لا يصح رفعه، إنما هو من قول ابن عباس. قال المصنف: إذا صح رفعه بشهادة الإمامين فلا يضرّ كونه موقوفاً أيضاً، ولا يُعدّ ذلك تعارضاً ولا اضطراباً.
+ومعنى هذا الحديث: أنه لو يُعطى الناس بمجرد دعواهم من غير بينة لادّعى رجال أموال قوم ودماءهم، لكن البيّنة على المدّعي واليمين على من أنكر. وهذا الحديث أصل من أصول الأحكام وأعظم مرجع عند التنازع والخصام، ويقتضي أن لا يحكم أحد بمجرد دعواه.
+وقوله (لادّعى رجال دماء رجال وأموالهم) استدل بهذا بعض الناس على إبطال قول القائل عند سماع قول القتيل (فلان قتلني) أو (دمي عند فلان)، لأنه إذا لم يُسمع قول فلان (له عند فلان دينار) لم يُسمع (دمي عند فلان) بطريق الأولى. ولا حجة لهم في ذلك، لأنه لم يُسند الدية أو القصاص على القتل إلى قول المدّعي، بل يجعل قول القتيل (دمي عند فلان) لوثاً ينبري به المدّعي إلى القسامة حتى يبرؤوا بالأيمان، كسائر أنواع اللوث.
 وقوله (ولكن اليمين على المدعى عليه) أجمع العلماء على استحقاق اليمين على المدعى عليه في الأموال، واختلفوا في غير ذلك من الحقوق والحدود، ومن العلماء من قال: يلزم المدعى عليه في كل حق يدّعى عليه من طلاق أو نكاح أو عتق أخذاً بظاهر عموم الحديث، وقال أبو حنيفة رحمه الله: يحلف على الطلاق والنكاح والعتق وإن نكل لزمه ذلك كله، ولا يستحلف في الحدود.</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>قاعدة عدالة أساسية: لا يُعطى أحد ما يدّعيه لمجرد ادعائه، لأنه لو كان ذلك ممكناً لادّعى الناس أموال غيرهم ودماءهم بلا وجه حق. لذلك وضع الشرع ضابطاً عادلاً: من يدّعي حقاً عليه أن يأتي بالدليل (البينة)، ومن يُنكر ادعاء ضده عليه أن يحلف اليمين. هذه القاعدة أساس النظام القضائي العادل في كل زمان ومكان، فهي تحمي الناس من الاتهامات الباطلة وتمنع الفوضى في حقوق الأفراد وأموالهم وأعراضهم، وتذكرنا أن الكلام وحده - مهما بدا مقنعاً - لا يكفي دليلاً.</t>
         </is>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="H34" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1530,23 +1884,41 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
+          <t>أبو سعيد الخدري رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي سَعِيدٍ الْخُدْرِيِّ رَضِيَ اللهُ عَنْهُ قَالَ: سَمِعْتُ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ يَقُولُ:</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
           <t>مَنْ رَأَى مِنْكُمْ مُنْكَرًا فَلْيُغَيِّرْهُ بِيَدِهِ، فَإِنْ لَمْ يَسْتَطِعْ فَبِلِسَانِهِ، فَإِنْ لَمْ يَسْتَطِعْ فَبِقَلْبِهِ، وَذَلِكَ أَضْعَفُ الْإِيمَانِ</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>أورد مسلم هذا الحديث عن طارق بن شهاب: أول من بدأ بالخطبة يوم العيد قبل الصلاة مروان، فقام إليه رجل فقال: الصلاة قبل الخطبة، فقال: قد تُرك ما هناك، فقال أبو سعيد: أما هذا فقد قضى ما عليه، سمعت رسول الله صلى الله عليه وسلم يقول (من رأى منكم منكراً فليغيره...) الحديث.
-إن الأمر بالمعروف والنهي عن المنكر فرض كفاية، إذا قام به من يكفي سقط عن الباقي، وإن تركه الجميع أثم كل من تمكن منه بلا عذر، إلا أن كان في موضع لا يتمكن من إزالته إلا هو، كأن يراه من زوجته أو ولده أو غلامه فيقصر. قال العلماء: ولا يسقط الأمر بالمعروف والنهي عن المنكر لكون المنكر لا يقبل بظنه، بل يجب عليه فعله. ولا يشترط في الآمر بالمعروف والناهي عن المنكر أن يكون كامل الحال ممتثلاً ما يأمر به مجتنباً ما ينهى عنه، بل عليه أن يأمر وينهى وإن كان مرتكباً خلاف ذلك، لأنه يجب عليه شيئان: أن يأمر نفسه وينهاها، وأن يأمر غيره وينهاه، فإذا ترك أحدهما لا يسقط الآخر.
-ولا يختص الأمر بالمعروف والنهي عن المنكر بأصحاب الولاية، بل ذلك ثابت لآحاد المسلمين، وإنما يأمر وينهى من كان عالماً بما يأمر به وينهى عنه، فإن كان من الأمور الظاهرة كالصلاة والزنا وشرب الخمر فكل المسلمين علماء بذلك، وإن كان من دقائق الأفعال والأقوال المتعلقة بالاجتهاد فليس ذلك للعوام مدخل فيه، بل ذلك للعلماء، ولا ينكر أحد على أحد المذهبين في المسائل المختلف فيها.
-قال الشيخ محيي الدين رحمه الله: واعلم أن باب الأمر بالمعروف والنهي عن المنكر قد ضُيّع أكثره من أزمان متطاولة، ولم يبق منه في هذه الأزمان إلا رسوم قليلة جداً، وهو باب عظيم به قوام الأمر وملاكه، وإذا كثرت الخبائث عمّ العقاب الصالح والطالح. وينبغي للآمر بالمعروف والناهي عن المنكر أن يكون ذلك برفق ليكون أقرب إلى تحصيل المقصود، فقد قال الإمام الشافعي رحمه الله تعالى: من وعظ أخاه سراً فقد نصحه وزانه، ومن وعظه علانية فقد فضحه وشانه.</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>أورد مسلم هذا الحديث عن طارق بن شهاب: أول من بدأ بالخطبة يوم العيد قبل الصلاة مروان، فقام إليه رجل فقال: الصلاة قبل الخطبة، فقال: قد تُرك ما هناك، فقال أبو سعيد: أما هذا فقد قضى ما عليه، سمعت رسول الله صلى الله عليه وسلم يقول (من رأى منكم منكراً فليغيره...) الحديث. وفي هذا دليل على أنه لم يعمل بذلك أحد قبل مروان.
+فإن قيل: كيف تأخر أبو سعيد عن تغيير هذا المنكر حتى أنكره هذا الرجل؟ قيل: يُحتمل أن أبا سعيد لم يكن حاضراً أول ما شرع مروان في تقديم الخطبة وأن الرجل أنكره عليه ثم دخل أبو سعيد، ويُحتمل أنه كان حاضراً لكنه خاف على نفسه حصول فتنة بسبب إنكاره فسقط عنه الإنكار، ويُحتمل أن أبا سعيد هَمَّ بالإنكار فبدره الرجل فأمضاه أبو سعيد، والله أعلم. وقد جاء في الحديث الآخر الذي اتفق عليه البخاري ومسلم في باب صلاة العيدين: أن أبا سعيد هو الذي جذب بيد مروان حين أراد أن يصعد المنبر قبل الصلاة، فيُحتمل أنهما قضيتان.
+وأما قوله (فليغيّره) فهو أمر إيجاب بإجماع الأمة، وقد تطابق الكتاب والسنة على وجوب الأمر بالمعروف والنهي عن المنكر، وهو أيضاً من أصول الدين. وأما قوله تعالى: (عليكم أنفسكم لا يضركم من ضلّ إذا اهتديتم) فليس مخالفاً لما ذكرنا، لأن المذهب الصحيح عند المحققين في معنى الآية أنكم إذا فعلتم ما كُلّفتم به من الأمر بالمعروف والنهي عن المنكر لا يضركم تقصير غيركم عن ذلك، كما قال تعالى: (ولا تزر وازرة وزر أخرى)، فمهما كُلّف به المسلم من الأمر بالمعروف والنهي عن المنكر، فإذا فعله ولم يمتثل المخاطَب به فلا عتب عليه، إنما عليه الأمر والنهي لا القبول، والله أعلم.
+ثم إن الأمر بالمعروف والنهي عن المنكر فرض كفاية، إذا قام به من يكفي سقط عن الباقي، وإن تركه الجميع أثم كل من تمكن منه بلا عذر، إلا أن كان في موضع لا يتمكن من إزالته إلا هو، كأن يراه من زوجته أو ولده أو غلامه فيقصر. قال العلماء: ولا يسقط الأمر بالمعروف والنهي عن المنكر لكون المنكر لا يُقبَل بظنه، بل يجب عليه فعله، قال الله تعالى: (وذكِّر فإن الذكرى تنفع المؤمنين)، وليس عليه القبول، قال الله تعالى: (ما على الرسول إلا البلاغ).
+ولا يُشترط في الآمر بالمعروف والناهي عن المنكر أن يكون كامل الحال ممتثلاً ما يأمر به مجتنباً ما ينهى عنه، بل عليه أن يأمر وينهى وإن كان مرتكباً خلاف ذلك، لأنه يجب عليه شيئان: أن يأمر نفسه وينهاها، وأن يأمر غيره وينهاه، فإذا ترك أحدهما لا يسقط الآخر.
+ولا يختص الأمر بالمعروف والنهي عن المنكر بأصحاب الولاية، بل ذلك ثابت لآحاد المسلمين، وإنما يأمر وينهى من كان عالماً بما يأمر به وينهى عنه، فإن كان من الأمور الظاهرة كالصلاة والزنا وشرب الخمر فكل المسلمين علماء بذلك، وإن كان من دقائق الأفعال والأقوال المتعلقة بالاجتهاد فليس ذلك للعوام مدخل فيه، بل ذلك للعلماء، ولا ينكر أحد على أحد المذهبين في المسائل المختلف فيها، لأن كل مجتهد مصيب عند كثير من المحققين، وعلى المذهب الآخر: المصيب واحد غير متعين لنا والإثم موضوع عن المخطئ، لكن على جهة النصيحة والخروج من الخلاف فِعله حسن مندوب إليه.
+قال الشيخ محيي الدين رحمه الله: واعلم أن باب الأمر بالمعروف والنهي عن المنكر قد ضُيّع أكثره من أزمان متطاولة، ولم يبق منه في هذه الأزمان إلا رسوم قليلة جداً، وهو باب عظيم به قوام الأمر وملاكه، وإذا كثرت الخبائث عمّ العقاب الصالح والطالح، وإذا لم يأخذوا على يد الظالم أوشك الله أن يعمّهم بعذاب. قال الله تعالى: (فليحذر الذين يخالفون عن أمره أن تصيبهم فتنة أو يصيبهم عذاب أليم). فينبغي لطالب الآخرة والساعي في تحصيل رضا الله عز وجل أن يعتني بهذا الباب، فإن نفعه عظيم ولا سيما لارتفاع مرتبته، ولا يهابنّ من ينكر عليه، لقوله تعالى: (ولينصرنّ الله من ينصره)، واعلم أن الأجر على قدر النصب. ولا يترك ذلك أيضاً لأجل مصادقته ومودته، فإن الصديق للإنسان هو الذي يسعى في عمارة آخرته وإن أدى ذلك إلى نقص في دنياه، وعدوّه من يسعى في ذهاب آخرته أو نقصها وإن حصل بسببه نفع في دنياه.
+وينبغي للآمر بالمعروف والناهي عن المنكر أن يكون ذلك برفق ليكون أقرب إلى تحصيل المقصود، فقد قال الإمام الشافعي رحمه الله تعالى: من وعظ أخاه سراً فقد نصحه وزانه، ومن وعظه علانية فقد فضحه وشانه.
+ومما يتساهل الناس فيه من هذا الباب: ما إذا رأوا إنساناً يبيع متاعاً أو حيواناً فيه عيب فلا يبيّنه للمشتري ولا يعرّفونه ذلك مع سؤالهم عنه، فإن الدين النصيحة، ومن لم ينصح فقد غشّ.
+وقوله صلى الله عليه وسلم (فليغيّره بيده فإن لم يستطع فبلسانه فإن لم يستطع فبقلبه) معناه: أن يُزيله بما هو في وسعه وطاقته، وليس الإنكار بالقلب إزالة له وتغييراً كاملاً، لكنه هو الذي في وسعه. وقوله (وذلك أضعف الإيمان) معناه -والله أعلم- أقلّه ثمرة، وقد جاء في رواية أخرى (وليس وراء ذلك من الإيمان حبة خردل)، أي لم يبق وراء ذلك مرتبة أخرى، والإيمان في هذا الحديث يعني الإسلام.
+وليس للآمر بالمعروف والناهي عن المنكر أن يبحث عن المنكر ويتفتش ويتجسس ويقتحم الدور ويتخمّن بالظنون، بل إن عثر على منكر غيره أنكره. قال الماوردي: ليس له أن يقتحم إلا أن يثق بأن رجلاً خلا برجل ليقتله، أو امرأة خلا بها ليزني بها، فيجوز له في مثل هذه الحال أن يتجسس ويُقدم على الكشف والبحث، حذراً من فوات ما لا يُستدرك.
+وفي هذا الحديث دليل على أن من خاف القتل أو الضرب سقط عنه التغيير، وهو مذهب المحققين سلفاً وخلفاً، وذهبت طائفة من الغلاة إلى أنه لا يسقط وإن خاف ذلك.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>تغيير المنكر واجب على كل مسلم بحسب استطاعته، وله ثلاث درجات: التغيير باليد لمن يملك القدرة والسلطة، فإن لم يستطع فباللسان بالنصح والكلام، فإن لم يستطع فبإنكاره بقلبه على الأقل وهذا أضعف درجات الإيمان لكنه ليس عدماً. هذا الواجب لا يقتصر على العلماء أو أصحاب السلطة، بل هو مسؤولية كل مسلم بحسب علمه وقدرته، ولا يشترط أن يكون الآمر بالمعروف كاملاً في نفسه، فلا يسقط عنه واجب النصح لغيره لمجرد تقصيره الشخصي. ويُستحب أن يكون ذلك برفق وسرية قدر الإمكان، فالنصح السري أدعى للقبول من التوبيخ العلني.</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="H35" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1561,27 +1933,38 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ رَضِيَ اللهُ عَنْهُ قَالَ: قَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ:</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
           <t>لَا تَحَاسَدُوا، وَلَا تَنَاجَشُوا، وَلَا تَبَاغَضُوا، وَلَا تَدَابَرُوا، وَلَا يَبِعْ بَعْضُكُمْ عَلَى بَيْعِ بَعْضٍ، وَكُونُوا عِبَادَ اللهِ إِخْوَانًا، الْمُسْلِمُ أَخُو الْمُسْلِمِ لَا يَظْلِمُهُ وَلَا يَخْذُلُهُ وَلَا يَكْذِبُهُ وَلَا يَحْقِرُهُ، التَّقْوَى هَاهُنَا -وَيُشِيرُ إِلَى صَدْرِهِ ثَلَاثَ مَرَّاتٍ- بِحَسْبِ امْرِئٍ مِنَ الشَّرِّ أَنْ يَحْقِرَ أَخَاهُ الْمُسْلِمَ، كُلُّ الْمُسْلِمِ عَلَى الْمُسْلِمِ حَرَامٌ: دَمُهُ وَمَالُهُ وَعِرْضُهُ</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>قوله (لا تحاسدوا): الحسد هو تمني زوال النعمة عن المحسود، وفي حديث آخر (إياكم والحسد فإن الحسد يأكل الحسنات كما تأكل النار الحطب). فأما الغبطة فهي تمني مثل حال المغبوط من غير تمني زوالها عنه، وهي جائزة، كما قال النبي صلى الله عليه وسلم (لا حسد إلا في اثنتين) أي لا غبطة.
 قوله (ولا تناجشوا): أصل النجش الختل، ومنه قيل للصائد (ناجش) لأنه يختل الصيد ويحتال له، والمراد هنا الزيادة في ثمن السلعة ممن لا يريد شراءها لخداع المشتري.
 قوله (ولا تباغضوا): أي لا تتعاطوا أسباب التباغض، لأن الحب والبغض معانٍ قلبية لا قدرة للإنسان على اكتسابها ابتداءً، كما قال النبي صلى الله عليه وسلم (هذا قسمي فيما أملك فلا تؤاخذني فيما تملك ولا أملك) يعني الحب والبغضاء. والتدابر: المعاداة، وقيل المقاطعة، لأن كل واحد يولي صاحبه دبره.
-قوله (ولا يبع بعضكم على بيع بعض): معناه أن يقول لمن اشترى سلعة في مدة الخيار: افسخ هذا البيع وأنا أبيعك مثله أو أجود منه بثمنه أو أقل، وهذا حرام بعد استقرار الثمن والرضى بين المتبايعين.
+قوله (ولا يبع بعضكم على بيع بعض): معناه أن يقول لمن اشترى سلعة في مدة الخيار: افسخ هذا البيع وأنا أبيعك مثله أو أجود منه بثمنه أو أقل، وهذا حرام بعد استقرار الثمن والرضى بين المتبايعين، وأما قبل الرضى فليس بحرام.
 ومعنى (كونوا عباد الله إخواناً): أي تعاملوا معاملة الإخوة الأشقاء في المودّة والرفق والتعاون والتلاطف. وقوله (المسلم أخو المسلم لا يظلمه ولا يخذله): الخذلان هو ترك الإعانة والنصرة، فإذا استعان به في دفع ظالم عنه لزمه إعانته إن أمكنه ولم يكن له عذر شرعي.
-قوله (التقوى هاهنا ويشير إلى صدره): أي إن الله لا ينظر إلى أجسادكم وصوركم، ولكن ينظر إلى قلوبكم، ومعناه أن الأعمال الظاهرة لا تحصل بها التقوى الحقيقية إلا بما يقع في القلب من عظمة الله وخشيته ومراقبته.
-قوله (بحسب امرئ من الشر أن يحقر أخاه المسلم): فيه تحذير عظيم، لأن الله تعالى لم يحقره إذ خلقه ورزقه وأحسن تقويم خلقه وسخّر له ما في السموات والأرض، ثم سماه مسلماً ومؤمناً وعبداً، فمن حقّر مسلماً فقد حقّر ما عظّمه الله عز وجل.</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
+وقوله (ولا يحقره) هو بالحاء المهملة والقاف: أي لا يتكبر عليه ويستصغره، وقد رواه بعضهم بضم الياء وبالحاء المعجمة وبالفاء، والمعروف الصواب هو الأول.
+قوله (التقوى هاهنا وأشار إلى صدره): أي إن الله لا ينظر إلى أجسادكم وصوركم، ولكن ينظر إلى قلوبكم، ومعناه أن الأعمال الظاهرة لا تحصل بها التقوى الحقيقية إلا بما يقع في القلب من عظمة الله وخشيته ومراقبته.
+قوله (بحسب امرئ من الشر أن يحقر أخاه المسلم): فيه تحذير عظيم، لأن الله تعالى لم يحقّره إذ خلقه ورزقه وأحسن تقويم خلقه وسخّر له ما في السموات والأرض، ثم سماه مسلماً ومؤمناً وعبداً، فمن حقّر مسلماً فقد حقّر ما عظّمه الله عز وجل. وكفاية ذلك في التحذير: أن من صور احتقار المسلم للمسلم أن لا يسلّم عليه إذا مرّ به، أو لا يردّ عليه السلام إذا بدأه به، ومنها أن يستصغره حتى كأنه لا يستحق في نظره أن يُدخله الله الجنة أو يُبعده من النار. وأما ما ينقصه العاقل من قدر الجاهل، أو العادل من قدر الفاسق، فليس ذلك احتقاراً للمسلم في ذاته، بل هو بسبب ما اتصف به من الجهل أو الفسق، فمتى فارق ذلك الوصف عاد إليه احترامه ورُفع قدره.</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>مجموعة توجيهات نبوية لبناء مجتمع متماسك ومتعاطف: لا حسد يتمنى زوال نعمة الآخرين، ولا خداع في البيع بالمزايدة الوهمية، ولا تباغض متعمد، ولا قطيعة، ولا إفساد لصفقات الآخرين. المسلمون إخوة يجب أن يتعاملوا بالمحبة والنصرة، لا ظلم ولا خذلان ولا كذب ولا احتقار بينهم. ويختم النبي صلى الله عليه وسلم بحقيقة عميقة: التقوى مكانها القلب لا المظهر الخارجي، واحتقار أي إنسان مسلم -مهما بدا بسيطاً في نظرنا- شر عظيم، لأن الله كرّم هذا الإنسان وخلقه وسخّر له الكون، فمن حقّره فقد استخف بما عظّمه الله.</t>
         </is>
       </c>
-      <c r="F36" s="2" t="n">
-        <v>6</v>
+      <c r="H36" s="2" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="37" ht="90" customHeight="1">
@@ -1595,24 +1978,34 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة رضي الله عنه</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ رَضِيَ اللهُ عَنْهُ عَنِ النَّبِيِّ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
           <t>مَنْ نَفَّسَ عَنْ مُؤْمِنٍ كُرْبَةً مِنْ كُرَبِ الدُّنْيَا نَفَّسَ اللهُ عَنْهُ كُرْبَةً مِنْ كُرَبِ يَوْمِ الْقِيَامَةِ، وَمَنْ يَسَّرَ عَلَى مُعْسِرٍ يَسَّرَ اللهُ عَلَيْهِ فِي الدُّنْيَا وَالْآخِرَةِ، وَمَنْ سَتَرَ مُسْلِمًا سَتَرَهُ اللهُ فِي الدُّنْيَا وَالْآخِرَةِ، وَاللهُ فِي عَوْنِ الْعَبْدِ مَا كَانَ الْعَبْدُ فِي عَوْنِ أَخِيهِ، وَمَنْ سَلَكَ طَرِيقًا يَلْتَمِسُ فِيهِ عِلْمًا سَهَّلَ اللهُ لَهُ بِهِ طَرِيقًا إِلَى الْجَنَّةِ، وَمَا اجْتَمَعَ قَوْمٌ فِي بَيْتٍ مِنْ بُيُوتِ اللهِ يَتْلُونَ كِتَابَ اللهِ وَيَتَدَارَسُونَهُ بَيْنَهُمْ إِلَّا نَزَلَتْ عَلَيْهِمُ السَّكِينَةُ وَغَشِيَتْهُمُ الرَّحْمَةُ وَحَفَّتْهُمُ الْمَلَائِكَةُ وَذَكَرَهُمُ اللهُ فِيمَنْ عِنْدَهُ، وَمَنْ بَطَّأَ بِهِ عَمَلُهُ لَمْ يُسْرِعْ بِهِ نَسَبُهُ</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>هذا الحديث جامع عظيم لأنواع من العلوم والقواعد والآداب، ففيه فضل قضاء حوائج المسلمين ونفعهم بما يتيسر من علم أو مال أو معاونة بإشارة أو مصلحة أو نصيحة أو غير ذلك، ومعنى تنفيس الكربة إزالتها.
-قوله (من ستر مسلماً) الستر عليه أن يستر زلاته، والمراد بالستر على من ليس معروفاً بالفساد، وهذا في ستر معصية وقعت وانقضت، أما إذا علم أنه مصمم على معصية وهو متلبس بها فيجب المبادرة عليه بالإنكار ومنعه منها.
+قوله (من ستر مسلماً): الستر عليه أن يستر زلاته، والمراد بالستر على من ليس معروفاً بالفساد، وهذا في ستر معصية وقعت وانقضت، أما إذا علم أنه مصمم على معصية وهو متلبس بها فيجب المبادرة عليه بالإنكار ومنعه منها إن لم يترتب على ذلك مفسدة. فأما من عُرف بالفساد فلا يُستحب الستر عليه، لأن ذلك يُطمِعه في الفساد والإيذاء وانتهاك المحرمات وجسارة غيره على مثله، بل يُستحب أن يُرفع أمره إلى ولي الأمر إذا أُمنت مفسدة ذلك. ويُستثنى من عموم فضل الستر أيضاً: جرح الرواة والشهود والأمناء على الصدقات والأوقاف والأيتام ونحوهم، فيجب بيان عيوبهم عند الحاجة إلى ذلك، ولا يحلّ الستر عليهم إذا رأى فيهم ما يقدح في أمانتهم أو أهليتهم، وليس هذا من الغيبة المحرمة، بل هو من النصيحة الواجبة لعموم المسلمين.
 وقوله (والله في عون العبد ما دام العبد في عون أخيه) هذا الجزاء الجميل الحاصل من الله تعالى بمعاونة العبد أخيه في حاجته. وفي الحديث فضل التيسير على المعسر وفضل السعي في طلب العلم، ويلزم من ذلك فضل الاشتغال بالعلم الشرعي، ويُشترط أن يقصد به وجه الله تعالى.
-قوله صلى الله عليه وسلم (وما اجتمع قوم في بيت من بيوت الله يتلون كتاب الله ويتدارسونه بينهم) هذا دليل على فضل الاجتماع على تلاوة القرآن في المساجد. و(السكينة) قال بعضهم: الرحمة، وقال بعضهم: الطمأنينة والوقار، وهذا أحسن. وقوله (وحفتهم الملائكة) أي أحدقوا بهم من كل جهة.
+قوله صلى الله عليه وسلم (وما اجتمع قوم في بيت من بيوت الله يتلون كتاب الله ويتدارسونه بينهم) هذا دليل على فضل الاجتماع على تلاوة القرآن في المساجد، وهو فضل عام لكل من اجتمع على ذلك ولو لم يكونوا علماء أو زهاداً. و(السكينة) قال بعضهم: الرحمة، وقال بعضهم -وهو الأحسن-: الطمأنينة والوقار. وقوله (وحفتهم الملائكة) أي أحدقوا بهم من كل جهة حتى كأنهم لا يتركون فرجة لشيطان. وقوله (وغشيتهم الرحمة): لا يُستعمل لفظ 'غشي' إلا فيما يشمل المغشي منه جميع أجزائه، فمعنى ذلك أن رحمة الله تنزل عليهم فتستوعبهم وتغمرهم بالكلية، حتى قيل: إن غشيان الرحمة هنا يكون بحيث يستوعب كل ذنب لهم إن شاء الله تعالى. وقوله (وذكرهم الله فيمن عنده) معناه أن الله تعالى يذكرهم في الملأ الأعلى فيمن عنده من الأنبياء وكرام الملائكة، وهذا غاية الشرف والتكريم لهم.
 وقوله (ومن بطّأ به عمله لم يسرع به نسبه) معناه: من كان قاصراً في عمله لم ينفعه شرف نسبه، فإن العمل الصالح هو الذي يبلغ درجات الآخرة ويرفع منزلة الإنسان عند الله، لا مجرد النسب دون عمل.</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>حديث جامع يعدد أنواعاً من الخير المتبادل: من ساعد مسلماً في تجاوز أزمته يسّر الله عليه أزماته يوم القيامة، ومن يسّر على معسر يسّر الله عليه في الدنيا والآخرة، ومن ستر عيب أخيه ستره الله، وطالب العلم يسهّل الله له طريقاً إلى الجنة، ومن اجتمع مع إخوانه على تلاوة القرآن ودراسته نزلت عليهم السكينة وحفتهم الملائكة. ويختم بتذكير مهم: النسب والمكانة الاجتماعية لا ترفع من قصّر في عمله، فالعمل الصالح هو معيار التقدم الحقيقي عند الله لا الانتساب لأسرة أو قبيلة معينة.</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="n">
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>حديث جامع يعدد أنواعاً من الخير المتبادل: من ساعد مسلماً في تجاوز أزمته يسّر الله عليه أزماته يوم القيامة، ومن يسّر على معسر يسّر الله عليه في الدنيا والآخرة، ومن ستر عيب أخيه ستره الله (إلا في حالات الشهادة والأمانة التي يجب فيها البيان لا الستر)، وطالب العلم يسهّل الله له طريقاً إلى الجنة، ومن اجتمع مع إخوانه على تلاوة القرآن ودراسته نزلت عليهم السكينة وغشيتهم الرحمة وحفتهم الملائكة وذكرهم الله فيمن عنده. ويختم بتذكير مهم: النسب والمكانة الاجتماعية لا ترفع من قصّر في عمله، فالعمل الصالح هو معيار التقدم الحقيقي عند الله لا الانتساب لأسرة أو قبيلة معينة.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1627,23 +2020,35 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
+          <t>عبد الله بن عباس رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>عَنِ ابْنِ عَبَّاسٍ رَضِيَ اللهُ عَنْهُمَا عَنْ رَسُولِ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ فِيمَا يَرْوِيهِ عَنْ رَبِّهِ تَبَارَكَ وَتَعَالَى قَالَ</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
           <t>إِنَّ اللهَ كَتَبَ الْحَسَنَاتِ وَالسَّيِّئَاتِ ثُمَّ بَيَّنَ ذَلِكَ: فَمَنْ هَمَّ بِحَسَنَةٍ فَلَمْ يَعْمَلْهَا كَتَبَهَا اللهُ عِنْدَهُ حَسَنَةً كَامِلَةً، وَإِنْ هَمَّ بِهَا فَعَمِلَهَا كَتَبَهَا اللهُ عِنْدَهُ عَشْرَ حَسَنَاتٍ إِلَى سَبْعِمِائَةِ ضِعْفٍ إِلَى أَضْعَافٍ كَثِيرَةٍ، وَإِنْ هَمَّ بِسَيِّئَةٍ فَلَمْ يَعْمَلْهَا كَتَبَهَا اللهُ عِنْدَهُ حَسَنَةً كَامِلَةً، وَإِنْ هَمَّ بِهَا فَعَمِلَهَا كَتَبَهَا اللهُ سَيِّئَةً وَاحِدَةً</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>هذا حديث شريف عظيم فيه بيان مقدار تفضل الله عز وجل على خلقه، بأن جعل هم العبد بالحسنة وإن لم يعملها حسنة كاملة، وجعل همه بالسيئة إن لم يعملها حسنة أيضاً، ولا يكتبها سيئة إلا إذا عملها فتُكتب سيئة واحدة فقط. وإنما جُعل الهمّ بالحسنة حسنة لأن إرادة الخير فعل من أفعال القلب.
-فإن قيل: يلزم على هذا أن يُكتب لمن همّ بالسيئة ولم يعملها سيئة أيضاً، لأن الهم بالشيء من عمل القلب أيضاً؟ قيل: ليس كذلك، فإن من كفّ عن الشر فقد فسخ اعتقاده للسيئة باعتقاد آخر نوى به الخير، وعصى هواه المريد للشر، فجوزي بذلك حسنة. وقد جاء في حديث آخر (إنما تركها من جرائي) أي من أجلي، وهذا كقوله صلى الله عليه وسلم (على كل مسلم صدقة، قالوا: فإن لم يفعل؟ قال: فليمسك عن الشر فإنه صدقة).
-وفي هذا الحديث تصحيح مقالة من قال: إن الحفظة (الملائكة الموكلين بالعبد) تكتب ما هم به العبد من حسنة أو سيئة وإن لم يظهر، والمعنى أن الملكين يعلمان ما يهم به العبد بأن الله تعالى قد جعل لهما إلى ذلك سبيلاً، كما جعل للأنبياء من علم الغيب سبيلاً.
-وهذا الفضل العظيم بأن ضاعف الله الحسنات ولم يضاعف السيئات، وإنما جعل الهمّ بالحسنة حسنة لأن إرادة الخير هو فعل القلب لعقد ذلك.</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>كرم إلهي مذهل: مجرد نيتك الصادقة لفعل الخير تُكتب لك حسنة كاملة حتى لو لم تستطع تنفيذها، وإن نفذتها ضوعفت من عشر حسنات إلى سبعمائة ضعف إلى أضعاف كثيرة. أما نية الشر فلا تُكتب عليك سيئة أبداً ما دمت لم تنفذها، بل تُكتب لك حسنة كاملة لأنك تركتها لله، وإن نفذتها فلا تُكتب إلا سيئة واحدة فقط دون مضاعفة. هذا الميزان الإلهي العادل والرحيم يشجعنا على استمرار النية الطيبة حتى لو تعثر التنفيذ، ويذكرنا أن الله لا يعاقب على مجرد الخواطر بل على الفعل فقط.</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="n">
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>هذا حديث شريف عظيم فيه بيان مقدار تفضل الله عز وجل على خلقه، بأن جعل هم العبد بالحسنة وإن لم يعملها حسنة كاملة، وجعل همه بالسيئة إن لم يعملها حسنة أيضاً، ولا يكتبها سيئة إلا إذا عملها فتُكتب سيئة واحدة فقط، فضاعف الله الحسنات ولم يضاعف السيئات. وتأمل ألفاظ الحديث ودقتها: فقوله (عنده) إشارة إلى شدة اعتناء الله بهذه الحسنة، وقوله (كاملة) للتأكيد، وقد أكّد بها الحسنة الحاصلة من الهمّ بالحسنة، كما أكّد بها الحسنة الكاملة الحاصلة من ترك السيئة، بينما أكّد قلة السيئة المعمولة بلفظ (واحدة) ولم يصفها بـ(كاملة)، فلله الحمد والمنة على هذا الفضل واللطف العظيم. وإنما جُعل الهمّ بالحسنة حسنة لأن إرادة الخير فعل من أفعال القلب وعقده على ذلك.
+فإن قيل: يلزم على هذا أن يُكتب لمن همّ بالسيئة ولم يعملها سيئة أيضاً، لأن الهم بالشيء من عمل القلب أيضاً؟ قيل: ليس كذلك، فإن من كفّ عن الشر فقد فسخ اعتقاده للسيئة باعتقاد آخر نوى به الخير، وعصى هواه المريد للشر، فجوزي بذلك حسنة. وقد جاء في حديث آخر (إنما تركها من جرائي) أي من أجلي، وهذا كقوله صلى الله عليه وسلم: (على كل مسلم صدقة، قالوا: فإن لم يجد؟ قال: فليمسك عن الشر فإنه له صدقة). أما من ترك السيئة مُكرَهاً عليها أو عاجزاً عنها فلا يدخل في معنى هذا الحديث.
+قال الطبري: وفي هذا الحديث تصحيح مقالة من قال: إن الحفظة (الملائكة الموكلين بالعبد) تكتب ما هم به العبد من حسنة أو سيئة وإن لم يظهر، خلافاً لمن زعم أن الحَفَظة لا تكتب إلا ما ظهر من عمل العبد أو نطق به لسانه. والمعنى أن الملكين يعلمان ما يهمّ به العبد من خير أو شر بريحٍ تظهر لهما من القلب، كما جعل الله تعالى للأنبياء من علم الغيب سبيلاً. وقد اختلف السلف في أي الذكر أفضل: ذكر القلب أم ذكر اللسان (العلانية)؟ وحكى هذا الخلاف كله ابن بطال.
+وقد بيّن أصحاب الشرح أن هذا التضعيف الكريم (إلى أضعاف كثيرة) جاء بلفظ التنكير (كثيرة) لا بعدد محدد، وهذا أشمل من ذكر عدد معين، لأن التنكير هنا يفتح الباب لأعظم ما يمكن تصوره من الكثرة، ليتسع هذا الوعد الكريم لكل عمل بر. ومثّلوا لذلك بمثال الحبة الواحدة: فمن تصدق بحبة، فإن فضل الله يحسبها بحسب ما كانت ستؤول إليه لو زُرعت في أرض طيبة وتُعوهدت بالحفظ والري، فإنها تنمو وتُحصد، ثم يُزرع حاصلها في السنة التالية، وهكذا يستمر تكاثرها إلى يوم القيامة، فتصير الحبة الواحدة من البُر أو الخردل بحجم الجبال الرواسي! وكذلك تُقاس قيمتها بسعرها في أعظم سوق تكون فيه تلك السلعة أنفق ما تكون، ثم تتضاعف قيمتها ويتردد ذلك إلى يوم القيامة، حتى تأتي الذرة الواحدة من الصدقة بما يعادل قدر الدنيا كلها في العظمة! وعلى هذا تُقاس جميع أعمال البر في معاملة العبد لربه، إذا خرجت عن نية خالصة صادقة.
+ومن مظاهر هذا التضعيف أيضاً: أن فضل الله يتضاعف بالتحويل، كأن يتصدق إنسان على فقير بدرهم، فيُؤثر ذلك الفقير بالدرهم فقيراً آخر أشد منه حاجة، فيؤثر به هذا الثالث رابعاً، والرابع خامساً، وهكذا؛ فإن الله تعالى يكتب للمتصدق الأول بذلك الدرهم عشر حسنات، فإذا انتقل الدرهم إلى الثاني كُتب للأول عشر أمثال ما كُتب للثاني، وهكذا كلما انتقل الدرهم من يدٍ إلى يدٍ تضاعف أجر من سبقوه في هذه السلسلة أضعافاً لا يعلم مقدارها إلا الله تعالى.
+ومن ذلك أيضاً: أن الله سبحانه إذا حاسب عبده المسلم يوم القيامة وكانت حسناته متفاوتة في القيمة، فإنه بجوده وكرمه يجازيه على جميع حسناته بسعر أعلى حسنة عنده، لأن جوده جل جلاله أعظم من أن يُحاسب عباده على تفاوت يسير بين حسنة وأخرى، وقد قال تعالى: (وَلَنَجْزِيَنَّهُمْ أَجْرَهُم بِأَحْسَنِ مَا كَانُوا يَعْمَلُونَ). ومن أمثلة هذا التضعيف العظيم أيضاً: أن العبد إذا خرج من سوق من أسواق المسلمين فقال: (لا إله إلا الله وحده لا شريك له...) رافعاً بها صوته، كتب الله له بذلك ألفي ألف حسنة، ومحا عنه ألفي ألف سيئة، وبنى له بيتاً في الجنة، كما جاء ذلك في الحديث. وكل هذا الذي ذُكر إنما هو على قدر ما بلغته معرفتنا بفضل الله سبحانه وتعالى، وإلا فإن فضله أعظم من أن يُحصر أو يُحيط به وصف مخلوق.</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>كرم إلهي مذهل: مجرد نيتك الصادقة لفعل الخير تُكتب لك حسنة كاملة حتى لو لم تستطع تنفيذها، وإن نفذتها ضوعفت من عشر حسنات إلى سبعمائة ضعف إلى أضعاف كثيرة لا يحدها عدد، كحبة الزرع التي تتكاثر عاماً بعد عام حتى تصير كالجبال، أو كالصدقة التي تنتقل من يد إلى يد فيتضاعف أجر كل من سبق فيها. أما نية الشر فلا تُكتب عليك سيئة أبداً ما دمت لم تنفذها، بل تُكتب لك حسنة كاملة لأنك تركتها لله، وإن نفذتها فلا تُكتب إلا سيئة واحدة فقط دون مضاعفة. هذا الميزان الإلهي العادل والرحيم يشجعنا على استمرار النية الطيبة حتى لو تعثر التنفيذ، ويذكرنا أن الله لا يعاقب على مجرد الخواطر بل على الفعل فقط.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1658,24 +2063,34 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
+          <t>أبو هريرة رضي الله عنه (حديث قدسي)</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي هُرَيْرَةَ رَضِيَ اللهُ عَنْهُ قَالَ: قَالَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ: إِنَّ اللهَ تَعَالَى قَالَ</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
           <t>مَنْ عَادَى لِي وَلِيًّا فَقَدْ آذَنْتُهُ بِالْحَرْبِ، وَمَا تَقَرَّبَ إِلَيَّ عَبْدِي بِشَيْءٍ أَحَبَّ إِلَيَّ مِمَّا افْتَرَضْتُهُ عَلَيْهِ، وَلَا يَزَالُ عَبْدِي يَتَقَرَّبُ إِلَيَّ بِالنَّوَافِلِ حَتَّى أُحِبَّهُ، فَإِذَا أَحْبَبْتُهُ كُنْتُ سَمْعَهُ الَّذِي يَسْمَعُ بِهِ، وَبَصَرَهُ الَّذِي يُبْصِرُ بِهِ، وَيَدَهُ الَّتِي يَبْطِشُ بِهَا، وَرِجْلَهُ الَّتِي يَمْشِي بِهَا، وَلَئِنْ سَأَلَنِي لَأُعْطِيَنَّهُ، وَلَئِنِ اسْتَعَاذَنِي لَأُعِيذَنَّهُ</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>هذا حديث قدسي عظيم يتضمن أن الله سبحانه وتعالى قدّم الإعذار إلى كل من عادى وليّاً من أوليائه بأنه قد آذنه بأنه محارب له سبحانه بنفس المعاداة، ووليّ الله هو المُتّبع لشرعه المخلص في عبادته، فليحذر الإنسان من إيذاء أولياء الله عز وجل.
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>هذا حديث قدسي عظيم يتضمن أن الله سبحانه وتعالى قدّم الإعذار إلى كل من عادى وليّاً من أوليائه بأنه قد آذنه بأنه محارب له سبحانه بنفس المعاداة، ووليّ الله هو المُتّبع لشرعه المخلص في عبادته، فليحذر الإنسان من إيذاء أولياء الله عز وجل. ومعنى المعاداة هنا: أن يتّخذه عدواً لأجل ولايته لله، لا لأي سبب آخر. أما إذا اقتضت الأحوال نزاعاً بين وليّين وتحاكما فيما بينهما لاستخراج حق غامض، فإن ذلك لا يدخل في هذا الحديث ولا يُعدّ من (المعاداة) المقصودة فيه؛ فقد جرت خصومة بين أبي بكر وعمر رضي الله عنهما، وبين العباس وعليّ رضي الله عنهما، وبين كثير من الصحابة رضي الله عنهم، وكلهم كانوا أولياء الله عز وجل. فمجرد الخلاف أو المنازعة في حق من الحقوق بين أهل الصلاح لا يُعدّ محاربة لله عز وجل، وإنما المذموم هو العداوة المتعمدة لذات الولاية والصلاح.
 قوله (وما تقرب إليّ عبدي بشيء أحب إليّ مما افترضته عليه) فيه إشارة إلى أنه لا يُتقدّم إلى نافلة قبل قضاء الفريضة، وإلا فلا يتناولها اسم النافلة، وإنما سُميت النافلة نافلة إذا قُضيت الفريضة.
 ويدل قوله (ولا يزال عبدي يتقرب إليّ بالنوافل حتى أحبه) على أن التقرب بالنوافل يكون بعد بلوغ أداء الفرائض، ومتى أدام العبد التقرب بالنوافل كان ذلك أفضى إلى أن يحبه الله عز وجل. ثم قال: (فإذا أحببته كنت سمعه الذي يسمع به، وبصره الذي يبصر به...) فهذه علامة ولاية الله لمن ذُكر بذلك، ومعناه أنه لا يسمع إلا ما يأذن الشرع له بسماعه، ولا يبصر إلا ما يأذن له فيه، ولا يبطش بيده إلا فيما أذن له الشرع، ولا يسعى برجله إلا فيما أذن له فيه، فهذا هو الأصل.
 قوله (ولئن سألني لأعطينه) يدل على أن العبد إذا صار من أهل حب الله تعالى لم يمتنع عن سؤال حوائجه، والله تعالى قادر على أن يعطيه قبل أن يسأله، ولكنه سبحانه متقرب إلى عباده بإعطاء السائلين وإعاذة المستعيذين.</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>حديث قدسي يصف أعلى درجات القرب من الله سبحانه: من عادى ولياً من أولياء الله فقد أعلن الله عليه الحرب، وأحب الأعمال إلى الله ما افترضه على عباده، فينبغي أداء الفرائض أولاً كأساس لا يُتجاوز. ثم يستمر العبد في التقرب بالنوافل حتى يبلغ درجة محبة الله، وعندها يوفقه الله في كل تصرفاته -سمعه وبصره ويده ورجله- بحيث لا يستخدمها إلا فيما يرضي الله، ويستجيب الله دعاءه ويحميه إذا استعاذ به. هذا الحديث يرسم طريقاً واضحاً للقرب من الله: الالتزام بالواجبات أولاً، ثم الإكثار من النوافل تدريجياً.</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="n">
-        <v>5</v>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>حديث قدسي يصف أعلى درجات القرب من الله سبحانه: من عادى ولياً من أولياء الله فقد أعلن الله عليه الحرب، وأحب الأعمال إلى الله ما افترضه على عباده، فينبغي أداء الفرائض أولاً كأساس لا يُتجاوز. ثم يستمر العبد في التقرب بالنوافل حتى يبلغ درجة محبة الله، وعندها يوفقه الله في كل تصرفاته -سمعه وبصره ويده ورجله- بحيث لا يستخدمها إلا فيما يرضي الله، ويستجيب الله دعاءه ويحميه إذا استعاذ به. والمعاداة المقصودة هنا هي العداوة المتعمدة بسبب الصلاح والولاية، لا مجرد خلاف أو خصومة في حق من الحقوق قد تقع حتى بين الصالحين أنفسهم، كما وقع بين كبار الصحابة رضي الله عنهم. هذا الحديث يرسم طريقاً واضحاً للقرب من الله: الالتزام بالواجبات أولاً، ثم الإكثار من النوافل تدريجياً.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="40" ht="90" customHeight="1">
@@ -1689,22 +2104,32 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
+          <t>عبد الله بن عباس رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>عَنِ ابْنِ عَبَّاسٍ رَضِيَ اللهُ عَنْهُمَا أَنَّ رَسُولَ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ قَالَ</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
           <t>إِنَّ اللهَ تَجَاوَزَ لِي عَنْ أُمَّتِي الْخَطَأَ وَالنِّسْيَانَ وَمَا اسْتُكْرِهُوا عَلَيْهِ</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>وقد جاء في التفسير في قوله عز وجل (إن تبدوا ما في أنفسكم أو تخفوه يحاسبكم به الله) أن هذه الآية لما نزلت شقّ ذلك على الصحابة رضي الله عنهم، فجاءوا إلى رسول الله صلى الله عليه وسلم وقالوا: كُلّفنا من العمل ما لا نطيق، إن أحدنا يحدّث نفسه بما لا يحب أن يثبت في قلبه. فقال النبي صلى الله عليه وسلم: لعلكم تقولون كما قالت بنو إسرائيل: سمعنا وعصينا؟ قولوا: سمعنا وأطعنا. واشتد ذلك عليهم ومكثوا حولاً، فأنزل الله تعالى الفرج والرحمة بقوله: (لا يكلف الله نفساً إلا وسعها، لها ما كسبت وعليها ما اكتسبت، ربنا لا تؤاخذنا إن نسينا أو أخطأنا)، قال الله تعالى: قد فعلت، فنزل التخفيف ونسخت الآية الأولى.
-قال الشافعي رحمه الله: قال الله جل ثناؤه (إلا من أُكره وقلبه مطمئن بالإيمان)، وللكفر أحكام، فلما وضع الله عنه أحكام الإكراه سقطت أحكامها كلها، لأن الأعظم أنه سقط مما هو أصغر منه.
-ثم ذكر حديث ابن عباس هذا: (إن الله تجاوز لي عن أمتي الخطأ والنسيان وما استُكرهوا عليه). وأسند أيضاً عن عائشة رضي الله عنها عن النبي صلى الله عليه وآله وسلم أنه قال: (لا طلاق ولا عتاق في إغلاق) وهو مذهب عمر وابن عمر رضي الله عنهما.</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>رحمة عظيمة من الله بهذه الأمة: تجاوز سبحانه عن ثلاثة أمور لا يملك الإنسان دفعها عن نفسه: الخطأ غير المتعمد، والنسيان، وما يُكره عليه الإنسان دون اختياره. هذا الحديث يريح كل من يخاف أن يُحاسب على خواطر عابرة أو أخطاء غير مقصودة، فالحساب الإلهي مبني على العدل التام: لا مؤاخذة إلا على ما يقصده الإنسان بإرادته الحرة. وقد نزلت هذه الرحمة تخفيفاً بعد أن شقّ على الصحابة تصور محاسبتهم على خواطر قلوبهم، فبيّن الله أنه لا يكلف نفساً إلا وسعها.</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="n">
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>وقد جاء في التفسير في قوله عز وجل (إن تبدوا ما في أنفسكم أو تخفوه يحاسبكم به الله) أن هذه الآية لما نزلت شقّ ذلك على الصحابة رضي الله عنهم، فجاء أبو بكر وعمر وعبد الرحمن بن عوف ومعاذ بن جبل رضي الله عنهم في ناسٍ إلى رسول الله صلى الله عليه وسلم وقالوا: كُلّفنا من العمل ما لا نطيق، إن أحدنا يحدّث نفسه بما لا يحب أن يثبت في قلبه وأن له الدنيا. فقال النبي صلى الله عليه وسلم: لعلكم تقولون كما قالت بنو إسرائيل: سمعنا وعصينا؟ قولوا: سمعنا وأطعنا. قالوا: سمعنا وأطعنا. واشتد ذلك عليهم ومكثوا حولاً، فأنزل الله تعالى الفرج والرحمة بقوله: (لا يكلف الله نفساً إلا وسعها، لها ما كسبت وعليها ما اكتسبت، ربنا لا تؤاخذنا إن نسينا أو أخطأنا)، قال الله تعالى: قد فعلت، فنزل التخفيف ونسخت الآية الأولى.
+قال الشافعي رحمه الله: قال الله جل ثناؤه (إلا من أُكره وقلبه مطمئن بالإيمان)، وللكفر أحكام، فلما وضع الله عنه أحكام الإكراه سقطت أحكامها كلها، لأن الأعظم إذا سقط سقط ما هو أصغر منه.
+ثم أسند حديث ابن عباس هذا: (إن الله تجاوز لي عن أمتي الخطأ والنسيان وما استُكرهوا عليه). وأسند أيضاً عن عائشة رضي الله عنها عن النبي صلى الله عليه وآله وسلم أنه قال: (لا طلاق ولا عتاق في إغلاق) وهو مذهب عمر وابن عمر رضي الله عنهما. وقد استدل بهذا الأصل الفقهاء في مسائل الطلاق والعتاق الواقعة في حال الإكراه والغضب الشديد المُذهِب للاختيار، فلا يقع طلاق المُكرَه ولا عتاقه.</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>رحمة عظيمة من الله بهذه الأمة: تجاوز سبحانه عن ثلاثة أمور لا يملك الإنسان دفعها عن نفسه: الخطأ غير المتعمد، والنسيان، وما يُكره عليه الإنسان دون اختياره. هذا الحديث يريح كل من يخاف أن يُحاسب على خواطر عابرة أو أخطاء غير مقصودة، فالحساب الإلهي مبني على العدل التام: لا مؤاخذة إلا على ما يقصده الإنسان بإرادته الحرة. وقد نزلت هذه الرحمة تخفيفاً بعد أن شقّ على الصحابة تصور محاسبتهم على خواطر قلوبهم، فبيّن الله أنه لا يكلف نفساً إلا وسعها. وعلى هذا الأصل بنى الفقهاء أحكاماً كثيرة، منها أن طلاق المُكرَه وعتاقه لا يقعان لأنه فعلهما بغير اختيار حقيقي.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1719,22 +2144,36 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
+          <t>عبد الله بن عمر رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>عَنِ ابْنِ عُمَرَ رَضِيَ اللهُ عَنْهُمَا قَالَ: أَخَذَ رَسُولُ اللهِ صَلَّى اللهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ بِمَنْكِبَيَّ فَقَالَ</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
           <t>كُنْ فِي الدُّنْيَا كَأَنَّكَ غَرِيبٌ أَوْ عَابِرُ سَبِيلٍ. وَكَانَ ابْنُ عُمَرَ رَضِيَ اللهُ تَعَالَى عَنْهُمَا يَقُولُ: إِذَا أَمْسَيْتَ فَلَا تَنْتَظِرِ الصَّبَاحَ، وَإِذَا أَصْبَحْتَ فَلَا تَنْتَظِرِ الْمَسَاءَ، وَخُذْ مِنْ صِحَّتِكَ لِمَرَضِكَ، وَمِنْ حَيَاتِكَ لِمَوْتِكَ</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>هذا الحديث حث على قصر الأمل في الدنيا، وعدم الركون إليها والاطمئنان بها، وأن يكون العبد فيها كالغريب الذي لا يألف الوطن ولا يستوطنه، أو كعابر السبيل الذي لا يقيم في مكان، وإنما همّه بلوغ منزله ووطنه الحقيقي.
-وقد كان ابن عمر رضي الله عنهما يقول: إذا أمسيت فلا تنتظر الصباح، وإذا أصبحت فلا تنتظر المساء، وخذ من صحتك لمرضك، ومن حياتك لموتك، يعني بادر بالأعمال الصالحة قبل فوات أوانها، فإن الإنسان لا يدري متى تأتيه المنية، فليغتنم أوقات الصحة والفراغ والحياة قبل أن تدركه أوقات المرض والشغل والموت.</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>وصية جامعة تختم الأربعين حديثاً: عش في الدنيا وكأنك غريب عابر سبيل، لا تتعلق بها كأنها وطنك الدائم أو مقرك الأبدي. وكان ابن عمر رضي الله عنهما يترجم هذا المعنى عملياً بنصيحة بليغة: لا تؤجل عملك الصالح انتظاراً للغد، فقد لا يأتي، واغتنم صحتك قبل أن يعتريك المرض، وحياتك قبل أن يفاجئك الموت. هذا الحديث ليس دعوة للقلق أو التشاؤم، بل لحسن استثمار الوقت المحدود الذي نملكه، فالغريب في بلد لا يضيع وقته في التعلق بما لن يبقى معه.</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>5</v>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>هذا الحديث حث عظيم على قصر الأمل في الدنيا وعدم الركون إليها والاطمئنان بها، وأصله أن النبي صلى الله عليه وآله وسلم أخذ بمنكبي عبد الله بن عمر رضي الله عنهما وقال له: (كن في الدنيا كأنك غريب أو عابر سبيل).
+قال أبو الزناد فيما نقله ابن بطال في شرح صحيح البخاري: معنى هذا الحديث الحضّ على قلة المخالطة وقلة الاقتناء والزهد في الدنيا. وبيان ذلك: أن الغريب قليل الانبساط إلى الناس، مستوحش منهم، إذ لا يكاد يعرف من يعرفه أو يأنس به، ويستكثر من مخالطته خائفاً وجلاً. وكذلك عابر السبيل لا يُثقل نفسه بشيء يمنعه من قطع سفره، فليس معه إلا زادٌ وراحلة يُبلّغانه إلى مقصده. وهذا يدل على أن الأولى بالمؤمن أن يؤثر من الدنيا البُلغة والكفاف فحسب، فكما لا يحتاج المسافر في غاية سفره إلى أكثر مما يبلغه، كذلك لا يحتاج المؤمن من الدنيا إلا إلى ما يبلغه إلى الآخرة.
+وقال العز بن عبد السلام رحمه الله: في هذا الحديث ما يدل على أن النبي صلى الله عليه وسلم حضّ على التشبه بالغريب، لأن الغريب إذا دخل بلدة لم ينافس أهلها في مجالسهم، ولا يجزع أن يراه أحد على خلاف عادته في الملبس، ولا يكون متدابراً معهم. وكذلك عابر السبيل لا يتخذ داراً ولا يلج في الخصومات مع الناس ومشاحنتهم، لعلمه أن مقامه معهم أيام يسيرة. فكل أحوال الغريب وعابر السبيل مستحبة أن تكون للمؤمن في الدنيا، لأن الدنيا ليست له وطناً، وإنما هي محل عبوره إلى داره الحقيقية، وهي الحائلة بينه وبين قراره في الآخرة.
+أما قول ابن عمر رضي الله عنهما: (إذا أمسيت فلا تنتظر الصباح، وإذا أصبحت فلا تنتظر المساء) فهو حضٌّ منه على أن المؤمن يستعد أبداً للموت، والموت يستعد له بالعمل الصالح، وهذا هو (قصر الأمل)، أي: لا تُؤخّر عمل الليل منتظراً الصباح، بل بادر بالعمل فوراً، وكذلك إذا أصبحت فلا تحدّث نفسك بتأخير أعمال الصباح إلى المساء. وقوله (وخذ من صحتك لمرضك) حضٌّ على اغتنام أيام الصحة والاجتهاد فيها خشية أن يحول بينك وبين العمل مرضٌ يعتريك. وكذلك قوله (ومن حياتك لموتك) تنبيه على اغتنام أيام الحياة، لأن من مات انقطع عمله، وفات أمله، وعظمت حسرته وندمه على تفريطه، وليعلم أنه سيأتي زمن طويل وهو تحت التراب لا يستطيع عملاً، فليبادر بالعمل الصالح في زمن سلامته وقدرته. فما أجمع هذا الحديث لمعاني النصح وأشرفها!
+وقد ذمّ العلماء طول الأمل، فقد ذمّ الله تعالى صاحبه بقوله: (ذَرْهُمْ يَأْكُلُوا وَيَتَمَتَّعُوا وَيُلْهِهِمُ الْأَمَلُ فَسَوْفَ يَعْلَمُونَ). وقال بعض السلف: ارتحلت الدنيا مدبرة، وارتحلت الآخرة مقبلة، ولكل واحدة منهما بنون، فكونوا من أبناء الآخرة ولا تكونوا من أبناء الدنيا، فإن اليوم عمل ولا حساب، وغداً حساب ولا عمل. وقال أنس رضي الله عنه: خطّ النبي صلى الله عليه وسلم خطوطاً فقال: (هذا الإنسان، وهذا أجله، وهذا أمله)، فبينما هو كذلك إذ جاءه الخط الأقرب وهو أجله المحيط به. وفي هذا تنبيه على وجوب تقصير الأمل واستقصار الأجل خشية بغتته، فمن غاب عنه أجله فهو جدير بتوقعه وانتظاره خشية هجومه عليه في حال غفلة، فليكافح المؤمن نفسه ويمنعها من الاستسلام لطول الأمل، فإن الإنسان يظل هواه وأمله يجولان به بعيداً عن الاستعداد الحقيقي.
+وقد روى عبد الله بن عمر رضي الله عنهما أن رسول الله صلى الله عليه وسلم رآه يوماً وهو يُطلي حائطاً له، فقال له: (ما هذا يا عبد الله؟) فقال: يا رسول الله، قد وهت (تصدّعت) فنحن نُصلحها. فقال صلى الله عليه وسلم: (الأمر أسرع من ذلك)، أي أن أجل الإنسان أقرب وأسرع من أن ينشغل بمثل هذه الإصلاحات الدنيوية التي لا تليق بحال الغريب أو عابر السبيل. نسأل الله العظيم أن يلطف بنا، وأن يزهدنا في الدنيا، وأن يجعل رغبتنا فيما لديه، وأن يحسن راحتنا يوم القيامة، إنه جواد كريم غفور رحيم.</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>وصية جامعة تختم الأربعين حديثاً: عش في الدنيا وكأنك غريب لا يألف البلد التي هو فيها ولا ينافس أهلها في مجالسهم، أو كعابر سبيل لا يحمل من الزاد إلا ما يبلغه إلى مقصده ولا يتعلق بمكان يمر به ولا يدخل في خصومات مع أهله. فالدنيا ليست وطناً دائماً للمؤمن، وإنما هي ممر إلى الآخرة وهي داره الحقيقية. وكان ابن عمر رضي الله عنهما يترجم هذا المعنى عملياً بمبدأ (قصر الأمل): لا تؤجل عملك الصالح انتظاراً للغد فقد لا يأتي، واغتنم صحتك قبل أن يعتريك المرض، وحياتك قبل أن يفاجئك الموت، فمن مات انقطع عمله وعظمت حسرته على تفريطه. وقد ذمّ الشرع طول الأمل الذي يُنسي الآخرة ويشغل صاحبه بعمارة الدنيا، وضرب النبي صلى الله عليه وسلم لذلك مثلاً بخطوط الإنسان والأجل والأمل التي يقطعها الأجل الأقرب فجأة. هذا الحديث ليس دعوة للقلق أو التشاؤم، بل لحسن استثمار الوقت المحدود الذي نملكه استعداداً للقاء الله.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="42" ht="90" customHeight="1">
@@ -1748,22 +2187,32 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
+          <t>أبو محمد عبد الله بن عمرو بن العاص رضي الله عنهما</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>عَنْ أَبِي مُحَمَّدٍ عَبْدِ اللَّهِ بْنِ عَمْرِو بْنِ الْعَاصِ رَضِيَ اللَّهُ عَنْهُمَا قَالَ: قَالَ رَسُولُ اللَّهِ صَلَّى اللَّهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ:</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
           <t>لَا يُؤْمِنُ أَحَدُكُمْ حَتَّى يَكُونَ هَوَاهُ تَبَعًا لِمَا جِئْتُ بِهِ</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>هذا الحديث يفسّره كلام الله سبحانه وتعالى (فلا وربك لا يؤمنون حتى يحكّموك فيما شجر بينهم ثم لا يجدوا في أنفسهم حرجاً مما قضيت ويسلّموا تسليماً)، وسبب نزولها: أن الزبير رضي الله عنه كان بينه وبين رجل من الأنصار خصومة في ماء، فتحاكما إلى رسول الله صلى الله عليه وسلم فقال: (اسقِ يا زبير ثم أرسل الماء إلى جارك)، فقال الأنصاري: أن كان ابن عمتك؟ فتلوّن وجه رسول الله صلى الله عليه وسلم ثم قال: (يا زبير احبس الماء حتى يبلغ الجدر) ثم سرّحه. وذلك أن رسول الله صلى الله عليه وسلم كان أشار على الزبير أولاً بما فيه مصلحة الأنصاري تيسيراً وتسامحاً، فلما اعترض الأنصاري بذلك القول أغضبه، فاستوعب للزبير حقه كاملاً واجباً، فنزلت هذه الآية تأكيداً على وجوب التسليم الكامل لحكم النبي صلى الله عليه وسلم دون تحرّج.
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>هذا الحديث يفسّره كلام الله سبحانه وتعالى (فلا وربك لا يؤمنون حتى يحكّموك فيما شجر بينهم ثم لا يجدوا في أنفسهم حرجاً مما قضيت ويسلّموا تسليماً)، وسبب نزولها: أن الزبير رضي الله عنه كان بينه وبين رجل من الأنصار خصومة في ماء، فتحاكما إلى رسول الله صلى الله عليه وسلم فقال: (اسق يا زبير وسرح الماء إلى جارك)، فقال الأنصاري: أن كان ابن عمتك؟ فتلوّن وجه رسول الله صلى الله عليه وسلم ثم قال: (يا زبير احبس الماء حتى يبلغ الجدر) ثم سرّحه. وذلك أن رسول الله صلى الله عليه وسلم كان أشار على الزبير بما فيه مصلحة الأنصاري، فلما أحفظه الأنصاري بما قال -أي أغضبه- استوعب للزبير حقه الذي يجب له، فنزلت هذه الآية.
 وقد صح عن النبي صلى الله عليه وسلم في حديث آخر أنه قال: (والذي نفسي بيده لا يؤمن أحدكم حتى أكون أحب إليه من والده وولده والناس أجمعين). قال أبو الزناد: هذا من جوامع الكلم، لأنه قد جمعت هذه الألفاظ اليسيرة معاني كثيرة، لأن أقسام المحبة ثلاثة: محبة إجلال وعظمة كمحبة الوالد، ومحبة شفقة ورحمة كمحبة الولد، ومحبة استحسان ومشاكلة كمحبة سائر الناس، فحصر أصناف المحبة جميعاً.
-قال ابن بطال: ومعنى الحديث -والله أعلم- أن من استكمل حق الإيمان علم أن حق رسول الله صلى الله عليه وسلم آكد من حق أبيه وابنه والناس أجمعين، لأن برسول الله صلى الله عليه وسلم استنقذه الله عز وجل من النار وجعل له هداه من الضلال. والمراد بالحديث: بذل النفس دونه صلى الله عليه وسلم، وقد كانت الصحابة رضي الله عنهم يقاتلون دونه معه آباءهم وأبناءهم وإخوانهم، وقد قتل أبو عبيدة لإيذائه رسول الله صلى الله عليه وسلم أباه، وتعرّض أبو بكر رضي الله عنه لولده عبد الرحمن يوم بدر لعله يتمكن منه فيقتله، فمن وجد من نفسه هذا فقد صح إيمانه تبعاً لما جاء به النبي صلى الله عليه وسلم.</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
+قال ابن بطال: ومعنى الحديث -والله أعلم- أن من استكمل الإيمان علم أن حق رسول الله صلى الله عليه وسلم وتفضيله آكد من حق أبيه وابنه والناس أجمعين، لأن برسول الله صلى الله عليه وسلم استنقذه الله عز وجل من النار وجعل له هداه من الضلال. والمراد بالحديث: بذل النفس دونه صلى الله عليه وسلم، وقد كانت الصحابة رضي الله عنهم يقاتلون دونه معه آباءهم وأبناءهم وإخوانهم، وقد قتل أبو عبيدة لإيذائه رسول الله صلى الله عليه وسلم أباه، وتعرّض أبو بكر رضي الله عنه لولده عبد الرحمن يوم بدر لعله يتمكن منه فيقتله، فمن وجد من نفسه هذا فقد صح إيمانه تبعاً لما جاء به النبي صلى الله عليه وسلم.</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
         <is>
           <t>الإيمان الكامل يقتضي أن تخضع رغباتنا وميولنا الشخصية لما جاء به النبي صلى الله عليه وسلم من هدي، لا أن نُخضع الدين لأهوائنا. وقصة الزبير مع جاره الأنصاري في تقسيم ماء السقي مثال حي: حكم النبي صلى الله عليه وسلم أولاً بحكم فيه تيسير، فلما اعترض الأنصاري ظناً منه بالمحاباة، أعطى النبي صلى الله عليه وسلم الزبير حقه كاملاً، فنزلت آية تؤكد أن الإيمان الحقيقي هو التسليم الكامل لحكم الشرع دون أي تحرّج في القلب، حتى لو خالف ذلك هوانا أو توقعاتنا الأولى. وهذا يمتد أيضاً إلى محبة النبي صلى الله عليه وسلم التي يجب أن تفوق محبتنا لأنفسنا وأقرب الناس إلينا.</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="H42" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1778,24 +2227,34 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>يَا ابْنَ آدَمَ، إِنَّكَ مَا دَعَوْتَنِي وَرَجَوْتَنِي غَفَرْتُ لَكَ عَلَى مَا كَانَ مِنْكَ وَلَا أُبَالِي، يَا ابْنَ آدَمَ لَوْ بَلَغَتْ ذُنُوبُكَ عَنَانَ السَّمَاءِ ثُمَّ اسْتَغْفَرْتَنِي غَفَرْتُ لَكَ، يَا ابْنَ آدَمَ إِنَّكَ لَوْ أَتَيْتَنِي بِقُرَابِ الْأَرْضِ خَطَايَا ثُمَّ لَقِيتَنِي لَا تُشْرِكُ بِي شَيْئًا لَأَتَيْتُكَ بِقُرَابِهَا مَغْفِرَةً</t>
+          <t>أنس بن مالك رضي الله عنه (حديث قدسي)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>في هذا الحديث بشارة عظيمة وكرم عظيم، وما لا يُحصى من أنواع الفضل والإحسان والرأفة والرحمة والامتنان. ومثل هذا قوله صلى الله عليه وسلم: (الله أفرح بتوبة عبده من أحدكم بضالّته إذا وجدها). وعن أبي أيوب رضي الله عنه لما حضرته الوفاة قال: كنت كتمت عنكم شيئاً سمعته من رسول الله صلى الله عليه وسلم، سمعته يقول: (لولا أنكم تذنبون لخلق الله خلقاً يذنبون فيغفر لهم). وقد جاءت أحاديث كثيرة موافقة لهذا الحديث.
-وقوله (يا ابن آدم إنك ما دعوتني ورجوتني) هذا موافق لقوله (أنا عند ظن عبدي بي). وقد جاء: إن العبد إذا أذنب ثم ندم فقال: ربي، أذنبت ذنباً فاغفر لي، فإنه لا يغفر الذنوب إلا أنت، فيقول الله تعالى: علم عبدي أن له رباً يغفر الذنب ويأخذ به، أشهدكم أني قد غفرت له. ثم يفعل ذلك ثانية وثالثة، فيقول الله عز وجل في كل مرة مثل ذلك، ثم يقول: (اعمل ما شئت فقد غفرت لك) يعني ما استمرّ يستغفر.
-واعلم أن للتوبة ثلاثة شروط: الإقلاع عن المعصية، والندم على ما فات، والعزم على أن لا يعود، وإن كانت بينه وبين آدمي ففيها كفارة رابع من فعل ذلك لابد منه، وهذا شرط رابع.
-قوله (على ما كان منك) أي من تكرار معصيتك (ولا أبالي) أي ولا أبالي بذنوبك في المغفرة. وقوله (يا ابن آدم لو بلغت ذنوبك عنان السماء ثم استغفرتني غفرت لك) أي لو كانت أشخاصاً من كثرتها تبلغ ما بين السماء والأرض، وهذا نهاية الكثرة، فتتلاشى ذنوب العبد عند حلم الله وعفوه.
-وقوله (يا ابن آدم إنك لو أتيتني بقراب الأرض خطايا ثم لقيتني لا تشرك بي شيئاً لأتيتك بقرابها مغفرة) أي على أساس التوحيد، وقد قال الله تعالى: (إن الله لا يغفر أن يشرك به ويغفر ما دون ذلك لمن يشاء). وقد قال صلى الله عليه وسلم: (ما أصرّ من استغفر وإن عاد في اليوم سبعين مرة). وقال أبو هريرة رضي الله عنه: قال رسول الله صلى الله عليه وسلم: (حسن الظن بالله من حسن عبادة الله).</t>
+          <t>عَنْ أَنَسٍ رَضِيَ اللَّهُ عَنْهُ قَالَ: سَمِعْتُ رَسُولَ اللَّهِ صَلَّى اللَّهُ عَلَيْهِ وَآلِهِ وَسَلَّمَ يَقُولُ: قَالَ اللَّهُ تَعَالَى:</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
+          <t>يَا ابْنَ آدَمَ، إِنَّكَ مَا دَعَوْتَنِي وَرَجَوْتَنِي غَفَرْتُ لَكَ عَلَى مَا كَانَ مِنْكَ وَلَا أُبَالِي، يَا ابْنَ آدَمَ لَوْ بَلَغَتْ ذُنُوبُكَ عَنَانَ السَّمَاءِ ثُمَّ اسْتَغْفَرْتَنِي غَفَرْتُ لَكَ، يَا ابْنَ آدَمَ لَوْ أَتَيْتَنِي بِقُرَابِ الْأَرْضِ خَطَايَا ثُمَّ لَقِيتَنِي لَا تُشْرِكُ بِي شَيْئًا لَأَتَيْتُكَ بِقُرَابِهَا مَغْفِرَةً</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>في هذا الحديث بشارة عظيمة وحلم وكرم عظيم، وما لا يُحصى من أنواع الفضل والإحسان والرأفة والرحمة والامتنان. ومثل هذا قوله صلى الله عليه وسلم: (الله أفرح بتوبة عبده من أحدكم بضالّته إذا وجدها). وعن أبي أيوب رضي الله عنه لما حضرته الوفاة قال: كنت كتمت عنكم شيئاً سمعته من رسول الله صلى الله عليه وسلم، سمعته يقول: (لولا أنكم تذنبون لخلق الله خلقاً يذنبون فيغفر لهم). وقد جاءت أحاديث كثيرة موافقة لهذا الحديث.
+وقوله (يا ابن آدم إنك ما دعوتني ورجوتني) هذا موافق لقوله (أنا عند ظن عبدي بي). وقد جاء: إن العبد إذا أذنب ثم ندم فقال: ربي، أذنبت ذنباً فاغفر لي، فإنه لا يغفر الذنوب إلا أنت، فيقول الله تعالى: علم عبدي أن له رباً يغفر الذنب ويأخذ به، أشهدكم أني قد غفرت له. ثم يفعل ذلك ثانية وثالثة، فيقول الله عز وجل في كل مرة مثل ذلك، ثم يقول: (اعمل ما شئت فقد غفرت لك) يعني: ما أذنبتَ واستغفرتَ.
+واعلم أن للتوبة ثلاثة شروط: الإقلاع عن المعصية، والندم على ما فات، والعزم على أن لا يعود. فإن كانت المعصية تتعلق بحق آدمي فليبادر بأداء الحق إليه والتحلل منه، وإن كانت بينه وبين الله تعالى ففيها كفارة فلا بد من فعل الكفارة، وهذا شرط رابع. ولو فعل الإنسان ذلك مراراً في يومه، فكلما تاب توبة مستوفية لشروطها غفر الله له.
+قوله (على ما كان منك) أي من تكرار معصيتك، (ولا أبالي) أي ولا أبالي بذنوبك. وقوله (يا ابن آدم لو بلغت ذنوبك عنان السماء ثم استغفرتني غفرت لك) أي لو كانت أشخاصاً تملأ ما بين السماء والأرض، وهذا نهاية الكثرة، ولكن كرمه سبحانه وحلمه وعفوه أكثر وأعظم، فتتلاشى ذنوب العبد عند حلمه وعفوه.
+وقوله (يا ابن آدم لو أتيتني بقراب الأرض خطايا ثم لقيتني لا تشرك بي شيئاً لأتيتك بقرابها مغفرة): قوله (ثم لقيتني) أي مُتَّ على الإيمان، ولا راحة للمؤمن دون لقاء ربه. وقد قال الله تعالى: (إن الله لا يغفر أن يشرك به ويغفر ما دون ذلك لمن يشاء). وقد قال صلى الله عليه وسلم: (ما أصرّ من استغفر وإن عاد في اليوم سبعين مرة). وقال أبو هريرة رضي الله عنه: قال رسول الله صلى الله عليه وسلم: (حسن الظن بالله من حسن عبادة الله).</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
           <t>ختام مؤثر للأربعين حديثاً: حديث قدسي يفتح أوسع أبواب الرجاء برحمة الله. مهما تكررت ذنوبك، إن دعوت الله ورجوته غفر لك دون مبالاة بكثرة الذنوب. ولو بلغت ذنوبك في الكثرة ما بين السماء والأرض ثم استغفرت الله غفرها لك. ولو لقيت الله بذنوب تملأ الأرض، ما دمت لم تشرك به شيئاً، لقيك بمغفرة تملأ الأرض. الشرط الوحيد المذكور صراحة هو التوحيد الخالص وعدم الإشراك، أما بقية الذنوب فهي في سعة رحمة الله ما دام العبد يدعو ويرجو ويستغفر بصدق. هذا الحديث يذكرنا أن حسن الظن بالله من أعظم أنواع العبادة.</t>
         </is>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="H43" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1810,7 +2269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D247"/>
+  <dimension ref="A1:D253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1868,7 +2327,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>مش كل تعب بيتحسب أجر. النية هي اللي بتحول التعب العادي لعبادة، وبتحول العبادة الفارغة لمجرد حركة.</t>
+          <t>قبل ما ترد على رسالة بغضب أو تعمل معروف لحد، اسأل نفسك: ده بقلبي ولا بس عشان الناس تشوفني؟</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1976,12 +2435,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>النية مش حاجة بتتقال مرة واحدة وخلاص، هي حوار مستمر مع نفسك في كل موقف بتاخد فيه قرار.</t>
+          <t>لما تساعد ولادك في الواجب أو تصبر على زعل حد قريب منك، مش لازم حد يشكرك عشان يبقى له قيمة. اللي محسوس بيه قلبك في اللحظة دي هو الأجر الحقيقي، حتى لو محدش لاحظ.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2489,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>الدين مش بس أفعال بنعملها، ولا بس إيمان جوانا مخفي. هو الاتنين مع بعض: قلب مصدّق، وسلوك بيترجم اللي جوه القلب.</t>
+          <t>تقدر تكون شكلك متدين قوي - لحية، حجاب، صلاة في وقتها - وتغش في البيع أو تكدب في شغلك. الحديث بيربط الاتنين ببعض: الإيمان اللي جوه لازم يبان في أمانتك وصدقك مع الناس، مش بس في مظهرك.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -2084,7 +2543,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>أحياناً بنفصل بين اللي إحنا مؤمنين بيه واللي إحنا بنعمله فعلاً، وكأنهم شيئين منفصلين. الحديث ده بيفكرنا إن الإيمان الحقيقي لازم يظهر أثره في أفعالنا اليومية، مش يفضل حبيس في القلب.</t>
+          <t>بترجع من الصلاة وتدخل تتكلم في الناس بالغيبة، أو تصوم وانت بتكدب في شغلك. مش معنى إن العبادة ماشية إن القلب والسلوك ماشيين مع بعض؛ الحديث بيقولنا إن الدين كله - جواك وبرّه - لازم يبقى صورة واحدة.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2138,7 +2597,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>خمس أركان بسيطة، لكنها كافية لو تمسكنا بيها بجد، إنها تبني حياة متزنة روحياً وعملياً.</t>
+          <t>زي ما مبنى المية طوابق مش هينفع من غير أساس، حياتك برضه: الشهادتين هي الأساس، وفوقها تقدر تبني صلاة وزكاة وصوم وحج، خطوة بخطوة مش كله مرة واحدة.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2246,12 +2705,12 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>الإيمان بالقدر مش تبرير للكسل، هو راحة نفسية إنك تبذل الجهد وتسيب النتيجة لربنا.</t>
+          <t>بتقدم على شغل وترفض، أو بتذاكر ومش طالع اللي إنت عايزه. مش معنى كده إن ربنا نسيك، ممكن يكون في حاجة تانية مكتوبة ليك إنت لسه مش شايفها.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2831,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>الدين له حدود واضحة، ومحبتنا ليه مش معناها إننا نضيف عليه من عندنا.</t>
+          <t>شفت ترند ديني جديد على السوشيال ميديا وحابب تطبقه؟ اسأل الأول: ده له أصل من القرآن والسنة، ولا بس حماس اللحظة؟</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2408,7 +2867,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>الالتزام بالأصل مش جمود، هو حماية. زي ما القانون بيحمي المجتمع من الفوضى، الحدود الشرعية بتحمي الدين من إنه يتحول لحاجة كل واحد بيفهمها زي ما هو عايز.</t>
+          <t>لما تيجي تصلي وتحس إنك عايز تزود ركعات أو تغير في شكل الصلاة عشان حاسس إنها هتبقى أقرب لربنا، وقف لحظة. النبي علّمنا الصلاة بشكلها الكامل، وأي إضافة من عندنا -حتى لو نيتها حلوة- ممكن تبعدنا عن الأصل مش تقربنا منه.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2480,7 +2939,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>قلبك هو اللي بيحدد اتجاه حياتك كلها، اهتم بيه قبل أي حاجة تانية.</t>
+          <t>لو حسّيت إنك بقيت بتضايق بسرعة من حاجات كانت هيّنة عليك زمان، دي ممكن تكون علامة إن قلبك محتاج مراجعة مش بس تجاهل.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2660,7 +3119,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>مجتمع بيحب بعضه هو اللي أفراده بيهتموا ببعض بصدق، مش بس بيتفرجوا على أخطاء بعض من بعيد.</t>
+          <t>زميلك في الشغل بيغلط في حاجة هتأثر عليه وعلى الفريق، وسكوتك عنها مش أدب ولا حياد، ده تقصير في حقه عليك.</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2786,7 +3245,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>مسؤوليتنا كبشر هي الظاهر، والباطن أمره لله. متحملش نفسك حكم على نوايا الناس.</t>
+          <t>لما تشوف حد بيصلي وانت مش متأكد لو نيته صافية أو لأ، سيبك من الحكم على قلبه، ركّز على اللي بتشوفه وسيب الباقي لربنا.</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2840,7 +3299,7 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>كتر السؤال أحياناً بيعقد حاجة كانت سهلة، خد بالبسيط وابدأ.</t>
+          <t>قبل ما تبدأ مشروع أو قرار مهم، وانت لسه بتسأل عن كل تفصيلة ممكنة، جرب تبدأ باللي واضح وسيب الباقي يتوضح في الطريق.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2876,7 +3335,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>في الحياة برضه، السؤال الكتير من غير فعل بيعطل. أحياناً لازم تاخد قرار وتمشي فيه بدل ما تفضل تسأل وتأجل.</t>
+          <t>لما تيجي تسيب حاجة حرام عليك، ماتفاوضش نفسك على نسبة منها. الأمر غير النهي: هنا المطلوب ترك كامل مش تدرّج.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -3020,7 +3479,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>الرجل في الحديث تعب كتير وسافر ودعا بإلحاح، ومع ذلك ما استُجيب دعاءه لحرمة مطعمه. ده درس إن التعب وحده مش ضمان للقبول، لازم يكون الأساس نظيف من البداية.</t>
+          <t>الرجل في الحديث تعب كتير وسافر ودعا بإلحاح، ومع ذلك ما استُجيب دعاؤه لحرمة مطعمه. ده درس إن التعب وحده مش ضمان للقبول، لازم يكون الأساس نظيف من البداية.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3164,7 +3623,7 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>الاهتمام بكل حاجة بيخليك متعب من غير فايدة حقيقية.</t>
+          <t>مش كل نقاش أو خناقة حواليك على السوشيال ميديا لازم يبقى ليك فيها رأي أو تعليق.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3380,12 +3839,12 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>العدالة في الإسلام دقيقة ومحكومة بضوابط واضحة، مش تُترك للأهواء.</t>
+          <t>لو حد ظلمك أو خطأ في حقك، مش من حقك تاخد القانون في إيدك وتحكم وتنفّذ بنفسك؛ العدل له طريقه ومؤسساته، مش انتقامك الشخصي.</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3857,7 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>الحياة الإنسانية قيمتها عالية جداً في الشرع، ومحدش له حق ياخدها إلا بضوابط قانونية واضحة، مش بمزاج شخصي أو انتقام.</t>
+          <t>في زمن المحاكمات على السوشيال ميديا، بنحكم على سمعة وحياة ناس من غير تحقيق ولا دليل. الشرع بيورينا إن الحكم على إنسان له ضوابط دقيقة، مش انطباع أو رأي عام.</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -3470,7 +3929,7 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>إكرام الجار والضيف مش رفاهية، هي جزء من كمال الإيمان.</t>
+          <t>جارك اللي بتقابله كل يوم في العمارة، حقه عليك إحسان حقيقي مش بس سلام رايح جاي.</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -3722,7 +4181,7 @@
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>الإحسان مش رفاهية بنضيفها لما نكون في مزاج كويس، هو مطلوب حتى في أصعب وأقسى المواقف.</t>
+          <t>فكرة شحذ السكين قبل الذبح بسيطة، بس معناها كبير: حتى في اللحظة اللي بتاخد فيها حق مشروع، جهّز نفسك تاخده بأخف أذى ممكن.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -3866,7 +4325,7 @@
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>حسن الخلق مش رفاهية اجتماعية، هو من صفات الأنبياء وعلامة كمال الإيمان الحقيقي.</t>
+          <t>يوم القيامة أثقل حاجة في الميزان مش الصلاة الطويلة ولا الصيام الكتير بس، هي خلقك مع الناس اللي حواليك.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -3992,7 +4451,7 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>أحياناً بنحس إن الكون كله ضدنا وكل حد بيحاول يضرنا، والحديث بيفكرنا إن محدش هيقدر يوصلك أذى إلا بإذن ربنا، وده بيديك أمان غريب وسط أي أزمة.</t>
+          <t>لما إبراهيم عليه السلام كان في الهوا وجبريل عرض عليه المساعدة، رد عليه: أما إليك فلا. طلبه كله كان من ربنا مباشرة. ده أعلى درجات التوكل.</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -4006,16 +4465,16 @@
         <v>121</v>
       </c>
       <c r="B122" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>الحياء مش خجل ضعيف، هو رادع أخلاقي بيحميك من نفسك.</t>
+          <t>أحياناً بنحس إن الكون كله ضدنا وكل حد بيحاول يضرنا، والحديث بيفكرنا إن محدش هيقدر يوصلك أذى إلا بإذن ربنا، وده بيديك أمان غريب وسط أي أزمة.</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4487,7 @@
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>لما تحس إنك ممكن تعمل حاجة لو محدش شافك، ده مقياس حقيقي لأخلاقك.</t>
+          <t>الحياء مش خجل ضعيف، هو رادع أخلاقي بيحميك من نفسك.</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -4046,12 +4505,12 @@
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>الحياء مش يعني السكوت عن حقك، هو حس داخلي بيمنعك من الفواحش ويدفعك للخير.</t>
+          <t>لما تحس إنك ممكن تعمل حاجة لو محدش شافك، ده مقياس حقيقي لأخلاقك.</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4523,7 @@
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>في زمن كل حاجة بقت مكشوفة وعادية، الحياء بقى قيمة نادرة لازم نحافظ عليها في كلامنا وتصرفاتنا.</t>
+          <t>الحياء مش يعني السكوت عن حقك، هو حس داخلي بيمنعك من الفواحش ويدفعك للخير.</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -4082,12 +4541,12 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>تربية الأولاد على الحياء مش معناها إسكاتهم، هي غرس ضمير داخلي بيوجههم صح حتى لو محدش بيراقبهم.</t>
+          <t>في زمن كل حاجة بقت مكشوفة وعادية، الحياء بقى قيمة نادرة لازم نحافظ عليها في كلامنا وتصرفاتنا.</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4096,16 +4555,16 @@
         <v>126</v>
       </c>
       <c r="B127" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>الإيمان سهل تقوله، لكن الاستقامة عليه يومياً هي الاختبار الحقيقي.</t>
+          <t>تربية الأولاد على الحياء مش معناها إسكاتهم، هي غرس ضمير داخلي بيوجههم صح حتى لو محدش بيراقبهم.</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4577,7 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>مش مهم تبدأ قوي، المهم تكمل ثابت.</t>
+          <t>الإيمان سهل تقوله، لكن الاستقامة عليه يومياً هي الاختبار الحقيقي.</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -4136,12 +4595,12 @@
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>كل يوم بتقرر فيه تكمل على المبادئ اللي مؤمن بيها حتى لو الظروف صعبة، ده استقامة حقيقية.</t>
+          <t>حماسك في أول الالتزام مش المقياس، المقياس إنك تكون لسه ثابت بعد ما يخلص الحماس ده بشهرين.</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -4154,7 +4613,7 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>الاستقامة مش الكمال، هي إنك ترجع للطريق الصح كل ما انحرفت عنه، مش إنك متنحرفش خالص.</t>
+          <t>كل يوم بتقرر فيه تكمل على المبادئ اللي مؤمن بيها حتى لو الظروف صعبة، ده استقامة حقيقية.</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -4172,7 +4631,7 @@
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>سؤال بسيط ليك النهاردة: هل أنا نفس الشخص في السر والعلن؟ ده جوهر الاستقامة.</t>
+          <t>الاستقامة مش الكمال، هي إنك ترجع للطريق الصح كل ما انحرفت عنه، مش إنك متنحرفش خالص.</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
@@ -4190,12 +4649,12 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>النبي قال إن سورة هود وأخواتها شيّبته من صعوبة الاستقامة اللي طُلبت فيها. لو الاستقامة كانت صعبة على النبي، فمن الطبيعي إنها تكون تحدي حقيقي لينا كمان.</t>
+          <t>سؤال بسيط ليك النهاردة: هل أنا نفس الشخص في السر والعلن؟ ده جوهر الاستقامة.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4204,16 +4663,16 @@
         <v>132</v>
       </c>
       <c r="B133" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>أدِّ فرائضك وابعد عن الحرام، وده كفاية تدخل بيه الجنة. الباقي زيادة خير.</t>
+          <t>النبي قال إن سورة هود وأخواتها شيّبته من صعوبة الاستقامة اللي طُلبت فيها. لو الاستقامة كانت صعبة على النبي، فمن الطبيعي إنها تكون تحدي حقيقي لينا كمان.</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4685,7 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>مش لازم تكون مثالي 100% عشان تكون مقبول عند ربنا، أدِّ الأساسيات بصدق.</t>
+          <t>أدِّ فرائضك وابعد عن الحرام، وده كفاية تدخل بيه الجنة. الباقي زيادة خير.</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -4244,12 +4703,12 @@
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>أحياناً بنحس إحباط لأننا مش بنعمل نوافل كتير، وننسى إن الالتزام بالفرائض الأساسية كفاية لتكون من أهل الجنة.</t>
+          <t>مش لازم تحس بالذنب لو مش بتصلي نوافل كتير أو بتصوم الاثنين والخميس، المهم إنك ثابت على فرايضك.</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -4262,7 +4721,7 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>الدين مش سباق مقارنة مع التانيين على مين بيعمل أكتر، هو علاقة شخصية بينك وبين ربنا بمقدار طاقتك.</t>
+          <t>أحياناً بنحس إحباط لأننا مش بنعمل نوافل كتير، وننسى إن الالتزام بالفرائض الأساسية كفاية لتكون من أهل الجنة.</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -4280,12 +4739,12 @@
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>النبي ما ضغطش على الرجل ده بمزيد من الطلبات رغم إنه كان ممكن، لأنه عرف إن قلبه لسه محتاج وقت. أحياناً الرحمة في إننا ماناخدش المعايير القصوى على كل حد بنفس الوتيرة.</t>
+          <t>الدين مش سباق مقارنة مع التانيين على مين بيعمل أكتر، هو علاقة شخصية بينك وبين ربنا بمقدار طاقتك.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4294,16 +4753,16 @@
         <v>137</v>
       </c>
       <c r="B138" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>أبسط حاجة زي الوضوء ممكن تكون نص طريقك للإيمان الكامل.</t>
+          <t>النبي ما ضغطش على الرجل ده بمزيد من الطلبات رغم إنه كان ممكن، لأنه عرف إن قلبه لسه محتاج وقت. أحياناً الرحمة في إننا ماناخدش المعايير القصوى على كل حد بنفس الوتيرة.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4316,7 +4775,7 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>كل تسبيحة وتكبيرة بتملأ الميزان، حتى لو حسيتها كلمة بسيطة.</t>
+          <t>أبسط حاجة زي الوضوء ممكن تكون نص طريقك للإيمان الكامل.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -4334,12 +4793,12 @@
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>القرآن إما حجة ليك أو عليك، بحسب إنت هتتعامل معاه إزاي: هتقراه وتعمل بيه، ولا هتسيبه على الرف؟</t>
+          <t>كل تسبيحة وتكبيرة بتملأ الميزان، حتى لو حسيتها كلمة بسيطة.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4811,7 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>الصبر مش استسلام، هو ضياء بينور طريقك في أحلك اللحظات لو صبرت فيها لله.</t>
+          <t>القرآن إما حجة ليك أو عليك، بحسب إنت هتتعامل معاه إزاي: هتقراه وتعمل بيه، ولا هتسيبه على الرف؟</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -4370,12 +4829,12 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>كل إنسان بيبيع نفسه كل يوم، إما لطاعته فيعتقها، أو لهواه فيهلكها. إنت بتبيع نفسك لمين النهاردة؟</t>
+          <t>الصبر مش إنك تكتم الألم جوه وتتظاهر إنك مبسوط. سيدنا أيوب عليه السلام قال لربنا 'أني مسني الضر' ومع كده ربنا وصفه إنه 'نعم العبد'. تقدر تشتكي لربنا وتفضل صابر في نفس الوقت.</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4388,12 +4847,12 @@
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>الصدقة برهان على صدق إيمانك، لأن المنافق بيتردد فيها. لو حسيت إنك مبسوط وانت بتدي، ده مؤشر كويس على قلبك.</t>
+          <t>كل إنسان بيبيع نفسه كل يوم، إما لطاعته فيعتقها، أو لهواه فيهلكها. إنت بتبيع نفسك لمين النهاردة؟</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4402,16 +4861,16 @@
         <v>143</v>
       </c>
       <c r="B144" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>ربنا حرّم الظلم على نفسه، فما بالك بيه بينا وبين بعض؟</t>
+          <t>الصدقة برهان على صدق إيمانك، لأن المنافق بيتردد فيها. لو حسيت إنك مبسوط وانت بتدي، ده مؤشر كويس على قلبك.</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4424,7 +4883,7 @@
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>طاعتك ما نفعتش ربنا، ومعصيتك ما ضرتوش. طاعتك رحمة لنفسك إنت.</t>
+          <t>ربنا حرّم الظلم على نفسه، فما بالك بيه بينا وبين بعض؟</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -4442,12 +4901,12 @@
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>'استهدوني أهدكم، استطعموني أطعمكم، استغفروني أغفر لكم' - كل حاجة محتاجها موجودة عند ربنا، بس محتاجة إنك تطلبها.</t>
+          <t>طاعتك ما نفعتش ربنا، ومعصيتك ما ضرتوش. طاعتك رحمة لنفسك إنت.</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4919,7 @@
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>لو كل البشر والجن كانوا على أتقى قلب رجل واحد، ما زاد ده في ملك ربنا حاجة. تقواك مش بتنفع ربنا، هي بتنفعك إنت.</t>
+          <t>'استهدوني أهدكم، استطعموني أطعمكم، استغفروني أغفر لكم' - كل حاجة محتاجها موجودة عند ربنا، بس محتاجة إنك تطلبها.</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -4478,7 +4937,7 @@
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>مهما كانت ذنوبك كتير، ربنا بيقول 'وأنا أغفر الذنوب جميعاً'. القنوط من رحمة الله أخطر من الذنب نفسه.</t>
+          <t>لو كل البشر والجن كانوا على أتقى قلب رجل واحد، ما زاد ده في ملك ربنا حاجة. تقواك مش بتنفع ربنا، هي بتنفعك إنت.</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -4496,12 +4955,12 @@
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>تخيل حد بيقولك 'اطلب مني أي حاجة عايزها وهديها لك من غير ما ينقص عندي حاجة'. ده بالظبط اللي ربنا بيعرضه علينا كل يوم، وإحنا كتير بنتجاهله.</t>
+          <t>مهما كانت ذنوبك كتير، ربنا بيقول 'وأنا أغفر الذنوب جميعاً'. القنوط من رحمة الله أخطر من الذنب نفسه.</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4973,7 @@
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>خطايانا بالليل والنهار محدش شايفها إلا ربنا، ومع ذلك بيفتح باب المغفرة قبل ما نطلبها حتى. ده كرم مش بنقدره كفاية.</t>
+          <t>تخيل حد بيقولك 'اطلب مني أي حاجة عايزها وهديها لك من غير ما ينقص عندي حاجة'. ده بالظبط اللي ربنا بيعرضه علينا كل يوم، وإحنا كتير بنتجاهله.</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -4528,16 +4987,16 @@
         <v>150</v>
       </c>
       <c r="B151" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>مش لازم تكون غني عشان تكسب أجر كبير، التسبيحة والتكبيرة صدقة برضه.</t>
+          <t>خطايانا بالليل والنهار محدش شايفها إلا ربنا، ومع ذلك بيفتح باب المغفرة قبل ما نطلبها حتى. ده كرم مش بنقدره كفاية.</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4550,7 +5009,7 @@
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>الأمر بالمعروف والنهي عن المنكر صدقة زي ما الفلوس صدقة بالظبط.</t>
+          <t>مش لازم تكون غني عشان تكسب أجر كبير، التسبيحة والتكبيرة صدقة برضه.</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -4568,7 +5027,7 @@
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>لو حسيت إنك مش قادر تتصدق بفلوس، افتكر إن كل كلمة خير بتقولها أو ابتسامة بتديها ممكن تكون صدقة عند ربنا.</t>
+          <t>المرة الجاية لما تنصح زميلك في الشغل يبطل غلط أو توقفه عن حاجة غلط، افتكر إن ده صدقة عند ربنا، وأجرها أحياناً أكبر من مجرد الذكر لأنه فرض كفاية.</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -4586,7 +5045,7 @@
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>حتى العلاقة الزوجية الحلال فيها أجر عند ربنا. الإسلام بيكرم كل تفاصيل حياتنا العادية لما نحطها في مكانها الصح.</t>
+          <t>لو حسيت إنك مش قادر تتصدق بفلوس، افتكر إن كل كلمة خير بتقولها أو ابتسامة بتديها ممكن تكون صدقة عند ربنا.</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -4604,12 +5063,12 @@
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>صحابة اتقلقوا إن الأغنياء سبقوهم في الأجر، فالنبي فتحلهم أبواب تانية للأجر مالهاش علاقة بالمال خالص. مفيش حد محروم من الفرصة.</t>
+          <t>حتى العلاقة الزوجية الحلال فيها أجر عند ربنا. الإسلام بيكرم كل تفاصيل حياتنا العادية لما نحطها في مكانها الصح.</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4622,7 +5081,7 @@
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>نفس الفعل ممكن يكون سبب أجر أو سبب وزر بحسب مكانه: الشهوة في الحلال أجر، وفي الحرام وزر. القاعدة دي بتنطبق على حاجات كتير في حياتنا.</t>
+          <t>صحابة اتقلقوا إن الأغنياء سبقوهم في الأجر، فالنبي فتحلهم أبواب تانية للأجر مالهاش علاقة بالمال خالص. مفيش حد محروم من الفرصة.</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -4636,16 +5095,16 @@
         <v>156</v>
       </c>
       <c r="B157" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>مش لازم تدور على فرصة صدقة كبيرة، إزالة حاجة مؤذية من الطريق صدقة بسيطة وسهلة.</t>
+          <t>نفس الفعل ممكن يكون سبب أجر أو سبب وزر بحسب مكانه: الشهوة في الحلال أجر، وفي الحرام وزر. القاعدة دي بتنطبق على حاجات كتير في حياتنا.</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4658,7 +5117,7 @@
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>كلمة طيبة بتقولها لحد محتاجها صدقة عند ربنا، جربها النهاردة.</t>
+          <t>مش لازم تدور على فرصة صدقة كبيرة، إزالة حاجة مؤذية من الطريق صدقة بسيطة وسهلة.</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -4676,12 +5135,12 @@
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>العدل بين اثنين في خلاف بسيط - حتى لو ولادك بيتخانقوا - صدقة عند ربنا. مش محتاج مناسبة كبيرة.</t>
+          <t>كلمة طيبة بتقولها لحد محتاجها صدقة عند ربنا، جربها النهاردة.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -4694,7 +5153,7 @@
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>كل خطوة بتمشيها للصلاة صدقة. يعني حتى المشوار البسيط للمسجد له أجر بيتحسب.</t>
+          <t>العدل بين اثنين في خلاف بسيط - حتى لو ولادك بيتخانقوا - صدقة عند ربنا. مش محتاج مناسبة كبيرة.</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -4712,7 +5171,7 @@
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>مساعدتك لحد يحمل حاجة تقيلة أو يوصل لمكانه صدقة، حتى لو ما حسبتهاش كده.</t>
+          <t>بتتأخر عن الصلاة بسبب الشغل وحاسس إنك مقصر؟ افتكر إن كل خطوة بتمشيها للمسجد، حتى وانت تعبان، صدقة متحسوبة لك.</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -4730,12 +5189,12 @@
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>يوم بيبدأ بالشمس بتطلع، وعلى كل مفصل فيك صدقة مطلوبة منك. فكرة جميلة إنك تبدأ يومك وانت فاكر إن جسمك كله عليه فرصة خير.</t>
+          <t>مساعدتك لحد يحمل حاجة تقيلة أو يوصل لمكانه صدقة، حتى لو ما حسبتهاش كده.</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4744,16 +5203,16 @@
         <v>162</v>
       </c>
       <c r="B163" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>حسن الخلق مش تفصيلة، هو تعريف البر كله في كلمة واحدة.</t>
+          <t>يوم بيبدأ بالشمس بتطلع، وعلى كل مفصل فيك صدقة مطلوبة منك. فكرة جميلة إنك تبدأ يومك وانت فاكر إن جسمك كله عليه فرصة خير.</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4766,7 +5225,7 @@
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>قلبك بيعرف الصح من الغلط قبل ما حد يفتيك، اسمع له.</t>
+          <t>حسن الخلق مش تفصيلة، هو تعريف البر كله في كلمة واحدة.</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -4784,12 +5243,12 @@
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>لو حاسس بعدم راحة تجاه قرار معين حتى لو الكل بيقولك إنه صح، ده إشارة إنك محتاج تفكر تاني.</t>
+          <t>قلبك بيعرف الصح من الغلط قبل ما حد يفتيك، اسمع له.</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -4802,7 +5261,7 @@
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>مش شرط تكون شخص مثالي عشان تكون صاحب خلق حسن، كفاية إنك منصف مع الناس ورفيق في تعاملك.</t>
+          <t>لو حاسس بعدم راحة تجاه قرار معين حتى لو الكل بيقولك إنه صح، ده إشارة إنك محتاج تفكر تاني.</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -4820,7 +5279,7 @@
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>أعرابي جذب رداء النبي بقسوة وطلب منه بجفاء، والنبي رد عليه بابتسامة وعطاء. ده مثال حي لحسن الخلق وقت الاستفزاز.</t>
+          <t>مش شرط تكون شخص مثالي عشان تكون صاحب خلق حسن، كفاية إنك منصف مع الناس ورفيق في تعاملك.</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -4838,12 +5297,12 @@
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>الإثم مش بس اللي القانون بيحرمه، هو كمان اللي بيسيب في قلبك إحساس مش مرتاح، حتى لو محدش قالك إنه غلط.</t>
+          <t>أعرابي جذب رداء النبي بعنف ونادى عليه باسمه المجرد 'يا محمد' بدل الأدب المعتاد في مخاطبته، والنبي ما ردش غير بابتسامة وعطاء. ده معنى حسن الخلق وقت الاستفزاز.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4852,16 +5311,16 @@
         <v>168</v>
       </c>
       <c r="B169" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>التمسك بالسنة وقت الاختلاف الكتير هو البوصلة اللي بتفضل تدلك على الصح.</t>
+          <t>الإثم مش بس اللي القانون بيحرمه، هو كمان اللي بيسيب في قلبك إحساس مش مرتاح، حتى لو محدش قالك إنه غلط.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4874,7 +5333,7 @@
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>البدعة في الدين خطر، لكن كل جديد مفيد ومالوش أصل مخالف مش بدعة مذمومة.</t>
+          <t>التمسك بالسنة وقت الاختلاف الكتير هو البوصلة اللي بتفضل تدلك على الصح.</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -4892,12 +5351,12 @@
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>النبي حذرنا من الاختلاف اللي هنشوفه بعده، وده بيفكرنا إن الثبات على الأصول وقت الفتن قيمة كبيرة.</t>
+          <t>البدعة في الدين خطر، لكن كل جديد مفيد ومالوش أصل مخالف مش بدعة مذمومة.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -4910,7 +5369,7 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>طاعة ولاة الأمر بالمعروف جزء من استقرار المجتمع، حتى لو مكنش القائد مثالي في كل حاجة.</t>
+          <t>النبي حذرنا من الاختلاف اللي هنشوفه بعده، وده بيفكرنا إن الثبات على الأصول وقت الفتن قيمة كبيرة.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -4928,12 +5387,12 @@
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>صحابة بكوا لما سمعوا الموعظة دي لأنها حسّوها كأنها وداع. أحياناً أقوى الكلام هو اللي بيتقال بصدق في لحظة حاسم فيها المتكلم إنه مهم.</t>
+          <t>طاعة ولاة الأمر بالمعروف جزء من استقرار المجتمع، حتى لو مكنش القائد مثالي في كل حاجة.</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4942,16 +5401,16 @@
         <v>173</v>
       </c>
       <c r="B174" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>ملاك كل خير: التحكم في لسانك. جرب تراقب كلامك يوم كامل وشوف الفرق.</t>
+          <t>صحابة بكوا لما سمعوا الموعظة دي لأنها حسّوها كأنها وداع. أحياناً أقوى الكلام هو اللي بيتقال بصدق في لحظة حاسم فيها المتكلم إنه مهم.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -4964,7 +5423,7 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>الصلاة عمود الدين، لو وقع العمود وقع البناء كله.</t>
+          <t>ملاك كل خير: التحكم في لسانك. جرب تراقب كلامك يوم كامل وشوف الفرق.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -4982,12 +5441,12 @@
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>أبواب الخير كتير: الصوم، الصدقة، قيام الليل. مش لازم تفتحهم كلهم مرة واحدة، ابدأ بواحد وكمل.</t>
+          <t>الصلاة عمود الدين، لو وقع العمود وقع البناء كله.</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5459,7 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>معاذ اتفاجئ إن اللسان سبب أساسي لدخول النار، وده بيفكرنا إن أكتر أخطاءنا بتيجي من كلام مش من أفعال.</t>
+          <t>أبواب الخير كتير: الصوم، الصدقة، قيام الليل. مش لازم تفتحهم كلهم مرة واحدة، ابدأ بواحد وكمل.</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -5018,12 +5477,12 @@
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>النبي جمع كل حاجة في جملة صغيرة: أصل، وعمود، وقمة. حياتك كمان محتاجة نفس الترتيب: إيمان أساسي، التزام يومي ثابت، وهدف تسعى ليه.</t>
+          <t>معاذ اتفاجئ إن اللسان سبب أساسي لدخول النار، وده بيفكرنا إن أكتر أخطاءنا بتيجي من كلام مش من أفعال.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5036,12 +5495,12 @@
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>'وهل يكب الناس في النار على وجوههم إلا حصائد ألسنتهم؟' جملة قوية بتخلينا نراجع كل كلمة بنقولها قبل ما نندم عليها.</t>
+          <t>في حاجات بتعملها في السر وحدك، زي قيام الليل، محدش شايفك فيها غير ربنا - وده بالذات اللي ليه أجر مخبّي محدش يعرف قيمته غيره.</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5050,16 +5509,16 @@
         <v>179</v>
       </c>
       <c r="B180" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>مش كل حاجة سكت عنها الدين لازم تدور على حكم ليها، أحياناً السكوت رحمة مش نسيان.</t>
+          <t>النبي جمع كل حاجة في جملة صغيرة: أصل، وعمود، وقمة. حياتك كمان محتاجة نفس الترتيب: إيمان أساسي، التزام يومي ثابت، وهدف تسعى ليه.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5068,16 +5527,16 @@
         <v>180</v>
       </c>
       <c r="B181" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>الحدود موجودة عشان تحميك مش عشان تضايقك، احترمها ومتتجاوزهاش.</t>
+          <t>'وهل يكب الناس في النار على وجوههم إلا حصائد ألسنتهم؟' جملة قوية بتخلينا نراجع كل كلمة بنقولها قبل ما نندم عليها.</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5090,12 +5549,12 @@
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>لو حسيت إن الدين بيضيق عليك في كل تفصيلة، افتكر إن فيه مساحة واسعة سكت عنها الشرع عمداً رحمة بينا.</t>
+          <t>مش كل حاجة سكت عنها الدين لازم تدور على حكم ليها، أحياناً السكوت رحمة مش نسيان.</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5108,12 +5567,12 @@
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>الفرائض أساس ثابت مايتفاوضش فيه، لكن باقي حياتك فيها مساحة حرية كبيرة اتركها لنفسك من غير تعقيد.</t>
+          <t>الحدود موجودة عشان تحميك مش عشان تضايقك، احترمها ومتتجاوزهاش.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5126,12 +5585,12 @@
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>أحياناً بنحمّل نفسنا تشدد في حاجات الدين نفسه ماطلبهاش، وده عكس الرحمة اللي قصدها الشرع من سكوته عن أشياء كتير.</t>
+          <t>لو حسيت إن الدين بيضيق عليك في كل تفصيلة، افتكر إن فيه مساحة واسعة سكت عنها الشرع عمداً رحمة بينا.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5140,16 +5599,16 @@
         <v>184</v>
       </c>
       <c r="B185" s="2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>قلة تعلقك بالدنيا بتخليك أخف وأسعد، جرب وشوف.</t>
+          <t>الفرائض أساس ثابت مايتفاوضش فيه، لكن باقي حياتك فيها مساحة حرية كبيرة اتركها لنفسك من غير تعقيد.</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5158,16 +5617,16 @@
         <v>185</v>
       </c>
       <c r="B186" s="2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>اللي في إيد الناس مش لازم يكون هدفك، ركز على اللي في إيدك إنت.</t>
+          <t>متبقاش زي بني إسرائيل، كتروا السؤال في حاجات مالهاش داعي لحد ما اتحرمت عليهم بسبب كتر أسئلتهم.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5176,16 +5635,16 @@
         <v>186</v>
       </c>
       <c r="B187" s="2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>الزهد مش يعني تسيب شغلك أو طموحك، هو يعني إنك متخليش قلبك معلق بالدنيا لدرجة إنها تحكمك.</t>
+          <t>أحياناً بنحمّل نفسنا تشدد في حاجات الدين نفسه ماطلبهاش، وده عكس الرحمة اللي قصدها الشرع من سكوته عن أشياء كتير.</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5198,12 +5657,12 @@
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>الشخص اللي مش متعلق بمظاهر الناس ومقتنياتهم بيبقى محبوب أكتر، لأنه بعيد عن الحسد والمقارنة.</t>
+          <t>قلة تعلقك بالدنيا بتخليك أخف وأسعد، جرب وشوف.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5216,12 +5675,12 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>من كانت الآخرة همه جمع الله شمله وجعل غناه في قلبه، ومن كانت الدنيا همه شتت الله عليه أمره. اختر أي هم يشغل قلبك بحكمة.</t>
+          <t>اللي في إيد الناس مش لازم يكون هدفك، ركز على اللي في إيدك إنت.</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5230,16 +5689,16 @@
         <v>189</v>
       </c>
       <c r="B190" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>متضرش حد من الأول، ومترد الضرر بضرر تاني.</t>
+          <t>الزهد مش يعني تسيب شغلك أو طموحك، هو يعني إنك متخليش قلبك معلق بالدنيا لدرجة إنها تحكمك.</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5248,16 +5707,16 @@
         <v>190</v>
       </c>
       <c r="B191" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>حريتك تقف عند حدود ضرر التاني، في البيت والشغل وكل مكان.</t>
+          <t>الشخص اللي مش متعلق بمظاهر الناس ومقتنياتهم بيبقى محبوب أكتر، لأنه بعيد عن الحسد والمقارنة.</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5266,16 +5725,16 @@
         <v>191</v>
       </c>
       <c r="B192" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>قاعدة بسيطة بس عميقة: أي قرار بتاخده لازم تفكر هل هيضر حد من حواليك ولا لأ.</t>
+          <t>من كانت الآخرة همه جمع الله شمله وجعل غناه في قلبه، ومن كانت الدنيا همه شتت الله عليه أمره. اختر أي هم يشغل قلبك بحكمة.</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5288,12 +5747,12 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>العلاقات القوية مبنية على إن الطرفين مايستخدموش بعض كأداة، ولا حد فيهم يضر التاني عشان يكسب هو.</t>
+          <t>متضرش حد من الأول، ومترد الضرر بضرر تاني.</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5306,12 +5765,12 @@
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>أحياناً بنفكر إن حقنا في الانتصار لنفسنا بيبرر أي رد فعل، والحديث بيفكرنا إن حتى الانتقام له حدود مايصحش نتجاوزها.</t>
+          <t>حريتك تقف عند حدود ضرر التاني، في البيت والشغل وكل مكان.</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5320,16 +5779,16 @@
         <v>194</v>
       </c>
       <c r="B195" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>الكلام لوحده مش دليل، لازم إثبات لأي ادعاء بتقوله.</t>
+          <t>قاعدة بسيطة بس عميقة: أي قرار بتاخده لازم تفكر هل هيضر حد من حواليك ولا لأ.</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5338,16 +5797,16 @@
         <v>195</v>
       </c>
       <c r="B196" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>العدالة بتحتاج دليل، مش مجرد تصديق أول كلام بيتقال.</t>
+          <t>العلاقات القوية مبنية على إن الطرفين مايستخدموش بعض كأداة، ولا حد فيهم يضر التاني عشان يكسب هو.</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5356,16 +5815,16 @@
         <v>196</v>
       </c>
       <c r="B197" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>لو كل واحد قدر ياخد حقه بمجرد ما يدّعيه، كانت الدنيا هتبقى فوضى. الدليل هو اللي بيحمي حقوق الجميع.</t>
+          <t>أحياناً بنفكر إن حقنا في الانتصار لنفسنا بيبرر أي رد فعل، والحديث بيفكرنا إن حتى الانتقام له حدود مايصحش نتجاوزها.</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5378,12 +5837,12 @@
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>قبل ما تصدق كلام حد على حد تاني، اسأل: فين الدليل؟ مش كل اتهام بيبقى صح لمجرد إنه اتقال بثقة.</t>
+          <t>الكلام لوحده مش دليل، لازم إثبات لأي ادعاء بتقوله.</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5396,12 +5855,12 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>في زمن الشائعات السريعة، قاعدة 'البينة على من ادعى' أهم من أي وقت، لأن الاتهام بلا دليل بقى سهل جداً ينتشر.</t>
+          <t>العدالة بتحتاج دليل، مش مجرد تصديق أول كلام بيتقال.</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5410,16 +5869,16 @@
         <v>199</v>
       </c>
       <c r="B200" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>مش قادر تغير الموقف؟ على الأقل ارفضه بقلبك، وده أضعف درجات الإيمان مش انعدامه.</t>
+          <t>لو كل واحد قدر ياخد حقه بمجرد ما يدّعيه، كانت الدنيا هتبقى فوضى. الدليل هو اللي بيحمي حقوق الجميع.</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5428,16 +5887,16 @@
         <v>200</v>
       </c>
       <c r="B201" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>التغيير له درجات: باليد، باللسان، بالقلب. ابدأ بأقصى ما تقدر عليه.</t>
+          <t>قبل ما تصدق كلام حد على حد تاني، اسأل: فين الدليل؟ مش كل اتهام بيبقى صح لمجرد إنه اتقال بثقة.</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5446,16 +5905,16 @@
         <v>201</v>
       </c>
       <c r="B202" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>النصح بيوصل أحسن لما يكون سراً بين اتنين، مش فضيحة قدام الناس. النبي علمنا إن الأسلوب مهم قد المضمون.</t>
+          <t>في زمن الشائعات السريعة، قاعدة 'البينة على من ادعى' أهم من أي وقت، لأن الاتهام بلا دليل بقى سهل جداً ينتشر.</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5468,12 +5927,12 @@
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>مش لازم تكون كامل عشان تنصح غيرك، المهم إنك تنصح نفسك كمان في نفس الوقت.</t>
+          <t>مش قادر تغير الموقف؟ على الأقل ارفضه بقلبك، وده أضعف درجات الإيمان مش انعدامه.</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5486,12 +5945,12 @@
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>الشيخ محيي الدين قال إن باب الأمر بالمعروف بقى مهمل في زمانه، فما بالنا دلوقتي؟ لو كل واحد اهتم بدايرته الصغيرة، كان المجتمع اتغير كتير.</t>
+          <t>التغيير له درجات: باليد، باللسان، بالقلب. ابدأ بأقصى ما تقدر عليه.</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5500,16 +5959,16 @@
         <v>204</v>
       </c>
       <c r="B205" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>التقوى في القلب مش في المظهر، ربنا شايف جواك مش شكلك بس.</t>
+          <t>النصح بيوصل أحسن لما يكون سراً بين اتنين مش فضيحة قدام الناس. الإمام الشافعي قال: اللي ينصحك سرًا يبقى زانك، واللي يفضحك قدام الناس يبقى شانك.</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5518,16 +5977,16 @@
         <v>205</v>
       </c>
       <c r="B206" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>احتقار أي إنسان خطأ كبير، لأن ربنا كرّمه وخلقه وسخّر له الكون.</t>
+          <t>مش لازم تكون كامل عشان تنصح غيرك، المهم إنك تنصح نفسك كمان في نفس الوقت.</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5536,16 +5995,16 @@
         <v>206</v>
       </c>
       <c r="B207" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>الحسد بياكل حسناتك زي ما النار بتاكل الحطب. لو حسيت إنه بيتسلل جواك، استعيذ بالله وذكّر نفسك بنعمك.</t>
+          <t>الشيخ محيي الدين قال إن باب الأمر بالمعروف بقى مهمل في زمانه، فما بالنا دلوقتي؟ لو كل واحد اهتم بدايرته الصغيرة، كان المجتمع اتغير كتير.</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5558,12 +6017,12 @@
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>كل مسلم أخوك: ماتظلموش، ماتخدلوش، ماتكذبوش، ماتحقروش. لو طبقنا الأربعة دول بس، كانت علاقاتنا اتغيرت كتير.</t>
+          <t>التقوى في القلب مش في المظهر، ربنا شايف جواك مش شكلك بس.</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5576,12 +6035,12 @@
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>بيع بعضكم على بيع بعض ممنوع - يعني منافسة غير أخلاقية في الشغل والتجارة ممنوعة برضه، مش بس في العبادات.</t>
+          <t>احتقار أي إنسان خطأ كبير، لأن ربنا كرّمه وخلقه وسخّر له الكون.</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5594,12 +6053,12 @@
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>'بحسب امرئ من الشر أن يحقر أخاه المسلم' - جملة قوية بتفكرنا إن الاستهانة بحد تانى، حتى لو بسيطة في نظرنا، ممكن تكون ذنب كبير عند ربنا.</t>
+          <t>متكبرش تسلم على حد أو ترد عليه السلام - ده من أبسط صور الاحتقار اللي النبي حذرنا منها، وعلاجه بسيط: ابتسامة وسلام.</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5608,16 +6067,16 @@
         <v>210</v>
       </c>
       <c r="B211" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>ساعدت حد يخرج من أزمته؟ ربنا هييسر عليك أزماتك أضعاف اللي عملته.</t>
+          <t>الحسد بياكل حسناتك زي ما النار بتاكل الحطب. لو حسيت إنه بيتسلل جواك، استعيذ بالله وذكّر نفسك بنعمك.</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5626,16 +6085,16 @@
         <v>211</v>
       </c>
       <c r="B212" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>ستر عيوب الناس مش تستيرها، هي بتحمي كرامتهم زي ما إنت عايز حد يحمي كرامتك.</t>
+          <t>كل مسلم أخوك: ماتظلموش، ماتخدلوش، ماتكذبوش، ماتحقروش. لو طبقنا الأربعة دول بس، كانت علاقاتنا اتغيرت كتير.</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5644,11 +6103,11 @@
         <v>212</v>
       </c>
       <c r="B213" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>العلم اللي بتتعلمه مش بس لنفسك، هو طريق بيسهّله ربنا لك للجنة. كل خطوة في التعلم لها قيمة أكبر مما تتخيل.</t>
+          <t>المنافسة الشريفة حاجة كويسة، بس تحاول تخطف عميل أو صفقة من زميلك بطرق ملتوية ده اللي الحديث بيحذر منه - في الشغل زي ما هو في البيع والشرا.</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -5662,16 +6121,16 @@
         <v>213</v>
       </c>
       <c r="B214" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>ربنا في عون العبد ما دام العبد في عون أخيه. يعني كل ما ساعدت حد، ربنا بيبقى معاك أكتر في حياتك.</t>
+          <t>'بحسب امرئ من الشر أن يحقر أخاه المسلم' - جملة قوية بتفكرنا إن الاستهانة بحد تانى، حتى لو بسيطة في نظرنا، ممكن تكون ذنب كبير عند ربنا.</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5684,12 +6143,12 @@
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>نسبك ومكانتك الاجتماعية مش هيقدّموك يوم القيامة لو عملك ضعيف. العمل هو اللي بيرفعك، مش اسم عيلتك.</t>
+          <t>ساعدت حد يخرج من أزمته؟ ربنا هييسر عليك أزماتك أضعاف اللي عملته.</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5702,12 +6161,12 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>جلسة بسيطة تقرا فيها القرآن مع ناس تانية بتنزل عليها السكينة وتحفها الملائكة. أحياناً أبسط اللحظات هي أقربنا لربنا.</t>
+          <t>ستر عيوب الناس مش تستيرها، هي بتحمي كرامتهم زي ما إنت عايز حد يحمي كرامتك.</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5716,16 +6175,16 @@
         <v>216</v>
       </c>
       <c r="B217" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>مجرد نيتك تعمل خير بتتكتب لك حسنة، حتى لو مقدرتش تنفذها.</t>
+          <t>العلم اللي بتتعلمه مش بس لنفسك، هو طريق بيسهّله ربنا لك للجنة. كل خطوة في التعلم لها قيمة أكبر مما تتخيل.</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5734,16 +6193,16 @@
         <v>217</v>
       </c>
       <c r="B218" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>ربنا بيضاعف حسناتك ومش بيضاعف سيئاتك. كرم مش بنقدره كفاية.</t>
+          <t>ربنا في عون العبد ما دام العبد في عون أخيه. يعني كل ما ساعدت حد، ربنا بيبقى معاك أكتر في حياتك.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5752,11 +6211,11 @@
         <v>218</v>
       </c>
       <c r="B219" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>فكرت تعمل خير ومقدرتش؟ متزعلش، النية وحدها كافية تتكتب حسنة كاملة عند ربنا.</t>
+          <t>نسبك ومكانتك الاجتماعية مش هيقدّموك يوم القيامة لو عملك ضعيف. العمل هو اللي بيرفعك، مش اسم عيلتك.</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -5770,16 +6229,16 @@
         <v>219</v>
       </c>
       <c r="B220" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>لو فكرت تعمل غلط وابتعدت عنه لله، ده كمان بيتكتب حسنة ليك. ترك الشر لله له أجر زي فعل الخير بالظبط.</t>
+          <t>جلسة بسيطة تقرا فيها القرآن مع ناس تانية بتنزل عليها السكينة وتحفها الملائكة. أحياناً أبسط اللحظات هي أقربنا لربنا.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5792,12 +6251,12 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>عشرة أضعاف على الأقل لكل حسنة، وسيئة واحدة بس لكل سيئة. الميزان مايل لصالحك من الأساس، فليه نيأس من رحمة ربنا؟</t>
+          <t>مجرد نيتك تعمل خير بتتكتب لك حسنة، حتى لو مقدرتش تنفذها.</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5806,11 +6265,11 @@
         <v>221</v>
       </c>
       <c r="B222" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>أدِّ فرائضك الأول، وبعدين زوّد بالنوافل. الفريضة أساس مايتفاوضش عليه.</t>
+          <t>ربنا بيضاعف حسناتك ومش بيضاعف سيئاتك. كرم مش بنقدره كفاية.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -5824,16 +6283,16 @@
         <v>222</v>
       </c>
       <c r="B223" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>القرب من ربنا بيبدأ بالواجب وبيكمل بالتطوع الزيادة.</t>
+          <t>صدقة بسيطة زي الحبة اللي بتتزرع: ممكن تكبر وتتضاعف على مر السنين لحد ما توصل لحجم مش متخيله. متقلّلش من أي خير بسيط بتعمله.</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5842,11 +6301,11 @@
         <v>223</v>
       </c>
       <c r="B224" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>لما تحب حد بجد، بتحس إنك عايز تزوده بحاجات مش لازمة عليك. علاقتك بربنا نفس الفكرة: افعل المفروض وزوّد بالتطوع من حبك.</t>
+          <t>لو فكرت تعمل غلط وابتعدت عنه لله، ده كمان بيتكتب حسنة ليك. ترك الشر لله له أجر زي فعل الخير بالظبط.</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -5860,16 +6319,16 @@
         <v>224</v>
       </c>
       <c r="B225" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>قرب العبد من ربنا مش هدف بعيد المنال، هو تراكم يومي بسيط: صلاة زيادة، صدقة زيادة، ذكر زيادة.</t>
+          <t>عشرة أضعاف على الأقل لكل حسنة، وسيئة واحدة بس لكل سيئة. الميزان مايل لصالحك من الأساس، فليه نيأس من رحمة ربنا؟</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5882,12 +6341,12 @@
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>'ولئن سألني لأعطينه' - ربنا بيوعدك إنه هيستجيب لو طلبت منه، فليه بنتردد نطلب؟</t>
+          <t>أدِّ فرائضك الأول، وبعدين زوّد بالنوافل. الفريضة أساس مايتفاوضش عليه.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -5896,11 +6355,11 @@
         <v>226</v>
       </c>
       <c r="B227" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>غلطت من غير قصد؟ ربنا متجاوز عنها، متعذبش نفسك.</t>
+          <t>القرب من ربنا بيبدأ بالواجب وبيكمل بالتطوع الزيادة.</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -5914,16 +6373,16 @@
         <v>227</v>
       </c>
       <c r="B228" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>النسيان مش ذنب، والإكراه مش اختيارك. ربنا عادل وبيفرق بين قصدك واللي بره إرادتك.</t>
+          <t>لما تحب حد بجد، بتحس إنك عايز تزوده بحاجات مش لازمة عليك. علاقتك بربنا نفس الفكرة: افعل المفروض وزوّد بالتطوع من حبك.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5932,11 +6391,11 @@
         <v>228</v>
       </c>
       <c r="B229" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>كتير مننا بيلوم نفسه على أخطاء عملها من غير قصد. الحديث بيريحنا: ربنا بيحاسب على النية مش على الزلة العابرة.</t>
+          <t>قرب العبد من ربنا مش هدف بعيد المنال، هو تراكم يومي بسيط: صلاة زيادة، صدقة زيادة، ذكر زيادة.</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -5950,16 +6409,16 @@
         <v>229</v>
       </c>
       <c r="B230" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>الصحابة قلقوا من آية بتحاسب على خواطر القلب، فربنا خفف عنهم ونسخ الحكم. ده بيوريك إن رحمة ربنا بتتجدد وبتراعي طاقتنا البشرية.</t>
+          <t>لو اختلفت مع حد صالح في رأي أو حق من الحقوق، ده مش معناه إنك بتحارب ولي من أولياء ربنا. الصحابة نفسهم اختلفوا فيما بينهم وكلهم كانوا أولياء الله. الخلاف في الرأي حاجة، والعداوة المتعمدة حاجة تانية خالص.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -5968,16 +6427,16 @@
         <v>230</v>
       </c>
       <c r="B231" s="2" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>عيش يومك وكأنه الأخير، مش خوفاً بس تقديراً للوقت.</t>
+          <t>'ولئن سألني لأعطينه' - ربنا بيوعدك إنه هيستجيب لو طلبت منه، فليه بنتردد نطلب؟</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -5986,11 +6445,11 @@
         <v>231</v>
       </c>
       <c r="B232" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>خد من صحتك لمرضك، ومن وقتك لشغلك المهم قبل ما يفوت الأوان.</t>
+          <t>غلطت من غير قصد؟ ربنا متجاوز عنها، متعذبش نفسك.</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -6004,16 +6463,16 @@
         <v>232</v>
       </c>
       <c r="B233" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>الغريب مش بيبني بيت دايم في بلد مش بلده، هو بس بيعدي. عيش الدنيا بنفس الإحساس: استخدمها ماتتعلقش بيها.</t>
+          <t>النسيان مش ذنب، والإكراه مش اختيارك. ربنا عادل وبيفرق بين قصدك واللي بره إرادتك.</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -6022,11 +6481,11 @@
         <v>233</v>
       </c>
       <c r="B234" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>'إذا أمسيت فلا تنتظر الصباح' - نصيحة عملية إنك تخلص شغلك ومهامك النهاردة، مش تأجلها على أمل بكرة.</t>
+          <t>كتير مننا بيلوم نفسه على أخطاء عملها من غير قصد. الحديث بيريحنا: ربنا بيحاسب على النية مش على الزلة العابرة.</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -6040,11 +6499,11 @@
         <v>234</v>
       </c>
       <c r="B235" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>ابن عمر كان بيعيش كل لحظة وكأنها ممكن تكون الأخيرة، مش بقلق، لكن بوعي واستثمار حقيقي للوقت. فكرة تستاهل نتبناها.</t>
+          <t>الصحابة قلقوا من آية بتحاسب على خواطر القلب، فربنا خفف عنهم ونسخ الحكم. ده بيوريك إن رحمة ربنا بتتجدد وبتراعي طاقتنا البشرية.</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -6058,11 +6517,11 @@
         <v>235</v>
       </c>
       <c r="B236" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>لما تحس إن رغبتك الشخصية بتتعارض مع أمر واضح من الدين، خليك عارف إيه اللي المفروض يحكم إيه.</t>
+          <t>إنت في الدنيا عابر سبيل، مش ساكن دايم. خد بالك من نفسك عشان الرحلة، مش عشان تستقر فيها للأبد.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -6076,11 +6535,11 @@
         <v>236</v>
       </c>
       <c r="B237" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>الإيمان الكامل مش إنك توافق الشرع لما يعجبك، هو إنك تسلّم له حتى لو خالف هواك.</t>
+          <t>خد من صحتك لمرضك، ومن حياتك لموتك - جهّز نفسك للقاء ربنا وانت لسه قادر، مش لما يفوت الأوان.</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -6094,11 +6553,11 @@
         <v>237</v>
       </c>
       <c r="B238" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>قصة الزبير مع الأنصاري في الماء مثال حي: النبي حكم بحكم فيه مصلحة، والرضا الكامل بيه حتى قبل ما يتضح السبب هو جوهر الإيمان.</t>
+          <t>الغريب مش بيبني بيت دايم في بلد مش بلده، هو بس بيعدي. عيش الدنيا بنفس الإحساس: استخدمها ماتتعلقش بيها.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -6112,11 +6571,11 @@
         <v>238</v>
       </c>
       <c r="B239" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>كل واحد فينا عنده أهواء ورغبات، والاختبار الحقيقي إننا نخلي القيم اللي مؤمنين بيها هي اللي بتوجه قراراتنا مش رغباتنا اللحظية.</t>
+          <t>'إذا أمسيت فلا تنتظر الصباح' - لو نويت تعمل خير أو تتوب عن حاجة، اعملها دلوقتي. بكرة مش حق مضمون لحد.</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -6130,16 +6589,16 @@
         <v>239</v>
       </c>
       <c r="B240" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>'حتى يكون هواه تبعاً لما جئت به' - جملة بسيطة بس بتلخص صراع داخلي كل إنسان بيمر بيه: مين اللي بيحكم قراراتك، عقلك ومبادئك، ولا مزاجك ورغباتك؟</t>
+          <t>ابن عمر كان بيصلّح حيطة في بيته فسأله النبي صلى الله عليه وسلم: 'زمن هذا؟' يعني ليه بتخطط وكأنك هتعيش للأبد؟ العمر بيجري أسرع مما نتخيل.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>reflective</t>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -6148,16 +6607,16 @@
         <v>240</v>
       </c>
       <c r="B241" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>مهما كانت ذنوبك، لو دعوت ورجوت ربنا هيغفرلك. متيأسش أبداً.</t>
+          <t>طول الأمل بينسينا إن العمر قصير والدنيا مجرد ممر، وقصر الأمل بيخلينا نعيش كل يوم وكأنه فرصتنا الحقيقية للتقرب من ربنا قبل ما نرجع لبيتنا الأخير.</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>reflective</t>
         </is>
       </c>
     </row>
@@ -6166,11 +6625,11 @@
         <v>241</v>
       </c>
       <c r="B242" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>باب التوبة مفتوح دايماً، مهما طال بعدك عن ربنا.</t>
+          <t>لما تلاقي نفسك بتدوّر على تبرير عشان يوافق اللي انت عايزه، ده وقتها هواك بقى هو اللي بيحكم مش دينك.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -6184,16 +6643,16 @@
         <v>242</v>
       </c>
       <c r="B243" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>'لو بلغت ذنوبك عنان السماء ثم استغفرتني غفرت لك' - جملة بتكسر أي حاجز نفسي بيمنعك من التوبة بسبب حجم ذنوبك.</t>
+          <t>الإيمان الكامل مش إنك توافق الشرع لما يعجبك، هو إنك تسلّم له حتى لو خالف هواك.</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>short</t>
         </is>
       </c>
     </row>
@@ -6202,11 +6661,11 @@
         <v>243</v>
       </c>
       <c r="B244" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>التوبة مش مجرد ندم، هي إقلاع عن الذنب، ندم صادق، وعزم إنك ما ترجعش ليه. لو فيها حق لحد تاني، لازم ترجعه.</t>
+          <t>قصة الزبير مع الأنصاري في الماء مثال حي: النبي حكم بحكم فيه مصلحة، والرضا الكامل بيه حتى قبل ما يتضح السبب هو جوهر الإيمان.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -6220,11 +6679,11 @@
         <v>244</v>
       </c>
       <c r="B245" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>حسن الظن بالله من حسن العبادة. لو دايماً متوقع رحمته وغفرانه، هتلاقي نفسك أقرب ليه من إنك تعيش في خوف دايم.</t>
+          <t>لما يجيلك موقف في الشغل أو البيت وتلاقي نفسك بتسأل مين هيفيدني مش إيه الصح، رجّع بالك للحديث ده: هواك مينفعش يبقى هو الحكم.</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -6238,11 +6697,11 @@
         <v>245</v>
       </c>
       <c r="B246" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>الشرط الوحيد المذكور صراحة في الحديث للمغفرة الكاملة هو عدم الشرك بالله. باقي الذنوب - مهما كانت كبيرة - في رحمة ربنا الواسعة لو تبت واستغفرت بصدق.</t>
+          <t>'حتى يكون هواه تبعاً لما جئت به' - جملة بسيطة بس بتلخص صراع داخلي كل إنسان بيمر بيه: مين اللي بيحكم قراراتك، عقلك ومبادئك، ولا مزاجك ورغباتك؟</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -6260,10 +6719,118 @@
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
+          <t>مهما كانت ذنوبك، لو دعوت ورجوت ربنا هيغفرلك. متيأسش أبداً.</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="40" customHeight="1">
+      <c r="A248" s="2" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>مش لازم تحس إنك 'مستحق' التوبة عشان تدعي ربنا. ادعيه دلوقتي زي ما انت، من غير ما تستنى تبقى أحسن.</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="40" customHeight="1">
+      <c r="A249" s="2" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>'لو بلغت ذنوبك عنان السماء ثم استغفرتني غفرت لك' - جملة بتكسر أي حاجز نفسي بيمنعك من التوبة بسبب حجم ذنوبك.</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="40" customHeight="1">
+      <c r="A250" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C250" s="3" t="inlineStr">
+        <is>
+          <t>التوبة مش مجرد ندم من جوّه: إقلاع عن الذنب، ندم صادق، وعزم إنك ما ترجعش تاني. ولو الذنب فيه حق لحد تاني، التوبة مش بتكتمل غير لما ترجّعله حقه وتطلب سماحه.</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="40" customHeight="1">
+      <c r="A251" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>حسن الظن بالله من حسن العبادة. لو دايماً متوقع رحمته وغفرانه، هتلاقي نفسك أقرب ليه من إنك تعيش في خوف دايم.</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" ht="40" customHeight="1">
+      <c r="A252" s="2" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>الشرط الوحيد المذكور صراحة في الحديث للمغفرة الكاملة هو عدم الشرك بالله. باقي الذنوب -مهما كانت كبيرة- في سعة رحمة ربنا لو تبت بصدق، إنما لو الذنب فيه حق لحد تاني، فالتوبة الكاملة بترجع الحق له مش بس بالندم في قلبك.</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>reflective</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="40" customHeight="1">
+      <c r="A253" s="2" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
           <t>ختام جميل للأربعين حديثاً: بعد كل الأحكام والقواعد والآداب، يذكرنا آخر حديث برحمة الله الواسعة التي تسع كل تقصيرنا، فالدين كله في النهاية طريق رجوع إلى رب رحيم غفور.</t>
         </is>
       </c>
-      <c r="D247" s="2" t="inlineStr">
+      <c r="D253" s="2" t="inlineStr">
         <is>
           <t>reflective</t>
         </is>

</xml_diff>

<commit_message>
feat(hadith): show المُخَرِّج instead of narrator, update workbook
The source workbook replaced its narrator column (الراوي) with who
extracted/collected each hadith (المخرج, e.g. "البخاري ومسلم"). Renamed
the Hadith model's narrator field to mukhrij, updated the detail/list
screens to show a "المُخَرِّج" chip with tashkeel instead of "الراوي",
regenerated hadiths.json from the updated workbook, and updated
import_hadiths_v2.py's column mapping to match. Also cleaned up a stale
comment in HadithRepository that claimed hadiths.json was absent from
the bundle.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/data/الأربعون_النووية_رسائل_يومية.xlsx
+++ b/assets/data/الأربعون_النووية_رسائل_يومية.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>الراوي</t>
+          <t>المخرج</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>عمر بن الخطاب رضي الله عنه</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -562,7 +562,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>عمر بن الخطاب رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>عبد الله بن عمر بن الخطاب رضي الله عنهما</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>أبو عبد الرحمن عبد الله بن مسعود رضي الله عنه</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>أم المؤمنين أم عبد الله عائشة بنت أبي بكر رضي الله عنها</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>النعمان بن بشير رضي الله عنهما</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>أبو رقية تميم بن أوس الداري رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>عبد الله بن عمر رضي الله عنهما</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة عبد الرحمن بن صخر رضي الله عنه</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>أبو محمد الحسن بن علي بن أبي طالب سبط رسول الله صلى الله عليه وسلم وريحانته رضي الله عنهما</t>
+          <t>الترمذي والنسائي</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة رضي الله عنه</t>
+          <t>الترمذي</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>أبو حمزة أنس بن مالك رضي الله عنه، خادم رسول الله صلى الله عليه وسلم</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>عبد الله بن مسعود رضي الله عنه</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة رضي الله عنه</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة رضي الله عنه</t>
+          <t>البخاري</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>أبو يعلى شداد بن أوس رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>أبو ذر جندب بن جنادة، وأبو عبد الرحمن معاذ بن جبل رضي الله عنهما</t>
+          <t>الترمذي</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>أبو العباس عبد الله بن عباس رضي الله عنهما</t>
+          <t>الترمذي</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>أبو مسعود عقبة بن عمرو الأنصاري البدري رضي الله عنه</t>
+          <t>البخاري</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>أبو عمرو -وقيل أبو عمرة- سفيان بن عبد الله رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>أبو عبد الله جابر بن عبد الله الأنصاري رضي الله عنهما</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>أبو مالك الحارث بن عاصم الأشعري رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>أبو ذر الغفاري رضي الله عنه، عن النبي صلى الله عليه وسلم فيما يرويه عن ربه عز وجل (حديث قدسي)</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>أبو ذر الغفاري رضي الله عنه (عن نفر من أصحاب رسول الله صلى الله عليه وسلم)</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة رضي الله عنه</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>النواس بن سمعان رضي الله عنه، ووابصة بن معبد رضي الله عنه</t>
+          <t>مسلم (حديث النواس بن سمعان)، وأحمد بن حنبل والدارمي (حديث وابصة بن معبد)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>أبو نجيح العرباض بن سارية رضي الله عنه</t>
+          <t>أبو داود والترمذي</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>معاذ بن جبل رضي الله عنه</t>
+          <t>الترمذي</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>أبو ثعلبة الخشني جرثوم بن ناشر رضي الله عنه</t>
+          <t>الدارقطني وغيره</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>أبو العباس سهل بن سعد الساعدي رضي الله عنه</t>
+          <t>ابن ماجه</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>أبو سعيد سعد بن مالك بن سنان الخدري رضي الله عنه</t>
+          <t>ابن ماجه والدارقطني (ورواه مالك في الموطأ مرسلاً)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>عبد الله بن عباس رضي الله عنهما</t>
+          <t>البيهقي (وبعضه رواه البخاري ومسلم في الصحيحين)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>أبو سعيد الخدري رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة رضي الله عنه</t>
+          <t>مسلم</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>عبد الله بن عباس رضي الله عنهما</t>
+          <t>البخاري ومسلم</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>أبو هريرة رضي الله عنه (حديث قدسي)</t>
+          <t>البخاري</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>عبد الله بن عباس رضي الله عنهما</t>
+          <t>ابن ماجه والبيهقي</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>عبد الله بن عمر رضي الله عنهما</t>
+          <t>البخاري</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>أبو محمد عبد الله بن عمرو بن العاص رضي الله عنهما</t>
+          <t>لم يخرجه أصحاب الكتب الستة، رواه صاحب كتاب الحجة بإسناد صحيح</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>أنس بن مالك رضي الله عنه (حديث قدسي)</t>
+          <t>الترمذي</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">

</xml_diff>